<commit_message>
Update TrendDates UI and mobile viewer cleanup
</commit_message>
<xml_diff>
--- a/excel_output/dates_wise_summary.xlsx
+++ b/excel_output/dates_wise_summary.xlsx
@@ -467,7 +467,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>40</v>
+        <v>86</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -476,7 +476,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CROMPTON, HEROMOTOCO, SAMMAANCAP, ABCAPITAL, AXISBANK, BAJAJHLDNG, BANKINDIA, BPCL, COLPAL, DABUR, DALBHARAT, DMART, DRREDDY, HAVELLS, HCLTECH, HINDALCO, HINDZINC, INDIANB, IOC, KFINTECH, KPITTECH, LUPIN, MAXHEALTH, MUTHOOTFIN, NESTLEIND, PATANJALI, PAYTM, PIDILITIND, POLICYBZR, PPLPHARMA, RBLBANK, SOLARINDS, SUPREMEIND, TATAELXSI, TATATECH, TCS, TORNTPOWER, TVSMOTOR, UNITDSPR, VBL</t>
+          <t>ABBOTINDIA, CROMPTON, ECLERX, HEROMOTOCO, NLCINDIA, SAMMAANCAP, ABCAPITAL, AEGISVOPAK, AGARWALEYE, AJANTPHARM, AKZOINDIA, ALKYLAMINE, APTUS, AXISBANK, BAJAJHLDNG, BANKINDIA, BAYERCROP, BLS, BPCL, CAPLIPOINT, CCL, CLEAN, COLPAL, CUB, DABUR, DALBHARAT, DMART, DRREDDY, EMAMILTD, ESCORTS, FACT, GILLETTE, HAPPSTMNDS, HAVELLS, HCLTECH, HEXT, HFCL, HINDALCO, HINDCOPPER, HINDZINC, HYUNDAI, INDIANB, IOB, IOC, JKCEMENT, JMFINANCIL, JPPOWER, JSWCEMENT, KFINTECH, KPITTECH, LLOYDSME, LTFOODS, LUPIN, MAXHEALTH, MUTHOOTFIN, NAM-INDIA, NATCOPHARM, NESTLEIND, PATANJALI, PAYTM, PIDILITIND, POLICYBZR, PPLPHARMA, PRAJIND, PVRINOX, RAMCOCEM, RBLBANK, SAGILITY, SOBHA, SOLARINDS, SONATSOFTW, SUMICHEM, SUPREMEIND, TATACHEM, TATAELXSI, TATATECH, TBOTEK, TCS, TORNTPOWER, TRIVENI, TVSMOTOR, UNITDSPR, VBL, VTL, WHIRLPOOL, ZENTEC</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>23</v>
+        <v>44</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -501,7 +501,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BRITANNIA, FEDERALBNK, HDFCLIFE, ICICIGI, MFSL, BAJAJFINSV, BEL, BHARATFORG, BHARTIARTL, BLUESTARCO, CDSL, CGPOWER, CUMMINSIND, EXIDEIND, ICICIPRULI, IDEA, KOTAKBANK, OFSS, RECLTD, SBILIFE, SHREECEM, ULTRACEMCO, VEDL</t>
+          <t>BRITANNIA, FEDERALBNK, GODREJIND, HDFCLIFE, ICICIGI, KARURVYSYA, MFSL, POONAWALLA, TATACOMM, AFFLE, AJANTPHARM, ALKYLAMINE, APARINDS, BAJAJFINSV, BEL, BHARATFORG, BHARTIARTL, BLUESTARCO, CARBORUNIV, CDSL, CGPOWER, CUMMINSIND, DATAPATTNS, ELECON, EXIDEIND, GRAVITA, HFCL, HONAUT, ICICIPRULI, IDEA, IGIL, INDGN, IPCALAB, KOTAKBANK, OFSS, RAILTEL, RAMCOCEM, RECLTD, SBILIFE, SHREECEM, SYRMA, TIMKEN, ULTRACEMCO, VEDL</t>
         </is>
       </c>
     </row>
@@ -517,16 +517,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>GMRAIRPORT, LICHSGFIN, MAZDOCK, ADANIPORTS, AMBUJACEM, BANKBARODA, BHARATFORG, CDSL, COLPAL, ETERNAL, ICICIGI, INFY, NHPC, PHOENIXLTD, RECLTD, RELIANCE, SHRIRAMFIN, SUZLON, TATAPOWER, UNOMINDA</t>
+          <t>TIMKEN, ACE, AFFLE, GMRAIRPORT, LICHSGFIN, MAZDOCK, AAVAS, ADANIPORTS, AMBUJACEM, ASTRAZEN, AWL, BANKBARODA, BEML, BHARATFORG, CDSL, COLPAL, ELECON, ETERNAL, HYUNDAI, ICICIGI, IIFL, INFY, INTELLECT, IOB, KPRMILL, NHPC, PHOENIXLTD, RECLTD, REDINGTON, RELIANCE, SAILIFE, SCI, SHRIRAMFIN, SUZLON, TATAPOWER, UNOMINDA, WHIRLPOOL</t>
         </is>
       </c>
     </row>
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -551,7 +551,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ADANIGREEN, ADANIENT, ADANIPORTS, PHOENIXLTD, ADANIENSOL, SBICARD, TIINDIA, UNOMINDA, AMBUJACEM, BHARTIARTL, BHEL, CAMS, KOTAKBANK, M&amp;M, MANAPPURAM, NHPC, POLYCAB, PREMIERENE, SIEMENS, SRF</t>
+          <t>ADANIGREEN, ADANIENT, ADANIPORTS, KPRMILL, PHOENIXLTD, ADANIENSOL, OLECTRA, SBICARD, THELEELA, TIINDIA, UNOMINDA, AMBUJACEM, BHARTIARTL, BHEL, CAMS, CEATLTD, FIRSTCRY, FLUOROCHEM, HBLENGINE, IFCI, IRCTC, KOTAKBANK, M&amp;M, MANAPPURAM, MMTC, MRF, NHPC, POLYCAB, PREMIERENE, SAGILITY, SAILIFE, SIEMENS, SOBHA, SRF, TBOTEK, WELCORP</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -576,7 +576,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BDL, BRITANNIA, CAMS, TATACONSUM</t>
+          <t>BDL, KIRLOSENG, SCI, AADHARHFC, AIAENG, BRITANNIA, CAMS, CENTRALBK, CGCL, GMDCLTD, GPIL, GVT&amp;D, IPCALAB, IRCTC, MOTILALOFS, NEWGEN, TATACONSUM, TBOTEK, UBL, UCOBANK</t>
         </is>
       </c>
     </row>
@@ -592,16 +592,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>HDFCLIFE, ADANIENT, CDSL, IDFCFIRSTB, INFY, ITC, NTPC, SBILIFE, TVSMOTOR</t>
+          <t>ATGL, FLUOROCHEM, CREDITACC, HDFCLIFE, ADANIENT, CDSL, DEEPAKNTR, ENRIN, FORCEMOT, GODREJIND, GRANULES, GUJGASLTD, GVT&amp;D, IDBI, IDFCFIRSTB, INFY, INOXINDIA, INTELLECT, ITC, NTPC, RADICO, SBILIFE, TVSMOTOR</t>
         </is>
       </c>
     </row>
@@ -617,7 +617,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -626,7 +626,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>GAIL, LT, 360ONE, BAJAJFINSV, BANDHANBNK, BRITANNIA, BSE, GODREJPROP, INDUSINDBK, JSWSTEEL, LTF, MCX, NBCC, NUVAMA, SONACOMS, SUNPHARMA, TMPV, UNIONBANK, WIPRO</t>
+          <t>GAIL, PFIZER, ARE&amp;M, DEEPAKFERT, HOMEFIRST, LT, NCC, SAGILITY, TEJASNET, WOCKPHARMA, 360ONE, APLLTD, ATHERENERG, BAJAJFINSV, BANDHANBNK, BLUEJET, BRITANNIA, BSE, CESC, CGCL, CHOLAHLDNG, DOMS, ENRIN, GESHIP, GODFRYPHLP, GODREJPROP, GRAVITA, HFCL, IIFL, INDUSINDBK, JSWSTEEL, LTF, M&amp;MFIN, MCX, MEDANTA, NBCC, NUVAMA, OLECTRA, SCHAEFFLER, SHYAMMETL, SONACOMS, SUNPHARMA, SUNTV, SWANCORP, TATACOMM, TMPV, UNIONBANK, WIPRO</t>
         </is>
       </c>
     </row>
@@ -642,16 +642,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>GLENMARK, GODREJPROP, INDHOTEL, JINDALSTEL, KFINTECH, LAURUSLABS, MCX, NTPC, SIEMENS, TRENT, UNIONBANK</t>
+          <t>ABLBL, ACMESOLAR, GRSE, APTUS, ASTERDM, ATHERENERG, CESC, DEEPAKNTR, ENDURANCE, FIRSTCRY, GESHIP, GLENMARK, GODREJPROP, GPIL, GSPL, HEXT, INDHOTEL, IRCON, ITI, JBMA, JINDALSTEL, JUBLPHARMA, KFINTECH, LAURUSLABS, MCX, METROPOLIS, NSLNISP, NTPC, ONESOURCE, RADICO, RITES, SBFC, SCI, SIEMENS, SWANCORP, TRENT, UNIONBANK</t>
         </is>
       </c>
     </row>
@@ -667,7 +667,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -676,7 +676,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>CANBK, HDFCBANK, INOXWIND, KOTAKBANK, NMDC, SBICARD, TATASTEEL, TIINDIA, TORNTPHARM, UNOMINDA, UPL</t>
+          <t>3MINDIA, ASTRAZEN, CANBK, CGCL, DCMSHRIRAM, DEEPAKFERT, EIDPARRY, GRANULES, GRAPHITE, GUJGASLTD, HDFCBANK, HONAUT, INOXINDIA, INOXWIND, J&amp;KBANK, JBCHEPHARM, JSWINFRA, KOTAKBANK, LATENTVIEW, MINDACORP, NMDC, POONAWALLA, PTCIL, SBFC, SBICARD, SHYAMMETL, SYRMA, TATASTEEL, TIINDIA, TORNTPHARM, TRITURBINE, UNOMINDA, UPL, VGUARD, ZFCVINDIA</t>
         </is>
       </c>
     </row>
@@ -692,7 +692,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>19</v>
+        <v>63</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -701,7 +701,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SWIGGY, COFORGE, DIVISLAB, GAIL, ADANIGREEN, ADANIPORTS, AMBUJACEM, BLUESTARCO, BRITANNIA, DIXON, HINDUNILVR, JINDALSTEL, MARICO, NTPC, PIDILITIND, RECLTD, SHREECEM, SONACOMS, ULTRACEMCO</t>
+          <t>SWIGGY, COFORGE, DIVISLAB, LALPATHLAB, BLUEDART, EMCURE, ERIS, FINCABLES, GAIL, GLAND, HBLENGINE, HOMEFIRST, MRPL, PFIZER, PGHH, WOCKPHARMA, AARTIIND, ABBOTINDIA, ADANIGREEN, ADANIPORTS, AIAENG, AIIL, AJANTPHARM, AMBUJACEM, ANANTRAJ, BLUESTARCO, BRITANNIA, CAMPUS, CCL, CHALET, CHAMBLFERT, CHENNPETRO, CREDITACC, DBREALTY, DEVYANI, DIXON, DOMS, FORCEMOT, GRAPHITE, GRSE, GSPL, HINDUNILVR, IKS, INDIACEM, ITI, JINDALSTEL, JUBLPHARMA, LEMONTREE, LTTS, MARICO, NIVABUPA, NSLNISP, NTPC, PIDILITIND, RECLTD, SAILIFE, SCHAEFFLER, SHREECEM, SJVN, SONACOMS, TIMKEN, TTML, ULTRACEMCO</t>
         </is>
       </c>
     </row>
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>27</v>
+        <v>70</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -726,7 +726,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>WAAREEENER, CROMPTON, HDFCBANK, LTM, BAJAJ-AUTO, BANKBARODA, BIOCON, BSE, CIPLA, COLPAL, DABUR, DELHIVERY, GLENMARK, HINDPETRO, INDHOTEL, JIOFIN, KFINTECH, MARUTI, NYKAA, PAGEIND, PAYTM, PERSISTENT, POWERGRID, PRESTIGE, SUPREMEIND, SUZLON, TECHM</t>
+          <t>WAAREEENER, AARTIIND, ABREL, ANANDRATHI, BLUEDART, BSOFT, MAPMYINDIA, SCHNEIDER, SIGNATURE, ATUL, BBTC, BLS, CROMPTON, ECLERX, HDFCBANK, JSL, LTM, NAVA, NTPCGREEN, TRIVENI, ACMESOLAR, ALKYLAMINE, ASTERDM, BAJAJ-AUTO, BAJAJHFL, BANKBARODA, BIOCON, BLUEJET, BSE, CHOICEIN, CIPLA, COLPAL, DABUR, DELHIVERY, ENGINERSIN, GLENMARK, GODIGIT, GVT&amp;D, HINDPETRO, IGL, IIFL, INDHOTEL, JBCHEPHARM, JIOFIN, KFINTECH, KIRLOSENG, KSB, LTTS, MARUTI, NCC, NH, NYKAA, PAGEIND, PAYTM, PERSISTENT, POWERGRID, PRAJIND, PRESTIGE, RITES, SARDAEN, SAREGAMA, SUPREMEIND, SUZLON, TECHM, TEJASNET, VTL, WELCORP, WHIRLPOOL, ZEEL, ZENSARTECH</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -751,7 +751,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>DRREDDY, PIIND, SRF, APOLLOHOSP, BIOCON, KALYANKJIL, SAMMAANCAP, ASIANPAINT, BANKINDIA, BOSCHLTD, BPCL, BSE, CONCOR, EXIDEIND, HINDALCO, HINDZINC, INDIANB, IOC, JIOFIN, JUBLFOOD, LUPIN, MAXHEALTH, MUTHOOTFIN, NMDC, PGEL, PREMIERENE, RBLBANK, SYNGENE, TATASTEEL, TORNTPHARM</t>
+          <t>CASTROLIND, DEVYANI, DRREDDY, FIVESTAR, HONASA, NAVINFLUOR, PIIND, SRF, ZENTEC, ABSLAMC, APOLLOHOSP, BAYERCROP, BIOCON, CHALET, KALYANKJIL, LINDEINDIA, LTFOODS, NLCINDIA, SAMMAANCAP, SUMICHEM, SUNDRMFAST, AIIL, AKZOINDIA, ASIANPAINT, BANKINDIA, BIKAJI, BOSCHLTD, BPCL, BRIGADE, BSE, CONCOR, COROMANDEL, CRISIL, ENGINERSIN, ENRIN, EXIDEIND, FINPIPE, GODFRYPHLP, HEXT, HINDALCO, HINDCOPPER, HINDZINC, INDIANB, IOC, JIOFIN, JKCEMENT, JSWINFRA, JUBLFOOD, JUBLPHARMA, KAJARIACER, KPIL, KSB, LUPIN, MAXHEALTH, MUTHOOTFIN, NAM-INDIA, NIACL, NMDC, PGEL, PREMIERENE, RAINBOW, RBLBANK, RKFORGE, SUNDARMFIN, SYNGENE, TARIL, TATASTEEL, THERMAX, TORNTPHARM, TTML</t>
         </is>
       </c>
     </row>
@@ -767,7 +767,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>25</v>
+        <v>65</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -776,7 +776,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>KPITTECH, TCS, HCLTECH, ICICIBANK, POWERINDIA, PRESTIGE, 360ONE, ADANIPORTS, BAJAJHLDNG, BANDHANBNK, CONCOR, DALBHARAT, DLF, IEX, INFY, JUBLFOOD, MARUTI, MPHASIS, NATIONALUM, PAGEIND, PERSISTENT, PETRONET, SOLARINDS, SYNGENE, WIPRO</t>
+          <t>BERGEPAINT, HAPPSTMNDS, KPITTECH, NATCOPHARM, SONATSOFTW, TCS, AEGISVOPAK, ALOKINDS, CRAFTSMAN, CREDITACC, FSL, HCLTECH, ICICIBANK, POWERINDIA, PRESTIGE, SJVN, 360ONE, ADANIPORTS, APLLTD, ASTRAZEN, BAJAJHLDNG, BANDHANBNK, BATAINDIA, BRIGADE, CAPLIPOINT, CONCOR, CRISIL, CYIENT, DALBHARAT, DCMSHRIRAM, DLF, EIDPARRY, ELGIEQUIP, HONAUT, HYUNDAI, IEX, IGL, INFY, IRB, JUBLFOOD, JWL, JYOTICNC, KIMS, KIRLOSBROS, KPIL, MAHSCOOTER, MARUTI, MGL, MPHASIS, NATIONALUM, NH, PAGEIND, PERSISTENT, PETRONET, RHIM, SAREGAMA, SOLARINDS, SYNGENE, TATACHEM, TATAINVEST, THERMAX, TIMKEN, TITAGARH, VMM, WIPRO</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -801,7 +801,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ANGELONE, HAVELLS, APOLLOHOSP, ASTRAL, AXISBANK, BAJAJHLDNG, BHEL, DALBHARAT, DIXON, DLF, DMART, ETERNAL, FORTIS, GODREJPROP, INDHOTEL, INDIGO, IREDA, LTF, LUPIN, MCX, NAUKRI, PIDILITIND, PNB, POLICYBZR, POLYCAB, SHRIRAMFIN, SOLARINDS, TORNTPOWER, VBL, YESBANK</t>
+          <t>ACMESOLAR, ANGELONE, ARE&amp;M, BAJAJHFL, ENGINERSIN, HAVELLS, NAVA, NCC, NTPCGREEN, RITES, TEJASNET, ABFRL, AFFLE, APOLLOHOSP, ASTRAL, AWL, AXISBANK, BAJAJHLDNG, BBTC, BHEL, CAPLIPOINT, CHENNPETRO, COCHINSHIP, DALBHARAT, DIXON, DLF, DMART, EMAMILTD, EMCURE, ENDURANCE, ERIS, ESCORTS, ETERNAL, FINPIPE, FORTIS, GODREJPROP, HFCL, HSCL, INDHOTEL, INDIGO, IREDA, KIMS, LATENTVIEW, LLOYDSME, LTF, LUPIN, MCX, MMTC, NAUKRI, PIDILITIND, PNB, POLICYBZR, POLYCAB, SARDAEN, SHRIRAMFIN, SOBHA, SOLARINDS, TATACHEM, TORNTPOWER, VBL, YESBANK</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -826,7 +826,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SBICARD, TIINDIA, APLAPOLLO, ASTRAL, BAJAJFINSV, BHEL, BPCL, COALINDIA, DIXON, ETERNAL, GODREJPROP, GRASIM, HAL, HINDALCO, HINDZINC, INDIANB, IOC, LAURUSLABS, MAZDOCK, MCX, MUTHOOTFIN, NBCC, POLYCAB, SHRIRAMFIN, SIEMENS, UNOMINDA, YESBANK, ZYDUSLIFE</t>
+          <t>AEGISLOG, BASF, SBICARD, TIINDIA, ACC, APLAPOLLO, APLLTD, ASTRAL, AWL, BAJAJFINSV, BBTC, BHEL, BLS, BPCL, COALINDIA, COCHINSHIP, DIXON, EIHOTEL, ETERNAL, GODIGIT, GODREJPROP, GRASIM, HAL, HINDALCO, HINDZINC, HSCL, HYUNDAI, IIFL, INDIAMART, INDIANB, IOC, IRB, IRCON, JMFINANCIL, KIRLOSENG, LAURUSLABS, MAZDOCK, MCX, MMTC, MUTHOOTFIN, NAM-INDIA, NBCC, NETWEB, NEULANDLAB, POLYCAB, RADICO, SAGILITY, SHRIRAMFIN, SIEMENS, UNOMINDA, YESBANK, ZYDUSLIFE</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -851,7 +851,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>FEDERALBNK, MFSL, ABB, ASIANPAINT, AXISBANK, CUMMINSIND, EICHERMOT, HDFCBANK, HUDCO, INFY, IREDA, JSWENERGY, PAYTM, PERSISTENT, PFC, RECLTD, TECHM, WIPRO</t>
+          <t>FEDERALBNK, KARURVYSYA, MFSL, VENTIVE, ABB, ASAHIINDIA, ASIANPAINT, AXISBANK, BALKRISIND, CEATLTD, CHALET, CUMMINSIND, DATAPATTNS, EICHERMOT, EIHOTEL, ELECON, GMDCLTD, HDFCBANK, HUDCO, INFY, IREDA, JBMA, JKTYRE, JSWENERGY, KEC, MRF, NEWGEN, PAYTM, PERSISTENT, PFC, PTCIL, RECLTD, RRKABEL, TARIL, TECHM, UTIAMC, VTL, WIPRO</t>
         </is>
       </c>
     </row>
@@ -867,16 +867,16 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>28</v>
+        <v>66</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>DIVISLAB, GMRAIRPORT, LICHSGFIN, BIOCON, CAMS, COFORGE, CUMMINSIND, DELHIVERY, EICHERMOT, HDFCAMC, HEROMOTOCO, HUDCO, IDEA, ITC, JSWENERGY, KOTAKBANK, LODHA, LT, LTM, MAXHEALTH, NHPC, PFC, SUNPHARMA, SUPREMEIND, SUZLON, SWIGGY, TVSMOTOR, ZYDUSLIFE</t>
+          <t>POONAWALLA, ABREL, ACE, BSOFT, DIVISLAB, GMRAIRPORT, LICHSGFIN, SCHNEIDER, AKUMS, ANANDRATHI, ATUL, BIKAJI, BIOCON, CAMS, CEATLTD, CENTURYPLY, CHOLAHLDNG, COFORGE, COROMANDEL, CUMMINSIND, DELHIVERY, EICHERMOT, ELECON, ENDURANCE, GMDCLTD, GSPL, HDFCAMC, HEROMOTOCO, HUDCO, IDEA, ITC, JBMA, JKTYRE, JSL, JSWENERGY, JUBLPHARMA, KEC, KOTAKBANK, LALPATHLAB, LODHA, LT, LTM, LTTS, MANYAVAR, MAPMYINDIA, MAXHEALTH, MRF, NHPC, PFC, RADICO, RAINBOW, REDINGTON, RPOWER, RRKABEL, SIGNATURE, SOBHA, SUNPHARMA, SUPREMEIND, SUZLON, SWIGGY, TVSMOTOR, UTIAMC, WELCORP, WELSPUNLIV, ZENSARTECH, ZYDUSLIFE</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -901,7 +901,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BAJFINANCE, MOTHERSON, SAIL, SBIN, TATACONSUM, BDL, BEL, CANBK, CGPOWER, CONCOR, DRREDDY, IRFC, ITC, JIOFIN, KALYANKJIL, NMDC, OBEROIRLTY, PIIND, SYNGENE, TATASTEEL, VEDL</t>
+          <t>AADHARHFC, BAJFINANCE, CANFINHOME, CENTRALBK, J&amp;KBANK, MINDACORP, MOTHERSON, SAIL, SBIN, TATACONSUM, UCOBANK, BAYERCROP, LTFOODS, SAGILITY, SUMICHEM, ZEEL, ZENTEC, APARINDS, APTUS, ASAHIINDIA, BDL, BEL, CANBK, CARBORUNIV, CASTROLIND, CGPOWER, CONCOR, DATAPATTNS, DCMSHRIRAM, DRREDDY, FIVESTAR, GVT&amp;D, HBLENGINE, HONASA, IGIL, INDGN, IOB, IRFC, ITC, JIOFIN, KALYANKJIL, KPIL, LINDEINDIA, MAHABANK, MOTILALOFS, NAVINFLUOR, NMDC, OBEROIRLTY, PCBL, PIIND, PTCIL, RAILTEL, SCI, SUNDRMFAST, SYNGENE, TATASTEEL, UBL, VEDL</t>
         </is>
       </c>
     </row>
@@ -917,7 +917,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -926,7 +926,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ALKEM, OFSS, AUBANK, BAJAJHLDNG, DALBHARAT, DIXON, HAVELLS, HCLTECH, ICICIPRULI, INDUSINDBK, JUBLFOOD, KPITTECH, SOLARINDS, TATATECH, TCS, TMPV, TORNTPOWER, TRENT, VBL, VOLTAS</t>
+          <t>ALKEM, GODREJAGRO, HEXT, VGUARD, OFSS, ABSLAMC, AEGISVOPAK, AUBANK, BAJAJHLDNG, CAPLIPOINT, DALBHARAT, DIXON, EIDPARRY, EMAMILTD, ENRIN, GRAVITA, HAPPSTMNDS, HAVELLS, HCLTECH, ICICIPRULI, INDUSINDBK, JUBLFOOD, KPITTECH, LLOYDSME, NATCOPHARM, SOLARINDS, SONATSOFTW, SUNDARMFIN, TATACHEM, TATATECH, TCS, TMPV, TORNTPOWER, TRENT, UBL, VBL, VOLTAS</t>
         </is>
       </c>
     </row>
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -951,7 +951,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>AMBER, KAYNES, OIL, PNBHOUSING, RELIANCE, SUZLON, BHARATFORG, BHARTIARTL, CDSL, ICICIPRULI, INDIGO, INDUSINDBK, MARUTI, NAUKRI, POWERGRID, RECLTD, SWIGGY, TATAPOWER, TRENT, UNOMINDA, VOLTAS</t>
+          <t>AMBER, KAYNES, OIL, PNBHOUSING, TECHNOE, HEG, RELIANCE, SUZLON, AAVAS, AIAENG, AWL, BHARATFORG, BHARTIARTL, CDSL, CHENNPETRO, CREDITACC, DBREALTY, EMCURE, ERIS, GRAVITA, GUJGASLTD, HFCL, ICICIPRULI, IGL, INDIGO, INDUSINDBK, INTELLECT, MARUTI, MEDANTA, MRPL, MSUMI, NAUKRI, PGHH, POLYMED, POWERGRID, RECLTD, SWIGGY, TATACOMM, TATAPOWER, TIMKEN, TRENT, UNOMINDA, VOLTAS</t>
         </is>
       </c>
     </row>
@@ -967,16 +967,16 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BANDHANBNK, ADANIGREEN, ADANIPORTS, AMBUJACEM, AXISBANK, EXIDEIND, JSWSTEEL, KEI, M&amp;M, PHOENIXLTD, SBICARD, SONACOMS, TATAELXSI, TIINDIA, TORNTPHARM, WIPRO</t>
+          <t>SUNTV, BANDHANBNK, JYOTICNC, KPRMILL, ADANIGREEN, ADANIPORTS, AFFLE, ALOKINDS, AMBUJACEM, AXISBANK, BALRAMCHIN, BLS, COHANCE, EXIDEIND, GODIGIT, HYUNDAI, IKS, JSWINFRA, JSWSTEEL, KEI, LEMONTREE, M&amp;M, M&amp;MFIN, NCC, OLECTRA, PHOENIXLTD, SAILIFE, SBICARD, SCI, SONACOMS, TATAELXSI, TEJASNET, THELEELA, TIINDIA, TORNTPHARM, WIPRO</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>23</v>
+        <v>53</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>IDFCFIRSTB, IEX, 360ONE, ABCAPITAL, ADANIENT, APLAPOLLO, BAJAJFINSV, BPCL, GLENMARK, GRASIM, HDFCBANK, HINDALCO, HINDZINC, INDHOTEL, INDIANB, IOC, JSWSTEEL, MUTHOOTFIN, PETRONET, RBLBANK, SONACOMS, SRF, TATASTEEL</t>
+          <t>APLLTD, IDFCFIRSTB, IEX, IRB, 360ONE, ABCAPITAL, ABREL, ACC, ACMESOLAR, ADANIENT, ANANDRATHI, APLAPOLLO, BAJAJFINSV, BASF, BPCL, BSOFT, CEATLTD, CGCL, COHANCE, CYIENT, DCMSHRIRAM, GLENMARK, GRASIM, HDFCBANK, HINDALCO, HINDZINC, IDBI, IFCI, IKS, INDHOTEL, INDIAMART, INDIANB, IOC, IPCALAB, ITI, JMFINANCIL, JPPOWER, JSWSTEEL, LEMONTREE, MAHABANK, MAPMYINDIA, MGL, MOTILALOFS, MUTHOOTFIN, NAM-INDIA, PETRONET, RBLBANK, RITES, SCHNEIDER, SIGNATURE, SONACOMS, SRF, TATASTEEL</t>
         </is>
       </c>
     </row>
@@ -1017,16 +1017,16 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>BIOCON, CAMS, CHOLAFIN, DRREDDY, PPLPHARMA, TATAELXSI</t>
+          <t>CREDITACC, GPIL, JSWINFRA, TARIL, TBOTEK, AADHARHFC, BIOCON, CAMS, CHOICEIN, CHOLAFIN, DEEPAKNTR, DRREDDY, GODREJIND, IRCTC, JMFINANCIL, JPPOWER, PCBL, PPLPHARMA, TATAELXSI, TRITURBINE, VENTIVE, WELCORP, ZENTEC</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1042,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>32</v>
+        <v>75</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ASIANPAINT, GAIL, HEROMOTOCO, TVSMOTOR, ABB, CIPLA, COALINDIA, ETERNAL, FORTIS, GODREJCP, HINDUNILVR, ICICIPRULI, IDEA, INOXWIND, KOTAKBANK, LT, LUPIN, MARICO, MAZDOCK, NATIONALUM, PETRONET, PGEL, PIIND, PNBHOUSING, SHREECEM, SIEMENS, SUNPHARMA, TATACONSUM, TATAPOWER, ULTRACEMCO, WIPRO, ZYDUSLIFE</t>
+          <t>ASIANPAINT, GODFRYPHLP, VMM, ARE&amp;M, ATGL, GAIL, HEROMOTOCO, HOMEFIRST, NCC, PFIZER, TEJASNET, TVSMOTOR, ABB, APLLTD, APOLLOTYRE, BATAINDIA, BHARTIHEXA, BIKAJI, CASTROLIND, CHALET, CHAMBLFERT, CIPLA, COALINDIA, COROMANDEL, CRAFTSMAN, EIHOTEL, ETERNAL, FINCABLES, FIVESTAR, FLUOROCHEM, FORTIS, GODREJCP, GRAVITA, GUJGASLTD, GVT&amp;D, HINDUNILVR, HONASA, ICICIPRULI, IDEA, INOXWIND, ITCHOTELS, JYOTHYLAB, KOTAKBANK, KSB, LATENTVIEW, LT, LUPIN, MAHSCOOTER, MAHSEAMLES, MARICO, MAZDOCK, METROPOLIS, NATIONALUM, NAVINFLUOR, NH, NIACL, NIVABUPA, NUVOCO, PETRONET, PGEL, PIIND, PNBHOUSING, RCF, SAPPHIRE, SHREECEM, SIEMENS, STARHEALTH, SUNPHARMA, TATACONSUM, TATAPOWER, TITAGARH, ULTRACEMCO, USHAMART, WIPRO, ZYDUSLIFE</t>
         </is>
       </c>
     </row>
@@ -1067,16 +1067,16 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>42</v>
+        <v>108</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BLUESTARCO, BHEL, COLPAL, CONCOR, DABUR, DMART, EXIDEIND, FORTIS, GODREJCP, HAL, HDFCAMC, HINDUNILVR, ICICIBANK, INDHOTEL, JSWSTEEL, KPITTECH, LODHA, MANAPPURAM, MANKIND, MARICO, MPHASIS, NESTLEIND, OFSS, ONGC, PATANJALI, PAYTM, PGEL, PNB, POLICYBZR, PRESTIGE, SHREECEM, SIEMENS, SUPREMEIND, SUZLON, SYNGENE, TCS, TITAN, TORNTPOWER, ULTRACEMCO, UNITDSPR, UPL, VBL</t>
+          <t>3MINDIA, ACMESOLAR, AWL, BLUESTARCO, DEEPAKFERT, EMCURE, ERIS, GLAND, MRPL, PGHH, RAINBOW, RITES, WOCKPHARMA, AADHARHFC, ABLBL, AGARWALEYE, AIIL, AJANTPHARM, AKUMS, ALKYLAMINE, ALOKINDS, ANANTRAJ, APTUS, BHARTIHEXA, BHEL, BIKAJI, BRIGADE, CLEAN, COLPAL, CONCOR, COROMANDEL, CUB, DABUR, DMART, DOMS, EIDPARRY, EMAMILTD, ENRIN, ESCORTS, EXIDEIND, FACT, FORTIS, FSL, GILLETTE, GODREJCP, HAL, HAPPSTMNDS, HDFCAMC, HEG, HINDUNILVR, ICICIBANK, INDHOTEL, INOXINDIA, IPCALAB, ITCHOTELS, JSWCEMENT, JSWSTEEL, JUBLPHARMA, JYOTHYLAB, KIRLOSBROS, KPIL, KPITTECH, LATENTVIEW, LLOYDSME, LODHA, MANAPPURAM, MANKIND, MANYAVAR, MARICO, MPHASIS, NATCOPHARM, NESTLEIND, NIACL, NIVABUPA, NUVOCO, OFSS, ONGC, PATANJALI, PAYTM, PGEL, PNB, POLICYBZR, PRESTIGE, PVRINOX, RAMCOCEM, RCF, RPOWER, SAPPHIRE, SAREGAMA, SHREECEM, SHYAMMETL, SIEMENS, SONATSOFTW, STARHEALTH, SUPREMEIND, SUZLON, SYNGENE, TCS, TITAN, TORNTPOWER, TTML, ULTRACEMCO, UNITDSPR, UPL, USHAMART, VBL, WHIRLPOOL, ZFCVINDIA</t>
         </is>
       </c>
     </row>
@@ -1092,7 +1092,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>31</v>
+        <v>66</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>MAXHEALTH, BANKINDIA, CROMPTON, HINDPETRO, MUTHOOTFIN, PIDILITIND, SAMMAANCAP, UNIONBANK, ABCAPITAL, APLAPOLLO, BAJAJ-AUTO, BAJAJFINSV, BAJAJHLDNG, BPCL, DALBHARAT, DLF, GLENMARK, HINDALCO, HINDZINC, INDIANB, IOC, IRFC, MOTHERSON, NBCC, NTPC, PAGEIND, PERSISTENT, POWERINDIA, RBLBANK, RVNL, SOLARINDS</t>
+          <t>ECLERX, MAXHEALTH, TRIVENI, AEGISLOG, AIAENG, BANKINDIA, CROMPTON, FINCABLES, HINDCOPPER, HINDPETRO, JKCEMENT, MUTHOOTFIN, PIDILITIND, SAMMAANCAP, UNIONBANK, ABBOTINDIA, ABCAPITAL, AJANTPHARM, AKZOINDIA, APLAPOLLO, BAJAJ-AUTO, BAJAJFINSV, BAJAJHLDNG, BPCL, CAMPUS, CAPLIPOINT, CCL, CHAMBLFERT, CLEAN, CRISIL, DALBHARAT, DLF, GLAXO, GLENMARK, GODREJAGRO, GRANULES, GRSE, HEXT, HFCL, HINDALCO, HINDZINC, IGIL, INDIANB, INOXINDIA, IOC, IRFC, MAHSEAMLES, MOTHERSON, NAM-INDIA, NBCC, NEULANDLAB, NLCINDIA, NTPC, PAGEIND, PERSISTENT, POWERINDIA, PRAJIND, PVRINOX, RBLBANK, RHIM, RVNL, SOBHA, SOLARINDS, TATACHEM, TATACOMM, UBL</t>
         </is>
       </c>
     </row>
@@ -1117,16 +1117,16 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>BLUESTARCO, DIVISLAB, FEDERALBNK, ICICIGI, MFSL, NESTLEIND, SHREECEM, SRF, TORNTPOWER, ULTRACEMCO, UNITDSPR, AXISBANK, BANKBARODA, COFORGE, COLPAL, CUMMINSIND, DABUR, DMART, GRASIM, HDFCBANK, ICICIPRULI, INFY, KOTAKBANK, MARICO, MAXHEALTH, NAUKRI, PATANJALI, PAYTM, POLICYBZR, SUPREMEIND, SWIGGY, TECHM, UNOMINDA, UPL, VBL</t>
+          <t>AJANTPHARM, KARURVYSYA, 3MINDIA, BLUESTARCO, DIVISLAB, EIDPARRY, FEDERALBNK, ICICIGI, MFSL, NESTLEIND, RAMCOCEM, SHREECEM, SJVN, SRF, TORNTPOWER, ULTRACEMCO, UNITDSPR, AGARWALEYE, ALKYLAMINE, APOLLOTYRE, AXISBANK, BANKBARODA, COFORGE, COLPAL, CUB, CUMMINSIND, DABUR, DMART, EMAMILTD, ESCORTS, FACT, GILLETTE, GMDCLTD, GODREJIND, GRAPHITE, GRASIM, HDFCBANK, HYUNDAI, ICICIPRULI, INFY, JBCHEPHARM, JSWCEMENT, KOTAKBANK, LALPATHLAB, LATENTVIEW, LLOYDSME, MARICO, MAXHEALTH, NAUKRI, PATANJALI, PAYTM, POLICYBZR, SUPREMEIND, SWIGGY, TECHM, UNOMINDA, UPL, USHAMART, VBL, WHIRLPOOL, ZFCVINDIA</t>
         </is>
       </c>
     </row>
@@ -1142,16 +1142,16 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>31</v>
+        <v>94</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>BANKBARODA, LICHSGFIN, BEL, BIOCON, BRITANNIA, CGPOWER, CHOLAFIN, COLPAL, DABUR, DELHIVERY, DMART, GMRAIRPORT, GODREJCP, GODREJPROP, HDFCLIFE, HINDUNILVR, ICICIGI, LODHA, LTM, MCX, NHPC, NYKAA, PIDILITIND, PREMIERENE, SONACOMS, SUPREMEIND, SUZLON, VEDL, VOLTAS, WAAREEENER, YESBANK</t>
+          <t>ALKYLAMINE, BLUEDART, ABBOTINDIA, ABREL, ACE, BAJAJHFL, BANKBARODA, BSOFT, ERIS, LICHSGFIN, NIVABUPA, NTPCGREEN, POONAWALLA, RAMCOCEM, SCHNEIDER, WOCKPHARMA, AARTIIND, AKUMS, ANANDRATHI, ANANTRAJ, APARINDS, ATHERENERG, ATUL, BBTC, BEL, BIKAJI, BIOCON, BRITANNIA, CAMPUS, CARBORUNIV, CCL, CESC, CGPOWER, CHALET, CHOLAFIN, COLPAL, CUB, DABUR, DATAPATTNS, DBREALTY, DELHIVERY, DEVYANI, DMART, ELECON, EMCURE, FINCABLES, GESHIP, GLAND, GMRAIRPORT, GODREJCP, GODREJPROP, GRAVITA, HDFCLIFE, HINDUNILVR, HSCL, ICICIGI, IGIL, INDGN, ITCHOTELS, JBMA, LODHA, LTM, LTTS, MAPMYINDIA, MCX, MRPL, NHPC, NIACL, NUVOCO, NYKAA, OLAELEC, PGHH, PIDILITIND, PREMIERENE, PVRINOX, RAILTEL, RAINBOW, RCF, REDINGTON, SARDAEN, SCHAEFFLER, SIGNATURE, SONACOMS, STARHEALTH, SUPREMEIND, SUZLON, SWANCORP, TIMKEN, VEDL, VOLTAS, WAAREEENER, WELSPUNLIV, YESBANK, ZENSARTECH</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>CROMPTON, DIXON, APOLLOHOSP, BAJAJ-AUTO, BANDHANBNK, COLPAL, DABUR, DRREDDY, HINDPETRO, HINDUNILVR, JIOFIN, KFINTECH, PAYTM, PERSISTENT, POLICYBZR, TORNTPHARM, WAAREEENER</t>
+          <t>ASTERDM, BAYERCROP, BLUEDART, CROMPTON, DIXON, ECLERX, ENGINERSIN, LTFOODS, NAVA, PRAJIND, SUMICHEM, WHIRLPOOL, ZENTEC, APOLLOHOSP, ASAHIINDIA, ASTRAZEN, BAJAJ-AUTO, BANDHANBNK, BBTC, BLS, BLUEJET, COLPAL, DABUR, DRREDDY, FINPIPE, HINDPETRO, HINDUNILVR, IOB, JIOFIN, JSWCEMENT, KFINTECH, PAYTM, PERSISTENT, POLICYBZR, SAGILITY, SAPPHIRE, SBFC, TORNTPHARM, TRIVENI, VIJAYA, WAAREEENER</t>
         </is>
       </c>
     </row>
@@ -1192,7 +1192,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ADANIPORTS, ADANIGREEN, SAMMAANCAP, BANKINDIA, BDL, BHARATFORG, BHARTIARTL, BPCL, BSE, CDSL, HINDALCO, HINDZINC, INDIANB, INDUSTOWER, IOC, JINDALSTEL, KALYANKJIL, LAURUSLABS, MUTHOOTFIN, PATANJALI, PHOENIXLTD, PIIND, RBLBANK, RECLTD, RELIANCE, SBICARD, SRF, TIINDIA</t>
+          <t>ADANIPORTS, KPRMILL, ADANIGREEN, DEVYANI, HINDCOPPER, NLCINDIA, SAMMAANCAP, ADANIPOWER, AGARWALEYE, AKZOINDIA, BANKINDIA, BDL, BHARATFORG, BHARTIARTL, BPCL, BSE, CASTROLIND, CDSL, FIRSTCRY, FIVESTAR, GSPL, GUJGASLTD, GVT&amp;D, HINDALCO, HINDZINC, HONASA, INDIANB, INDUSTOWER, IOC, ITI, JINDALSTEL, JKCEMENT, JKTYRE, KALYANKJIL, LAURUSLABS, LINDEINDIA, MUTHOOTFIN, NAM-INDIA, NAVINFLUOR, NSLNISP, ONESOURCE, PATANJALI, PHOENIXLTD, PIIND, RBLBANK, RECLTD, RELIANCE, SBICARD, SCI, SOBHA, SRF, SUNDRMFAST, TIINDIA, TIMKEN</t>
         </is>
       </c>
     </row>
@@ -1217,16 +1217,16 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>ADANIGREEN, BRITANNIA, CONCOR, HCLTECH, IDFCFIRSTB, INFY, JUBLFOOD, KPITTECH, NESTLEIND, SYNGENE, TCS</t>
+          <t>KIRLOSENG, THERMAX, ABSLAMC, ADANIGREEN, AEGISVOPAK, AFCONS, BERGEPAINT, BRITANNIA, CONCOR, ENRIN, GODFRYPHLP, HAPPSTMNDS, HCLTECH, IDBI, IDFCFIRSTB, INFY, INTELLECT, JUBLFOOD, KPIL, KPITTECH, NATCOPHARM, NESTLEIND, RADICO, SAILIFE, SONATSOFTW, SYNGENE, TCS, WELCORP</t>
         </is>
       </c>
     </row>
@@ -1242,16 +1242,16 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>36</v>
+        <v>89</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>CUMMINSIND, KOTAKBANK, OIL, ABCAPITAL, ASTRAL, AUROPHARMA, BAJAJ-AUTO, BANKBARODA, BANKINDIA, BHARATFORG, CANBK, CHOLAFIN, GMRAIRPORT, HINDPETRO, ICICIBANK, IDFCFIRSTB, INDIANB, JIOFIN, LICI, MANKIND, MARICO, MAZDOCK, NBCC, PATANJALI, PGEL, PNB, RBLBANK, SAMMAANCAP, SBILIFE, SBIN, SHRIRAMFIN, SUPREMEIND, TMPV, UNIONBANK, UNOMINDA, WIPRO</t>
+          <t>NIVABUPA, IGIL, CUMMINSIND, JUBLPHARMA, KOTAKBANK, OIL, ZEEL, ABBOTINDIA, ABCAPITAL, ABFRL, ABREL, ABSLAMC, AIIL, ARE&amp;M, ASTRAL, ASTRAZEN, ATUL, AUROPHARMA, BAJAJ-AUTO, BAJAJHFL, BANKBARODA, BANKINDIA, BASF, BERGEPAINT, BHARATFORG, BRIGADE, CANBK, CHAMBLFERT, CHENNPETRO, CHOICEIN, CHOLAFIN, COHANCE, COROMANDEL, DBREALTY, DEEPAKFERT, DEEPAKNTR, EIHOTEL, ENGINERSIN, FINCABLES, FINPIPE, FIVESTAR, FORCEMOT, GMRAIRPORT, GODFRYPHLP, GRAVITA, GSPL, HINDPETRO, ICICIBANK, IDFCFIRSTB, IKS, INDGN, INDIANB, JIOFIN, JSWINFRA, JWL, KSB, LICI, MANKIND, MANYAVAR, MARICO, MAZDOCK, MRPL, NAVINFLUOR, NBCC, PATANJALI, PGEL, PNB, POONAWALLA, RBLBANK, SAMMAANCAP, SBFC, SBILIFE, SBIN, SHRIRAMFIN, SHYAMMETL, SUMICHEM, SUNDRMFAST, SUPREMEIND, TARIL, TATAINVEST, TEJASNET, TMPV, UNIONBANK, UNOMINDA, VMM, WHIRLPOOL, WIPRO, WOCKPHARMA, ZFCVINDIA</t>
         </is>
       </c>
     </row>
@@ -1267,16 +1267,16 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>JSWENERGY, 360ONE, ADANIPORTS, CDSL, CROMPTON, GODREJCP, HDFCLIFE, HEROMOTOCO, INDIGO, JIOFIN, MARICO, PGEL</t>
+          <t>PCBL, JSWENERGY, 360ONE, ACE, ACMESOLAR, ADANIPORTS, ADANIPOWER, ALOKINDS, ATHERENERG, BATAINDIA, CDSL, CROMPTON, CYIENT, ECLERX, GODREJCP, GRSE, HDFCLIFE, HEROMOTOCO, INDIGO, JIOFIN, JYOTHYLAB, KSB, MARICO, PGEL, SARDAEN, THELEELA</t>
         </is>
       </c>
     </row>
@@ -1292,7 +1292,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>CIPLA, DABUR, MARUTI, TORNTPOWER, VOLTAS, APOLLOHOSP, BAJFINANCE, HAVELLS, INFY, JUBLFOOD, KEI, MUTHOOTFIN, OFSS, PAGEIND, TECHM</t>
+          <t>ADANIPOWER, CARBORUNIV, CIPLA, DABUR, J&amp;KBANK, MARUTI, OLECTRA, TORNTPOWER, VOLTAS, AFFLE, APOLLOHOSP, ATUL, BAJFINANCE, FINCABLES, HAVELLS, INFY, INTELLECT, JBCHEPHARM, JKCEMENT, JUBLFOOD, KAJARIACER, KEI, MUTHOOTFIN, NAM-INDIA, NUVOCO, OFSS, PAGEIND, RADICO, RAINBOW, SARDAEN, SONATSOFTW, SUNDRMFAST, SYRMA, TECHM, TITAGARH, TRIVENI, ZENSARTECH</t>
         </is>
       </c>
     </row>
@@ -1317,16 +1317,16 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SYNGENE, TRENT, BAJAJFINSV, BAJAJHLDNG, HDFCBANK, INDIGO, LICI, MAXHEALTH, MCX, MOTHERSON, NMDC, PERSISTENT, PFC, SBICARD, TCS, TVSMOTOR, WAAREEENER</t>
+          <t>CHOLAHLDNG, IPCALAB, TTML, AKUMS, BBTC, CEATLTD, JWL, LTFOODS, MRF, OLECTRA, RHIM, SIGNATURE, SYNGENE, TRENT, ABLBL, ACMESOLAR, ASTERDM, ATHERENERG, BAJAJFINSV, BAJAJHLDNG, BALRAMCHIN, DEEPAKFERT, GRANULES, HDFCBANK, INDIGO, ITCHOTELS, JYOTHYLAB, LICI, MAXHEALTH, MCX, METROPOLIS, MINDACORP, MOTHERSON, NMDC, PERSISTENT, PFC, RAINBOW, SBICARD, TCS, TVSMOTOR, VENTIVE, WAAREEENER</t>
         </is>
       </c>
     </row>
@@ -1342,7 +1342,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>CIPLA, DABUR, GMRAIRPORT, IREDA, KAYNES, PPLPHARMA, TATATECH, TRENT, YESBANK</t>
+          <t>BLUEJET, CIPLA, DABUR, HAPPSTMNDS, J&amp;KBANK, JSWCEMENT, RHIM, SCI, AADHARHFC, AKUMS, BEML, BIKAJI, CAPLIPOINT, COCHINSHIP, CRAFTSMAN, DATAPATTNS, FLUOROCHEM, GMRAIRPORT, GVT&amp;D, IFCI, IREDA, JBCHEPHARM, JPPOWER, JUBLPHARMA, JYOTICNC, KAYNES, KPIL, LALPATHLAB, LLOYDSME, METROPOLIS, MSUMI, NATCOPHARM, PFIZER, PPLPHARMA, SCHAEFFLER, TATATECH, TITAGARH, TRENT, TRIDENT, YESBANK</t>
         </is>
       </c>
     </row>
@@ -1367,16 +1367,16 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>AMBUJACEM, BAJAJFINSV, BLUESTARCO, EICHERMOT, JSWSTEEL, MAXHEALTH, NAUKRI, TVSMOTOR, WIPRO</t>
+          <t>CHOLAHLDNG, MINDACORP, SIGNATURE, AKZOINDIA, AMBUJACEM, BAJAJFINSV, BLUESTARCO, DOMS, EICHERMOT, ENDURANCE, GVT&amp;D, HAPPSTMNDS, JSWSTEEL, MAXHEALTH, MMTC, NAUKRI, RAINBOW, SBFC, SCI, TVSMOTOR, WIPRO</t>
         </is>
       </c>
     </row>
@@ -1392,16 +1392,16 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>GODREJPROP, HAVELLS, M&amp;M, RECLTD, WAAREEENER, ANGELONE, BAJAJ-AUTO, COFORGE, DALBHARAT, HDFCBANK, KPITTECH, MOTHERSON, MUTHOOTFIN, NATIONALUM, NHPC, NMDC, NUVAMA, PAYTM, PFC, PIIND, PREMIERENE, SBICARD, TATACONSUM, TATAELXSI</t>
+          <t>AFCONS, USHAMART, FLUOROCHEM, GODREJPROP, HAVELLS, HYUNDAI, IRB, JINDALSAW, M&amp;M, NIACL, RECLTD, WAAREEENER, AIAENG, ANANTRAJ, ANGELONE, APOLLOTYRE, ASAHIINDIA, ASTERDM, BAJAJ-AUTO, BLS, CEATLTD, CENTURYPLY, COFORGE, CONCORDBIO, CRISIL, DALBHARAT, EMAMILTD, GLAND, GMDCLTD, GRSE, HDFCBANK, HEXT, JBCHEPHARM, JPPOWER, JUBLPHARMA, KAJARIACER, KARURVYSYA, KPITTECH, MANYAVAR, MOTHERSON, MOTILALOFS, MSUMI, MUTHOOTFIN, NATIONALUM, NHPC, NMDC, NUVAMA, PAYTM, PFC, PIIND, PREMIERENE, PTCIL, RITES, SBICARD, SUNDARMFIN, TATACONSUM, TATAELXSI</t>
         </is>
       </c>
     </row>
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>CAMS, DIXON, ABB, BDL, CDSL, CGPOWER, CHOLAFIN, CROMPTON, DALBHARAT, GLENMARK, IDEA, KAYNES, KFINTECH, MFSL, NATIONALUM, PETRONET, POWERINDIA, PRESTIGE, SRF</t>
+          <t>CAMS, DIXON, RPOWER, ECLERX, INDIAMART, JINDALSAW, MAHSCOOTER, NCC, 3MINDIA, AADHARHFC, ABB, ANANDRATHI, APOLLOTYRE, ASAHIINDIA, BDL, CDSL, CGPOWER, CHOLAFIN, CONCORDBIO, CRISIL, CROMPTON, DALBHARAT, EIDPARRY, EMAMILTD, ERIS, FIRSTCRY, GLAND, GLENMARK, GODREJIND, HEXT, IDEA, IGL, JUBLINGREA, KAYNES, KFINTECH, MAPMYINDIA, MFSL, NATIONALUM, ONESOURCE, PCBL, PETRONET, POWERINDIA, PRESTIGE, SARDAEN, SRF, TECHNOE, THELEELA, TRIDENT</t>
         </is>
       </c>
     </row>
@@ -1442,7 +1442,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>31</v>
+        <v>66</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>CAMS, GAIL, INDUSTOWER, JINDALSTEL, ASIANPAINT, COALINDIA, DLF, GRASIM, HINDZINC, INDUSINDBK, PNBHOUSING, SONACOMS, TATASTEEL, VEDL, AMBER, AUBANK, BLUESTARCO, BOSCHLTD, DIXON, HCLTECH, HDFCAMC, INOXWIND, IOC, IRFC, KEI, LUPIN, PAGEIND, PGEL, PIIND, POWERGRID, PRESTIGE</t>
+          <t>BAYERCROP, CAMS, GAIL, INDUSTOWER, JINDALSTEL, APARINDS, ASIANPAINT, BHARTIHEXA, CESC, COALINDIA, CUB, DLF, ENRIN, GRASIM, HINDZINC, INDUSINDBK, IOB, JSL, NEWGEN, NSLNISP, PNBHOUSING, RAMCOCEM, SONACOMS, TATASTEEL, VEDL, AARTIIND, AMBER, ATGL, AUBANK, BALKRISIND, BLUESTARCO, BOSCHLTD, CENTRALBK, CYIENT, DCMSHRIRAM, DIXON, GODIGIT, GODREJAGRO, GPIL, GRAPHITE, HCLTECH, HDFCAMC, INOXINDIA, INOXWIND, IOC, IRCTC, IRFC, KEI, KIMS, KPIL, LUPIN, ONESOURCE, PAGEIND, PGEL, PIIND, POWERGRID, PRESTIGE, RAILTEL, RPOWER, SCHAEFFLER, SIGNATURE, THERMAX, TRITURBINE, VTL, ZENSARTECH, ZENTEC</t>
         </is>
       </c>
     </row>
@@ -1467,7 +1467,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>IEX, POLICYBZR, ABB, BAJAJ-AUTO, CGPOWER, COALINDIA, EXIDEIND, HDFCAMC, HINDALCO, ICICIGI, KALYANKJIL, LAURUSLABS, MCX, NTPC, PAYTM, RELIANCE, SIEMENS, SUNPHARMA, TMPV, TORNTPOWER</t>
+          <t>3MINDIA, AAVAS, AWL, DCMSHRIRAM, HEG, HSCL, IEX, JBMA, NSLNISP, POLICYBZR, PVRINOX, SCHNEIDER, VGUARD, VMM, ABB, ARE&amp;M, ATUL, BAJAJ-AUTO, BAJAJHFL, BHARTIHEXA, CERA, CGCL, CGPOWER, CHALET, COALINDIA, CRAFTSMAN, DEEPAKFERT, EXIDEIND, FIRSTCRY, GMDCLTD, GRANULES, HDFCAMC, HINDALCO, HOMEFIRST, ICICIGI, INOXINDIA, ITCHOTELS, KALYANKJIL, KIRLOSENG, LAURUSLABS, MCX, NAM-INDIA, NIACL, NTPC, PAYTM, RELIANCE, RRKABEL, SIEMENS, SUNPHARMA, TECHNOE, TMPV, TORNTPOWER, UBL, VENTIVE</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1492,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>35</v>
+        <v>92</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ETERNAL, APLAPOLLO, ASIANPAINT, CONCOR, CUMMINSIND, GAIL, HINDPETRO, JINDALSTEL, LT, OBEROIRLTY, OIL, SHREECEM, SYNGENE, UNIONBANK, 360ONE, AUROPHARMA, BHEL, DIVISLAB, GMRAIRPORT, HAL, HDFCLIFE, INDUSTOWER, INOXWIND, ITC, JSWSTEEL, KALYANKJIL, LICI, ONGC, PGEL, PIDILITIND, PNBHOUSING, SBIN, SONACOMS, SWIGGY, VBL</t>
+          <t>ETERNAL, HBLENGINE, AARTIIND, ABSLAMC, APLAPOLLO, ASIANPAINT, BIKAJI, CANFINHOME, CONCOR, CUMMINSIND, DBREALTY, FINPIPE, GAIL, HINDPETRO, JINDALSTEL, JSWINFRA, KPRMILL, LT, NTPCGREEN, OBEROIRLTY, OIL, SAGILITY, SHREECEM, SUMICHEM, SYNGENE, TATACHEM, UNIONBANK, WELCORP, ZEEL, ZFCVINDIA, 360ONE, ABLBL, AIIL, AJANTPHARM, APLLTD, ARE&amp;M, AUROPHARMA, BHEL, CLEAN, COHANCE, DIVISLAB, ELGIEQUIP, EMCURE, ESCORTS, FACT, FORCEMOT, GESHIP, GILLETTE, GMRAIRPORT, GODFRYPHLP, GPIL, GRAVITA, HAL, HDFCLIFE, INDIACEM, INDUSTOWER, INOXWIND, IPCALAB, ITC, JKCEMENT, JSWSTEEL, JUBLPHARMA, JWL, KALYANKJIL, KEC, LALPATHLAB, LICI, MANYAVAR, MINDACORP, MRPL, MSUMI, NAVINFLUOR, NEWGEN, ONGC, PGEL, PIDILITIND, PNBHOUSING, RAILTEL, RCF, SBIN, SHYAMMETL, SONACOMS, SUNDRMFAST, SWIGGY, TATAINVEST, TBOTEK, TIMKEN, UTIAMC, VBL, VENTIVE, VGUARD, ZENTEC</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>34</v>
+        <v>80</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1526,7 +1526,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>HINDALCO, HUDCO, ICICIPRULI, JUBLFOOD, RBLBANK, SHRIRAMFIN, ABCAPITAL, ADANIENSOL, ASTRAL, BANKBARODA, BANKINDIA, BIOCON, BRITANNIA, CANBK, FEDERALBNK, ICICIBANK, IDFCFIRSTB, INDIANB, IRFC, MANKIND, MFSL, MOTHERSON, NBCC, NMDC, NTPC, OBEROIRLTY, PATANJALI, PNB, POLYCAB, POWERINDIA, SAMMAANCAP, TMPV, UPL, WAAREEENER</t>
+          <t>AKZOINDIA, BLUEDART, CASTROLIND, CGCL, HINDALCO, HUDCO, ICICIPRULI, IIFL, JBMA, JKTYRE, JUBLFOOD, KIRLOSENG, POLYMED, RBLBANK, SCHNEIDER, SHRIRAMFIN, ABCAPITAL, ABFRL, ABREL, ABSLAMC, ACC, ADANIENSOL, ASTRAL, ASTRAZEN, ATGL, AWL, BALKRISIND, BANKBARODA, BANKINDIA, BATAINDIA, BIKAJI, BIOCON, BRITANNIA, BSOFT, CANBK, CENTRALBK, CHALET, CHENNPETRO, CHOICEIN, DEEPAKNTR, ELGIEQUIP, ENDURANCE, ENGINERSIN, FACT, FEDERALBNK, FINCABLES, HEG, HOMEFIRST, ICICIBANK, IDBI, IDFCFIRSTB, IKS, INDGN, INDIANB, INTELLECT, IRFC, MANKIND, MFSL, MOTHERSON, NBCC, NLCINDIA, NMDC, NTPC, OBEROIRLTY, OLECTRA, PATANJALI, PNB, POLYCAB, POWERINDIA, SAGILITY, SAILIFE, SAMMAANCAP, SAPPHIRE, SOBHA, TITAGARH, TMPV, UCOBANK, UPL, WAAREEENER, WOCKPHARMA</t>
         </is>
       </c>
     </row>
@@ -1542,7 +1542,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>25</v>
+        <v>65</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>LTF, PETRONET, SHREECEM, TORNTPOWER, WIPRO, ADANIENSOL, ADANIGREEN, BIOCON, BSE, CUMMINSIND, DMART, ETERNAL, HAL, HAVELLS, HEROMOTOCO, ICICIPRULI, ITC, MAZDOCK, MPHASIS, ONGC, RBLBANK, SWIGGY, UNIONBANK, UNITDSPR, VBL</t>
+          <t>AEGISVOPAK, ALKYLAMINE, CAMPUS, IGL, JMFINANCIL, LTF, MEDANTA, PETRONET, SBFC, SHREECEM, TORNTPOWER, WIPRO, 3MINDIA, ADANIENSOL, ADANIGREEN, AIIL, AKZOINDIA, APLLTD, ATGL, BIOCON, BLS, BLUEDART, BRIGADE, BSE, CANFINHOME, CARBORUNIV, CASTROLIND, CLEAN, CUMMINSIND, DEEPAKFERT, DMART, ELGIEQUIP, ENGINERSIN, ETERNAL, FACT, FINPIPE, FORCEMOT, GESHIP, GILLETTE, HAL, HAVELLS, HEROMOTOCO, ICICIPRULI, IDBI, INTELLECT, ITC, JKCEMENT, KEC, LINDEINDIA, MAZDOCK, METROPOLIS, MPHASIS, ONGC, POLYMED, RBLBANK, RCF, REDINGTON, SAPPHIRE, SWIGGY, TATACOMM, TIMKEN, UCOBANK, UNIONBANK, UNITDSPR, VBL</t>
         </is>
       </c>
     </row>
@@ -1567,16 +1567,16 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>COLPAL, ULTRACEMCO, BHARATFORG, DALBHARAT, HINDZINC, ICICIBANK, ICICIGI, LICI, LODHA, MANKIND, MUTHOOTFIN, PIDILITIND, POLYCAB, UNITDSPR</t>
+          <t>CERA, ACC, APTUS, COLPAL, FLUOROCHEM, GICRE, JWL, MAHSEAMLES, SAREGAMA, SJVN, ULTRACEMCO, AIIL, ALKYLAMINE, APLLTD, BATAINDIA, BAYERCROP, BHARATFORG, CHENNPETRO, COROMANDEL, DALBHARAT, DOMS, EIDPARRY, ERIS, FINCABLES, FIVESTAR, HINDZINC, ICICIBANK, ICICIGI, INDIAMART, INTELLECT, JKCEMENT, KEC, KPRMILL, LICI, LODHA, MANKIND, MUTHOOTFIN, PCBL, PGHH, PIDILITIND, POLYCAB, SAILIFE, SIGNATURE, SOBHA, TIMKEN, TITAGARH, UNITDSPR</t>
         </is>
       </c>
     </row>
@@ -1592,7 +1592,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>SRF, BANKINDIA, FORTIS, LTM, NESTLEIND, ASHOKLEY, AXISBANK, BAJAJHLDNG, BOSCHLTD, CDSL, DRREDDY, GODREJCP, HDFCBANK, HEROMOTOCO, INFY, JIOFIN, JSWENERGY, KEI, MAZDOCK, PAGEIND, PERSISTENT, SAIL, SUZLON, TECHM</t>
+          <t>SRF, BANKINDIA, FORTIS, LTM, NESTLEIND, STARHEALTH, SWANCORP, ASHOKLEY, ASTRAZEN, AXISBANK, BAJAJHLDNG, BBTC, BOSCHLTD, CDSL, CEATLTD, DRREDDY, EMAMILTD, FLUOROCHEM, GODREJCP, HDFCBANK, HEROMOTOCO, HFCL, INFY, JIOFIN, JSWENERGY, KAJARIACER, KEI, KIRLOSBROS, KPIL, MAHSCOOTER, MAZDOCK, NAM-INDIA, NIVABUPA, NUVOCO, OLECTRA, PAGEIND, PERSISTENT, RADICO, RCF, REDINGTON, SAIL, SARDAEN, SUZLON, TATACOMM, TECHM, TEJASNET, THELEELA</t>
         </is>
       </c>
     </row>
@@ -1617,7 +1617,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1626,7 +1626,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>ADANIGREEN, AXISBANK, BANDHANBNK, BHARATFORG, BHEL, BPCL, BRITANNIA, CGPOWER, HDFCBANK, ICICIGI, PERSISTENT, PREMIERENE, RELIANCE, TECHM</t>
+          <t>ABLBL, ADANIGREEN, AXISBANK, BANDHANBNK, BBTC, BHARATFORG, BHEL, BPCL, BRITANNIA, CCL, CEATLTD, CGPOWER, COCHINSHIP, EMCURE, HDFCBANK, ICICIGI, IFCI, ITI, MAHSCOOTER, PERSISTENT, PFIZER, PREMIERENE, RADICO, RELIANCE, RRKABEL, SUNDARMFIN, SUNTV, TECHM, THERMAX</t>
         </is>
       </c>
     </row>
@@ -1642,7 +1642,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>NAUKRI, PFC, HAVELLS, M&amp;M, POLICYBZR, BAJAJ-AUTO, BLUESTARCO, HINDUNILVR, JSWSTEEL, KAYNES, PNBHOUSING, SAIL, VEDL</t>
+          <t>BEML, MRF, NAUKRI, PFC, ALOKINDS, AWL, CARBORUNIV, HAVELLS, HSCL, M&amp;M, NIACL, POLICYBZR, TRITURBINE, VENTIVE, BAJAJ-AUTO, BALKRISIND, BHARTIHEXA, BLUEDART, BLUESTARCO, CENTRALBK, CUB, DCMSHRIRAM, ELECON, GMDCLTD, HEG, HINDUNILVR, INOXINDIA, JSWSTEEL, KAYNES, LTFOODS, MAHABANK, PNBHOUSING, RCF, SAIL, TBOTEK, VEDL, ZENSARTECH</t>
         </is>
       </c>
     </row>
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>OIL, BRITANNIA, DALBHARAT, HAL, ICICIBANK, LODHA, MANKIND, MCX, MOTHERSON, NMDC, PIDILITIND, PREMIERENE, SONACOMS</t>
+          <t>NIVABUPA, OIL, 3MINDIA, ARE&amp;M, BLS, BRITANNIA, CHENNPETRO, COHANCE, DALBHARAT, GRANULES, HAL, ICICIBANK, IGIL, IKS, INDIAMART, IOB, ITCHOTELS, LODHA, MANKIND, MCX, MOTHERSON, MSUMI, NMDC, PGHH, PIDILITIND, PREMIERENE, RAINBOW, SONACOMS, VTL, ZENTEC</t>
         </is>
       </c>
     </row>
@@ -1692,16 +1692,16 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>APLAPOLLO, CDSL, DLF, LICHSGFIN, OFSS, SOLARINDS, TIINDIA</t>
+          <t>SUNTV, AAVAS, ABSLAMC, AIIL, ANANDRATHI, ANANTRAJ, APLAPOLLO, BSOFT, CDSL, CREDITACC, DLF, FIRSTCRY, GODREJIND, HINDCOPPER, JSWCEMENT, JUBLINGREA, JYOTHYLAB, KIRLOSBROS, KPIL, LICHSGFIN, MAPMYINDIA, NTPCGREEN, OFSS, RITES, SAGILITY, SOLARINDS, TEJASNET, THELEELA, TIINDIA, TRIDENT</t>
         </is>
       </c>
     </row>
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>18</v>
+        <v>41</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -1726,7 +1726,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>CIPLA, DABUR, JIOFIN, MARICO, BANKINDIA, CUMMINSIND, INFY, INOXWIND, KFINTECH, KOTAKBANK, MARUTI, PGEL, SONACOMS, TATACONSUM, TECHM, TVSMOTOR, UNIONBANK, VBL</t>
+          <t>CIPLA, DABUR, J&amp;KBANK, JIOFIN, MARICO, NUVOCO, ASTRAZEN, BANKINDIA, BLUEDART, CGCL, CLEAN, CUMMINSIND, DOMS, FINPIPE, INFY, INOXWIND, INTELLECT, JKCEMENT, KFINTECH, KOTAKBANK, KSB, LTTS, MARUTI, MOTILALOFS, PCBL, PGEL, RAINBOW, RITES, SONACOMS, SUMICHEM, SUNDARMFIN, TATACONSUM, TBOTEK, TECHM, TRIVENI, TVSMOTOR, UNIONBANK, VBL, VIJAYA, WELSPUNLIV, ZFCVINDIA</t>
         </is>
       </c>
     </row>
@@ -1742,7 +1742,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>33</v>
+        <v>74</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -1751,7 +1751,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>AMBUJACEM, CHOLAFIN, MFSL, POWERINDIA, SYNGENE, ADANIENSOL, BEL, BIOCON, COFORGE, DIVISLAB, DMART, EICHERMOT, GODREJPROP, IDEA, INDHOTEL, INOXWIND, ITC, KEI, LICHSGFIN, MCX, MPHASIS, NYKAA, ONGC, PAGEIND, PNBHOUSING, PPLPHARMA, RBLBANK, TATAELXSI, TATAPOWER, TATATECH, TMPV, WIPRO, YESBANK</t>
+          <t>AMBUJACEM, CHOLAFIN, ECLERX, FSL, MFSL, NAVA, POWERINDIA, CHOLAHLDNG, SIGNATURE, SYNGENE, AAVAS, ADANIENSOL, ADANIPOWER, AKUMS, ALOKINDS, BAYERCROP, BEL, BIOCON, BLUEJET, CANFINHOME, CAPLIPOINT, CHALET, COFORGE, DATAPATTNS, DIVISLAB, DMART, EICHERMOT, ENGINERSIN, GESHIP, GILLETTE, GODREJAGRO, GODREJPROP, GRANULES, HYUNDAI, IDBI, IDEA, INDHOTEL, INOXWIND, IPCALAB, IRB, ITC, ITCHOTELS, JPPOWER, JYOTICNC, KEI, LICHSGFIN, LINDEINDIA, LLOYDSME, LTTS, MCX, MPHASIS, NAM-INDIA, NATCOPHARM, NCC, NYKAA, OLECTRA, ONGC, PAGEIND, PNBHOUSING, PPLPHARMA, PTCIL, RADICO, RBLBANK, SARDAEN, SCHAEFFLER, TATAELXSI, TATAPOWER, TATATECH, TMPV, TTML, UCOBANK, WELSPUNLIV, WIPRO, YESBANK</t>
         </is>
       </c>
     </row>
@@ -1767,16 +1767,16 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>360ONE, GLENMARK, INDIGO, IREDA, IRFC, KPITTECH, LUPIN, MAZDOCK, PHOENIXLTD, TATAPOWER, TCS, ULTRACEMCO, WAAREEENER</t>
+          <t>CRAFTSMAN, HONAUT, GUJGASLTD, SCI, 360ONE, ABSLAMC, ACMESOLAR, AKZOINDIA, ATHERENERG, AWL, CCL, EIDPARRY, ERIS, FORCEMOT, GLENMARK, HEG, HONASA, INDIAMART, INDIGO, IREDA, IRFC, KPITTECH, LALPATHLAB, LATENTVIEW, LUPIN, MANYAVAR, MAZDOCK, METROPOLIS, MGL, MINDACORP, MSUMI, PHOENIXLTD, RRKABEL, SCHAEFFLER, TATAPOWER, TCS, TECHNOE, THERMAX, ULTRACEMCO, WAAREEENER</t>
         </is>
       </c>
     </row>
@@ -1792,7 +1792,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>34</v>
+        <v>73</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>EXIDEIND, RECLTD, IDEA, MUTHOOTFIN, TATAELXSI, WIPRO, ANGELONE, ASHOKLEY, ASTRAL, BEL, BHARATFORG, BHARTIARTL, BSE, COFORGE, DELHIVERY, DMART, GLENMARK, GODREJPROP, HDFCAMC, HINDZINC, IEX, INFY, KPITTECH, LTF, LUPIN, MAZDOCK, NATIONALUM, NUVAMA, PATANJALI, PAYTM, PHOENIXLTD, RELIANCE, SUNPHARMA, TECHM</t>
+          <t>ATGL, EXIDEIND, RECLTD, CAMPUS, CRISIL, GLAND, GVT&amp;D, IDEA, ITI, MEDANTA, MOTILALOFS, MUTHOOTFIN, TATAELXSI, WIPRO, AEGISVOPAK, AJANTPHARM, ANGELONE, APOLLOTYRE, ASHOKLEY, ASTRAL, BALKRISIND, BALRAMCHIN, BEL, BHARATFORG, BHARTIARTL, BSE, CENTRALBK, COFORGE, CONCORDBIO, DELHIVERY, DMART, FIVESTAR, FORCEMOT, GLENMARK, GMDCLTD, GODIGIT, GODREJPROP, HDFCAMC, HEXT, HINDZINC, HONASA, HYUNDAI, IEX, IFCI, INFY, IRB, JMFINANCIL, KAJARIACER, KARURVYSYA, KIMS, KPITTECH, LTF, LUPIN, M&amp;MFIN, MAHSCOOTER, MANYAVAR, MAZDOCK, MGL, NATIONALUM, NIACL, NIVABUPA, NUVAMA, PATANJALI, PAYTM, PHOENIXLTD, PTCIL, RELIANCE, SUNDARMFIN, SUNPHARMA, SYRMA, TATACOMM, TECHM, WHIRLPOOL</t>
         </is>
       </c>
     </row>
@@ -1817,7 +1817,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>28</v>
+        <v>62</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -1826,7 +1826,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>AUROPHARMA, INDUSINDBK, SBILIFE, SBIN, CROMPTON, DLF, GMRAIRPORT, SAIL, TATASTEEL, VEDL, ABCAPITAL, AMBUJACEM, AUBANK, BAJAJFINSV, BDL, BHARATFORG, GRASIM, HAL, JSWSTEEL, KPITTECH, MANAPPURAM, MAXHEALTH, NBCC, NESTLEIND, PHOENIXLTD, POWERGRID, TORNTPOWER, TVSMOTOR</t>
+          <t>AUROPHARMA, ENRIN, INDUSINDBK, JSL, SBILIFE, SBIN, AFCONS, BASF, CESC, CROMPTON, CUB, DLF, EIHOTEL, FLUOROCHEM, GMRAIRPORT, IKS, IRCTC, KPIL, RAMCOCEM, SAIL, TATASTEEL, USHAMART, VEDL, ABCAPITAL, AIAENG, AMBUJACEM, APARINDS, ASAHIINDIA, AUBANK, BAJAJFINSV, BATAINDIA, BDL, BHARATFORG, BHARTIHEXA, CHOICEIN, COCHINSHIP, DCMSHRIRAM, EMAMILTD, FIVESTAR, GRASIM, GSPL, HAL, HOMEFIRST, HYUNDAI, IFCI, INDIACEM, IRB, JSWSTEEL, KPITTECH, MANAPPURAM, MAXHEALTH, NBCC, NESTLEIND, NH, PHOENIXLTD, POWERGRID, PVRINOX, SUNTV, SWANCORP, TORNTPOWER, TVSMOTOR, WHIRLPOOL</t>
         </is>
       </c>
     </row>
@@ -1842,7 +1842,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>44</v>
+        <v>98</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>COFORGE, GODREJPROP, SUPREMEIND, ANGELONE, COLPAL, HCLTECH, LT, NUVAMA, PAYTM, RECLTD, SUNPHARMA, ADANIENT, AMBER, APLAPOLLO, ASHOKLEY, BAJAJ-AUTO, BHARTIARTL, CAMS, CHOLAFIN, CONCOR, DALBHARAT, DELHIVERY, EICHERMOT, FORTIS, HEROMOTOCO, HINDUNILVR, ICICIBANK, IDFCFIRSTB, INDIANB, IOC, IRFC, KAYNES, KPITTECH, LICI, LODHA, LTM, LUPIN, MANKIND, NATIONALUM, NESTLEIND, PIDILITIND, RELIANCE, SAMMAANCAP, SRF</t>
+          <t>COFORGE, GODREJPROP, KIMS, SUPREMEIND, 3MINDIA, ANGELONE, APTUS, COLPAL, CONCORDBIO, GICRE, GLAND, GODIGIT, HCLTECH, HEXT, HONASA, JINDALSAW, KARURVYSYA, LT, MAHSEAMLES, NUVAMA, PAYTM, RECLTD, SAREGAMA, SJVN, SUNDARMFIN, SUNPHARMA, ABBOTINDIA, ABREL, ADANIENT, AIAENG, AMBER, APLAPOLLO, APOLLOTYRE, ASAHIINDIA, ASHOKLEY, BAJAJ-AUTO, BHARTIARTL, BRIGADE, CAMS, CANFINHOME, CHAMBLFERT, CHENNPETRO, CHOLAFIN, CONCOR, COROMANDEL, CRISIL, DALBHARAT, DEEPAKNTR, DELHIVERY, EICHERMOT, FORTIS, GODFRYPHLP, HBLENGINE, HEROMOTOCO, HFCL, HINDUNILVR, HYUNDAI, ICICIBANK, IDFCFIRSTB, IGL, INDIACEM, INDIANB, INTELLECT, IOC, IRFC, JKCEMENT, JKTYRE, JWL, KAJARIACER, KAYNES, KPITTECH, LICI, LODHA, LTM, LUPIN, M&amp;MFIN, MANKIND, MOTILALOFS, NATIONALUM, NESTLEIND, NTPCGREEN, PIDILITIND, POONAWALLA, PTCIL, RADICO, RELIANCE, SAGILITY, SAMMAANCAP, SHYAMMETL, SRF, STARHEALTH, SUNDRMFAST, SUNTV, TARIL, TBOTEK, TEJASNET, TRIDENT, WOCKPHARMA</t>
         </is>
       </c>
     </row>
@@ -1867,7 +1867,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>CAMS, IDEA, JINDALSTEL, ASIANPAINT, CUMMINSIND, DIXON, GAIL, HINDPETRO, UNIONBANK, BANKINDIA, BOSCHLTD, HDFCBANK, HUDCO, INDUSTOWER, JUBLFOOD, MOTHERSON, NMDC, PERSISTENT, POLYCAB, RELIANCE, SAIL, SAMMAANCAP, SBICARD, TCS, TIINDIA</t>
+          <t>CAMS, GRAVITA, IDEA, JINDALSTEL, AARTIIND, ASIANPAINT, BAJAJHFL, BASF, CUMMINSIND, DBREALTY, DIXON, EIHOTEL, FINPIPE, GAIL, GODIGIT, HINDPETRO, JSWINFRA, NAVINFLUOR, RPOWER, TATAINVEST, UNIONBANK, ZEEL, ZFCVINDIA, ABBOTINDIA, ABREL, ACC, ASTERDM, ASTRAZEN, ATGL, ATUL, BANKINDIA, BAYERCROP, BOSCHLTD, BRIGADE, CEATLTD, CHAMBLFERT, CLEAN, COROMANDEL, DEEPAKFERT, DEEPAKNTR, DOMS, ECLERX, FINCABLES, GODFRYPHLP, GPIL, GSPL, HDFCBANK, HUDCO, IIFL, INDIAMART, INDUSTOWER, JUBLFOOD, KIRLOSBROS, MOTHERSON, MRPL, NEWGEN, NMDC, PCBL, PERSISTENT, POLYCAB, POONAWALLA, RELIANCE, SAIL, SAMMAANCAP, SBICARD, SHYAMMETL, SUMICHEM, SUNDRMFAST, SWANCORP, TARIL, TCS, TEJASNET, TIINDIA, UBL, VMM</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1892,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>36</v>
+        <v>74</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO, COALINDIA, HCLTECH, IOC, POLICYBZR, PRESTIGE, VEDL, ABCAPITAL, ASTRAL, AUBANK, BANKBARODA, BEL, CAMS, CANBK, DLF, GRASIM, HAVELLS, HDFCLIFE, IDFCFIRSTB, INDIANB, INDUSINDBK, JIOFIN, JSWENERGY, KOTAKBANK, MARICO, MPHASIS, NBCC, OFSS, PATANJALI, PGEL, PNB, POWERGRID, RBLBANK, SHRIRAMFIN, SOLARINDS, TATASTEEL</t>
+          <t>APARINDS, AWL, BAJAJ-AUTO, BATAINDIA, BHARTIHEXA, CESC, COALINDIA, CUB, HCLTECH, HSCL, IGIL, IOC, JBMA, NSLNISP, PGHH, POLICYBZR, PRESTIGE, SCHNEIDER, TRITURBINE, VEDL, ABCAPITAL, ABFRL, ASTRAL, AUBANK, BANKBARODA, BEL, CAMS, CANBK, CHOICEIN, DCMSHRIRAM, DLF, ENGINERSIN, ENRIN, FLUOROCHEM, GLAXO, GRAPHITE, GRASIM, HAVELLS, HDFCLIFE, HEG, IDFCFIRSTB, IKS, INDGN, INDIANB, INDUSINDBK, IRCTC, JIOFIN, JSL, JSWENERGY, KOTAKBANK, KSB, LATENTVIEW, M&amp;MFIN, MARICO, MPHASIS, NBCC, NIVABUPA, OFSS, ONESOURCE, PATANJALI, PGEL, PNB, POWERGRID, PVRINOX, RAMCOCEM, RBLBANK, SARDAEN, SCHAEFFLER, SHRIRAMFIN, SOLARINDS, TATASTEEL, VENTIVE, VGUARD, WOCKPHARMA</t>
         </is>
       </c>
     </row>
@@ -1917,7 +1917,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>HINDALCO, OIL, SHREECEM, CGPOWER, COALINDIA, COFORGE, DMART, ETERNAL, GMRAIRPORT, HINDZINC, IREDA, JUBLFOOD, MANAPPURAM, MARUTI, SIEMENS, SUNPHARMA, SWIGGY, TORNTPOWER</t>
+          <t>CARBORUNIV, CGCL, CRAFTSMAN, HINDALCO, JUBLPHARMA, KIRLOSENG, NAM-INDIA, NSLNISP, OIL, SHREECEM, SUNDRMFAST, SYRMA, TATACHEM, ABBOTINDIA, BIKAJI, CGPOWER, CHAMBLFERT, COALINDIA, COCHINSHIP, COFORGE, COHANCE, DEEPAKNTR, DMART, ECLERX, ETERNAL, FINCABLES, GILLETTE, GMRAIRPORT, GODFRYPHLP, HINDZINC, IREDA, JUBLFOOD, KEC, KIRLOSBROS, KPIL, LEMONTREE, LTFOODS, MANAPPURAM, MANYAVAR, MARUTI, PFIZER, PTCIL, RRKABEL, SIEMENS, SUNPHARMA, SWIGGY, TITAGARH, TORNTPOWER, TRIDENT</t>
         </is>
       </c>
     </row>
@@ -1942,16 +1942,16 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>28</v>
+        <v>72</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>CUMMINSIND, LICI, TRENT, APLAPOLLO, BHEL, BLUESTARCO, CDSL, CONCOR, GODREJCP, HDFCLIFE, HINDPETRO, ICICIBANK, INDIGO, JSWSTEEL, KEI, LT, MANKIND, MOTHERSON, NAUKRI, NMDC, PAGEIND, PIDILITIND, PNBHOUSING, SBIN, SONACOMS, TORNTPHARM, UNIONBANK, WAAREEENER</t>
+          <t>AKZOINDIA, MINDACORP, CANFINHOME, CUMMINSIND, GRSE, HBLENGINE, JWL, LICI, SBFC, TRENT, ZEEL, ABLBL, ACMESOLAR, ADANIPOWER, AKUMS, APLAPOLLO, ATHERENERG, BHEL, BLUESTARCO, CASTROLIND, CDSL, CHENNPETRO, CHOLAHLDNG, CONCOR, DBREALTY, ELGIEQUIP, EMCURE, FACT, FINPIPE, GODFRYPHLP, GODREJCP, GRAVITA, HDFCLIFE, HINDPETRO, ICICIBANK, INDIACEM, INDIGO, JSWINFRA, JSWSTEEL, KEI, LT, MANKIND, MOTHERSON, MRPL, NAUKRI, NAVINFLUOR, NH, NMDC, NTPCGREEN, PAGEIND, PIDILITIND, PNBHOUSING, POLYMED, RAILTEL, RAINBOW, REDINGTON, RHIM, SAGILITY, SBIN, SHYAMMETL, SIGNATURE, SONACOMS, SUMICHEM, TARIL, TATAINVEST, TEJASNET, THELEELA, THERMAX, TORNTPHARM, UNIONBANK, WAAREEENER, ZFCVINDIA</t>
         </is>
       </c>
     </row>
@@ -1967,7 +1967,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -1976,7 +1976,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>DABUR, PPLPHARMA, YESBANK, CIPLA, DALBHARAT, NTPC, NYKAA, PGEL, SUPREMEIND, TATATECH, TRENT, VOLTAS, WAAREEENER</t>
+          <t>DABUR, DATAPATTNS, HAPPSTMNDS, J&amp;KBANK, JYOTHYLAB, JYOTICNC, PPLPHARMA, RHIM, YESBANK, ABREL, BLUEDART, BLUEJET, CAPLIPOINT, CENTURYPLY, CIPLA, DALBHARAT, IIFL, IPCALAB, JPPOWER, JSWCEMENT, LLOYDSME, MAHSCOOTER, NATCOPHARM, NTPC, NYKAA, PGEL, SAPPHIRE, SUPREMEIND, TATATECH, TITAGARH, TRENT, TTML, UBL, VOLTAS, WAAREEENER, ZENTEC</t>
         </is>
       </c>
     </row>
@@ -1992,16 +1992,16 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>UPL, ALKEM, BHARATFORG, DALBHARAT, INDUSTOWER, LAURUSLABS, SHREECEM, VOLTAS, ASIANPAINT, BSE, ETERNAL, HAVELLS, M&amp;M, MANKIND, MAZDOCK, PATANJALI, RVNL, TITAN, WAAREEENER</t>
+          <t>LINDEINDIA, UPL, ALKEM, BALKRISIND, BHARATFORG, CANFINHOME, DALBHARAT, DCMSHRIRAM, EMAMILTD, INDGN, INDUSTOWER, JKTYRE, LAURUSLABS, METROPOLIS, MINDACORP, NETWEB, RAINBOW, SHREECEM, VOLTAS, AEGISLOG, AEGISVOPAK, AFCONS, AJANTPHARM, ASIANPAINT, BLS, BSE, EMCURE, ETERNAL, GESHIP, GODFRYPHLP, GODREJAGRO, HAVELLS, JSWINFRA, LALPATHLAB, M&amp;M, MANKIND, MAZDOCK, MOTILALOFS, PATANJALI, RAILTEL, RAMCOCEM, RVNL, TITAN, VMM, WAAREEENER</t>
         </is>
       </c>
     </row>
@@ -2017,16 +2017,16 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>HCLTECH, IEX, PGEL, SRF, CGPOWER, CIPLA, DABUR, DALBHARAT, GODREJPROP, HINDUNILVR, ITC, LICHSGFIN, POWERINDIA, WAAREEENER</t>
+          <t>SWANCORP, VTL, ACE, BERGEPAINT, GODREJAGRO, HCLTECH, HONAUT, IEX, ITI, KIMS, LTTS, NETWEB, PGEL, SAPPHIRE, SRF, AFCONS, ASTERDM, BHARTIHEXA, CASTROLIND, CENTRALBK, CGPOWER, CHALET, CIPLA, DABUR, DALBHARAT, DCMSHRIRAM, FIVESTAR, GLAND, GODREJPROP, HINDUNILVR, INOXINDIA, INTELLECT, IPCALAB, ITC, KPRMILL, KSB, LICHSGFIN, MAHABANK, NEWGEN, NIVABUPA, POWERINDIA, SAGILITY, SJVN, TBOTEK, UTIAMC, WAAREEENER</t>
         </is>
       </c>
     </row>
@@ -2042,7 +2042,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>OFSS, ASTRAL, BHARTIARTL, CAMS, CDSL, HEROMOTOCO, HINDALCO, MAZDOCK, POWERINDIA, TITAN, ZYDUSLIFE</t>
+          <t>CCL, DOMS, HOMEFIRST, LINDEINDIA, OFSS, ASTRAL, BHARTIARTL, BLUEDART, CAMS, CDSL, COCHINSHIP, CUB, DATAPATTNS, DEEPAKNTR, FIRSTCRY, GRAPHITE, HEROMOTOCO, HINDALCO, IDBI, IGIL, JPPOWER, JSL, MAZDOCK, POWERINDIA, RADICO, TITAN, ZYDUSLIFE</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2067,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -2076,7 +2076,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>BHARATFORG, VOLTAS, BLUESTARCO, BSE, CAMS, CDSL, CROMPTON, IEX, KPITTECH, PIDILITIND, SYNGENE, TITAN, UNITDSPR</t>
+          <t>BHARATFORG, METROPOLIS, VOLTAS, BLUESTARCO, BSE, CAMS, CAPLIPOINT, CDSL, COHANCE, CROMPTON, DATAPATTNS, ENDURANCE, ENGINERSIN, FSL, IDBI, IEX, JPPOWER, JSL, KIRLOSBROS, KPITTECH, PIDILITIND, RADICO, REDINGTON, SYNGENE, SYRMA, TITAN, UNITDSPR</t>
         </is>
       </c>
     </row>
@@ -2092,7 +2092,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>20</v>
+        <v>59</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>EICHERMOT, JIOFIN, PIIND, AUROPHARMA, GRASIM, HCLTECH, HUDCO, INDIGO, INFY, KPITTECH, MARUTI, MAZDOCK, PAYTM, PGEL, SBICARD, SBILIFE, TORNTPOWER, VOLTAS, WIPRO, ZYDUSLIFE</t>
+          <t>ACC, EICHERMOT, FIVESTAR, ITCHOTELS, KSB, TBOTEK, BALRAMCHIN, BERGEPAINT, CONCORDBIO, HOMEFIRST, HONAUT, ITI, J&amp;KBANK, JIOFIN, NEULANDLAB, PIIND, SARDAEN, SOBHA, STARHEALTH, ZENTEC, 3MINDIA, ABLBL, ACE, AEGISVOPAK, ANANDRATHI, ANANTRAJ, AUROPHARMA, CAPLIPOINT, CHOLAHLDNG, FACT, FLUOROCHEM, GODFRYPHLP, GRASIM, GRSE, HCLTECH, HUDCO, INDIGO, INFY, INTELLECT, JBCHEPHARM, KPITTECH, MANYAVAR, MARUTI, MAZDOCK, NAM-INDIA, NAVA, PAYTM, PGEL, SAILIFE, SBICARD, SBILIFE, SUNDARMFIN, SWANCORP, TORNTPOWER, VIJAYA, VMM, VOLTAS, WIPRO, ZYDUSLIFE</t>
         </is>
       </c>
     </row>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>INFY, ANGELONE, VEDL, ABB, AMBER, ASIANPAINT, BHARTIARTL, DIVISLAB, GODREJPROP, HINDZINC, INDIANB, INDUSINDBK, MARICO, MUTHOOTFIN, NYKAA, PATANJALI, PETRONET, PGEL, PIDILITIND, PNBHOUSING, POWERGRID, RECLTD, RVNL, SAIL, TATACONSUM, YESBANK</t>
+          <t>INFY, ANGELONE, ECLERX, ENRIN, POONAWALLA, SJVN, VEDL, ABB, ABBOTINDIA, ABFRL, ADANIPOWER, AKUMS, AMBER, ARE&amp;M, ASIANPAINT, BATAINDIA, BHARTIARTL, BSOFT, CASTROLIND, CEATLTD, CERA, CHAMBLFERT, DBREALTY, DIVISLAB, GODREJPROP, HINDCOPPER, HINDZINC, INDIANB, INDUSINDBK, JKCEMENT, JKTYRE, JMFINANCIL, JUBLPHARMA, KPRMILL, LATENTVIEW, LEMONTREE, LTFOODS, MARICO, MINDACORP, MUTHOOTFIN, NAM-INDIA, NH, NLCINDIA, NYKAA, PATANJALI, PETRONET, PGEL, PIDILITIND, PNBHOUSING, POWERGRID, RAILTEL, RCF, RECLTD, RHIM, RVNL, SAIL, SUNDRMFAST, SWANCORP, TATACONSUM, TRIDENT, TRIVENI, YESBANK</t>
         </is>
       </c>
     </row>
@@ -2142,7 +2142,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>27</v>
+        <v>70</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>HAL, MAXHEALTH, TATATECH, TATAELXSI, ADANIENSOL, AUBANK, BAJFINANCE, BDL, BRITANNIA, CIPLA, COLPAL, CROMPTON, DABUR, DIVISLAB, DIXON, IDFCFIRSTB, JSWENERGY, JSWSTEEL, KFINTECH, MANKIND, PAYTM, PIDILITIND, PPLPHARMA, SAMMAANCAP, SBILIFE, TATAPOWER, UPL</t>
+          <t>ANANDRATHI, ASAHIINDIA, HAL, JMFINANCIL, KPIL, MAXHEALTH, TATATECH, ZFCVINDIA, CARBORUNIV, GMDCLTD, KIRLOSENG, TATAELXSI, AARTIIND, ABBOTINDIA, ADANIENSOL, APTUS, ATUL, AUBANK, BAJFINANCE, BDL, BRIGADE, BRITANNIA, CANFINHOME, CAPLIPOINT, CENTURYPLY, CHOICEIN, CIPLA, CLEAN, COLPAL, CRAFTSMAN, CROMPTON, DABUR, DIVISLAB, DIXON, EIHOTEL, ENGINERSIN, FORCEMOT, GLAXO, GVT&amp;D, HEG, HINDCOPPER, HSCL, HYUNDAI, IDFCFIRSTB, INDIACEM, JBMA, JSWENERGY, JSWSTEEL, JUBLINGREA, KAJARIACER, KFINTECH, MANKIND, MSUMI, NEWGEN, NIVABUPA, NSLNISP, PAYTM, PIDILITIND, PPLPHARMA, RPOWER, RRKABEL, SAMMAANCAP, SAREGAMA, SBFC, SBILIFE, SUMICHEM, TATAPOWER, TRIVENI, TTML, UPL</t>
         </is>
       </c>
     </row>
@@ -2167,7 +2167,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>30</v>
+        <v>83</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -2176,7 +2176,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>NMDC, POLYCAB, GAIL, NBCC, PIIND, SAIL, ULTRACEMCO, ADANIENT, APLAPOLLO, BAJAJFINSV, BAJFINANCE, BANKINDIA, BLUESTARCO, BOSCHLTD, BRITANNIA, DMART, HDFCAMC, HINDPETRO, INDIGO, JUBLFOOD, KALYANKJIL, LT, M&amp;M, MUTHOOTFIN, ONGC, PETRONET, POWERINDIA, TECHM, TRENT, YESBANK</t>
+          <t>LATENTVIEW, NIACL, NMDC, POLYCAB, RKFORGE, ASTRAZEN, BASF, ERIS, FINPIPE, GAIL, INDIAMART, LLOYDSME, MOTILALOFS, NBCC, PIIND, SAIL, SIGNATURE, ULTRACEMCO, 3MINDIA, ABSLAMC, ADANIENT, ADANIPOWER, AEGISLOG, AKUMS, ALOKINDS, APLAPOLLO, ARE&amp;M, BAJAJFINSV, BAJFINANCE, BANKINDIA, BAYERCROP, BIKAJI, BLUEJET, BLUESTARCO, BOSCHLTD, BRITANNIA, CAMPUS, CRAFTSMAN, DBREALTY, DMART, ELECON, FSL, GODIGIT, GRANULES, GRSE, GUJGASLTD, HDFCAMC, HINDPETRO, IGL, IKS, INDIGO, IRCON, JKCEMENT, JUBLFOOD, JYOTHYLAB, KALYANKJIL, LEMONTREE, LT, M&amp;M, MEDANTA, MUTHOOTFIN, NATCOPHARM, NEULANDLAB, ONGC, PETRONET, PFIZER, PGHH, POWERINDIA, RADICO, RITES, SARDAEN, SCHAEFFLER, SOBHA, SUNTV, TARIL, TATACHEM, TECHM, TEJASNET, TRENT, UTIAMC, VTL, YESBANK, ZENTEC</t>
         </is>
       </c>
     </row>
@@ -2192,16 +2192,16 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>44</v>
+        <v>98</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>BAJAJFINSV, BRITANNIA, CANBK, GAIL, MPHASIS, SOLARINDS, UNOMINDA, 360ONE, APLAPOLLO, APOLLOHOSP, BAJAJHLDNG, BANKBARODA, BHARTIARTL, BIOCON, CAMS, CDSL, CGPOWER, COALINDIA, COFORGE, COLPAL, CROMPTON, DLF, FEDERALBNK, GMRAIRPORT, HEROMOTOCO, HINDALCO, HINDPETRO, IDEA, IDFCFIRSTB, IOC, IRFC, ITC, JSWSTEEL, LODHA, NESTLEIND, OIL, PAYTM, PHOENIXLTD, SIEMENS, SUZLON, SWIGGY, TMPV, UNIONBANK, WIPRO</t>
+          <t>ESCORTS, TIMKEN, BAJAJFINSV, BRITANNIA, CANBK, FORCEMOT, GAIL, JBCHEPHARM, MPHASIS, NLCINDIA, POLYMED, PTCIL, SOLARINDS, TRITURBINE, UNOMINDA, 360ONE, AAVAS, ABLBL, AIIL, APLAPOLLO, APOLLOHOSP, APTUS, BAJAJHLDNG, BANKBARODA, BHARTIARTL, BIOCON, BLUEDART, BRIGADE, CAMS, CASTROLIND, CDSL, CENTRALBK, CGPOWER, CHOLAHLDNG, CLEAN, COALINDIA, COFORGE, COLPAL, COROMANDEL, CROMPTON, DATAPATTNS, DEEPAKNTR, DLF, ECLERX, FACT, FEDERALBNK, FINCABLES, FIRSTCRY, GLAND, GLAXO, GMDCLTD, GMRAIRPORT, HAPPSTMNDS, HEG, HEROMOTOCO, HEXT, HINDALCO, HINDPETRO, HSCL, IDBI, IDEA, IDFCFIRSTB, IOC, IPCALAB, IRFC, ITC, JBMA, JPPOWER, JSL, JSWSTEEL, KAJARIACER, LODHA, NAM-INDIA, NESTLEIND, NSLNISP, OIL, PAYTM, PHOENIXLTD, RAMCOCEM, REDINGTON, RPOWER, RRKABEL, SAPPHIRE, SARDAEN, SBFC, SHYAMMETL, SIEMENS, SOBHA, SUMICHEM, SUZLON, SWIGGY, TECHNOE, TMPV, UNIONBANK, USHAMART, WIPRO, ZEEL, ZENSARTECH</t>
         </is>
       </c>
     </row>
@@ -2217,7 +2217,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -2226,7 +2226,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>ADANIENT, TATAELXSI, AXISBANK, BAJAJFINSV, BRITANNIA, DMART, FEDERALBNK, FORTIS, KALYANKJIL, KFINTECH, PFC, SBICARD, SOLARINDS, TIINDIA, TRENT, UNIONBANK, VOLTAS</t>
+          <t>ADANIENT, DEVYANI, HBLENGINE, NATCOPHARM, POLYMED, TATAELXSI, ABSLAMC, ACMESOLAR, AEGISLOG, AGARWALEYE, ALOKINDS, AXISBANK, BAJAJFINSV, BAYERCROP, BLUEJET, BRITANNIA, CENTURYPLY, DMART, DOMS, ELECON, EMCURE, FEDERALBNK, FORTIS, GODIGIT, GRANULES, IGL, KALYANKJIL, KFINTECH, MRPL, PFC, SBICARD, SOLARINDS, SONATSOFTW, TATACHEM, TIINDIA, TRENT, UBL, UNIONBANK, VENTIVE, VOLTAS</t>
         </is>
       </c>
     </row>
@@ -2242,7 +2242,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -2251,7 +2251,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>ALKEM, INDUSTOWER, MCX, NBCC, ABB, ANGELONE, ASHOKLEY, AUROPHARMA, BHEL, DLF, GLENMARK, GRASIM, HDFCAMC, HINDZINC, IOC, IRFC, KAYNES, KPITTECH, MANAPPURAM, MARICO, MFSL, NTPC, NUVAMA, NYKAA, OIL, PNB, POWERINDIA, SIEMENS, SONACOMS, TCS, TECHM, TMPV</t>
+          <t>ALKEM, BALKRISIND, BASF, COCHINSHIP, HFCL, INDUSTOWER, JKTYRE, MCX, MINDACORP, MOTILALOFS, NBCC, NIACL, ABB, AEGISVOPAK, AKZOINDIA, ANGELONE, ASHOKLEY, AUROPHARMA, BHEL, DLF, FINCABLES, GLENMARK, GRASIM, HDFCAMC, HINDCOPPER, HINDZINC, INDIAMART, IOC, IRFC, KAYNES, KPITTECH, MANAPPURAM, MARICO, MFSL, MRF, NH, NTPC, NUVAMA, NUVOCO, NYKAA, OIL, PNB, POWERINDIA, RADICO, RCF, SCHNEIDER, SCI, SHYAMMETL, SIEMENS, SONACOMS, SUNDRMFAST, TCS, TECHM, TECHNOE, TMPV</t>
         </is>
       </c>
     </row>
@@ -2267,7 +2267,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -2276,7 +2276,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>EICHERMOT, 360ONE, AXISBANK, BHEL, BPCL, DIXON, ETERNAL, GLENMARK, HDFCBANK, HINDALCO, HUDCO, ICICIGI, INFY, MOTHERSON, PNB, RELIANCE, SUPREMEIND, TCS, TECHM, VEDL</t>
+          <t>EICHERMOT, ESCORTS, 360ONE, AAVAS, ABBOTINDIA, AKZOINDIA, APARINDS, AXISBANK, BHEL, BIKAJI, BPCL, CARBORUNIV, COCHINSHIP, DBREALTY, DIXON, ENRIN, ETERNAL, GICRE, GLENMARK, HDFCBANK, HINDALCO, HUDCO, ICICIGI, INFY, LALPATHLAB, MAHSCOOTER, MOTHERSON, PGHH, PNB, POONAWALLA, RELIANCE, RHIM, SAGILITY, SCI, SONATSOFTW, SUNTV, SUPREMEIND, SWANCORP, TCS, TECHM, UBL, VEDL, WOCKPHARMA, ZEEL</t>
         </is>
       </c>
     </row>
@@ -2292,16 +2292,16 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>21</v>
+        <v>53</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>ABCAPITAL, DABUR, EXIDEIND, HAL, HINDUNILVR, IOC, ITC, KEI, LTM, MAXHEALTH, MOTHERSON, NTPC, OIL, PAGEIND, PFC, PHOENIXLTD, SUNPHARMA, TATATECH, TIINDIA, UNOMINDA, UPL</t>
+          <t>AGARWALEYE, SAPPHIRE, AADHARHFC, ABCAPITAL, APARINDS, BAJAJHFL, BEML, CAPLIPOINT, CENTRALBK, CRAFTSMAN, CUB, DABUR, ELGIEQUIP, ENGINERSIN, EXIDEIND, FSL, HAL, HAPPSTMNDS, HFCL, HINDUNILVR, IIFL, IOC, IPCALAB, IRB, ITC, ITCHOTELS, JBCHEPHARM, JYOTHYLAB, KEI, LTM, MAPMYINDIA, MAXHEALTH, MOTHERSON, NAVINFLUOR, NCC, NIVABUPA, NTPC, OIL, ONESOURCE, PAGEIND, PFC, PHOENIXLTD, RAINBOW, REDINGTON, SUNPHARMA, TATATECH, TIINDIA, TRITURBINE, UNOMINDA, UPL, WELSPUNLIV, ZEEL, ZENSARTECH</t>
         </is>
       </c>
     </row>
@@ -2317,16 +2317,16 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>CIPLA, HCLTECH, KEI, LTM, MANAPPURAM, NMDC, NUVAMA, PATANJALI, POLYCAB</t>
+          <t>BIKAJI, ACC, AWL, BAJAJHFL, CHALET, CIPLA, ERIS, GILLETTE, HCLTECH, IIFL, INDGN, KEI, KIMS, KPRMILL, LTM, LTTS, MANAPPURAM, NMDC, NUVAMA, PATANJALI, POLYCAB, RKFORGE, SCHNEIDER, SOBHA, TATACOMM, VTL, WELSPUNLIV</t>
         </is>
       </c>
     </row>
@@ -2342,7 +2342,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>JIOFIN, AMBER, BIOCON, GRASIM, INFY, LICHSGFIN, MANKIND, MPHASIS, NATIONALUM, SUNPHARMA</t>
+          <t>BALRAMCHIN, CONCORDBIO, FACT, J&amp;KBANK, JIOFIN, STARHEALTH, ZENTEC, ADANIPOWER, AJANTPHARM, AKUMS, AMBER, ANANTRAJ, ARE&amp;M, ASTRAZEN, BIOCON, BSOFT, CYIENT, GRASIM, GRSE, INFY, JKCEMENT, JUBLPHARMA, JYOTHYLAB, LICHSGFIN, LTFOODS, MAHABANK, MANKIND, MOTILALOFS, MPHASIS, NATIONALUM, NUVOCO, PRAJIND, PTCIL, SIGNATURE, SUNPHARMA, THERMAX</t>
         </is>
       </c>
     </row>
@@ -2367,7 +2367,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>17</v>
+        <v>52</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -2376,7 +2376,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>LAURUSLABS, SHREECEM, AUROPHARMA, BANDHANBNK, BANKINDIA, BEL, CAMS, CANBK, CDSL, CONCOR, CUMMINSIND, DRREDDY, MAZDOCK, OFSS, PRESTIGE, SBILIFE, TIINDIA</t>
+          <t>INDGN, LAURUSLABS, MRPL, PFIZER, SHREECEM, AARTIIND, ABREL, ASAHIINDIA, AUROPHARMA, BANDHANBNK, BANKINDIA, BBTC, BEL, CAMS, CANBK, CAPLIPOINT, CDSL, CHALET, CONCOR, CUMMINSIND, DATAPATTNS, DRREDDY, EMCURE, ENGINERSIN, FLUOROCHEM, GODFRYPHLP, HEG, HSCL, IDBI, INDIACEM, IRB, JBMA, JINDALSAW, JPPOWER, JSL, JYOTICNC, KAJARIACER, KARURVYSYA, KIRLOSBROS, KIRLOSENG, LINDEINDIA, MANYAVAR, MAZDOCK, MMTC, MSUMI, NSLNISP, OFSS, PRESTIGE, SBILIFE, THELEELA, TIINDIA, VMM</t>
         </is>
       </c>
     </row>
@@ -2392,7 +2392,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>19</v>
+        <v>52</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>ANGELONE, SRF, AMBUJACEM, BANDHANBNK, BHARTIARTL, DELHIVERY, DRREDDY, HCLTECH, IEX, INDIANB, INDUSINDBK, LICHSGFIN, MARICO, NYKAA, OBEROIRLTY, PAGEIND, PRESTIGE, SBILIFE, TORNTPHARM</t>
+          <t>ANGELONE, SRF, ABFRL, ABREL, ADANIPOWER, AKUMS, AMBUJACEM, ANANTRAJ, APLLTD, BANDHANBNK, BHARTIARTL, BHARTIHEXA, CAMPUS, CEATLTD, CHENNPETRO, CLEAN, CUB, DELHIVERY, DRREDDY, FINPIPE, FLUOROCHEM, GODFRYPHLP, HBLENGINE, HCLTECH, HSCL, IEX, INDIANB, INDUSINDBK, JBMA, JINDALSAW, JUBLPHARMA, JYOTICNC, KAJARIACER, KARURVYSYA, KIRLOSBROS, LICHSGFIN, MANYAVAR, MARICO, MMTC, NCC, NYKAA, OBEROIRLTY, PAGEIND, PRESTIGE, SBILIFE, SUNDRMFAST, TATACHEM, THERMAX, TIMKEN, TORNTPHARM, VENTIVE, VMM</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2417,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>24</v>
+        <v>50</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>BHARATFORG, VOLTAS, ADANIGREEN, BANKINDIA, BSE, CANBK, DALBHARAT, DELHIVERY, DLF, GLENMARK, GODREJCP, HAVELLS, HDFCAMC, IREDA, LT, MAZDOCK, PERSISTENT, RECLTD, SAMMAANCAP, TATAPOWER, TATASTEEL, TMPV, TVSMOTOR, WAAREEENER</t>
+          <t>BHARATFORG, GESHIP, GODREJAGRO, INTELLECT, METROPOLIS, NETWEB, VOLTAS, ABFRL, ADANIGREEN, AFCONS, APLLTD, ARE&amp;M, BANKINDIA, BSE, CANBK, CESC, DALBHARAT, DCMSHRIRAM, DELHIVERY, DLF, EMAMILTD, EMCURE, GLENMARK, GODREJCP, HAVELLS, HDFCAMC, IREDA, LEMONTREE, LINDEINDIA, LT, MAZDOCK, MGL, NAVA, NH, PERSISTENT, RAILTEL, RCF, RECLTD, SAMMAANCAP, SHYAMMETL, SIGNATURE, SJVN, TATACHEM, TATAPOWER, TATASTEEL, TECHNOE, TMPV, TVSMOTOR, UCOBANK, WAAREEENER</t>
         </is>
       </c>
     </row>
@@ -2442,16 +2442,16 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>ASIANPAINT, CROMPTON, DIXON, DLF, EXIDEIND, GODREJCP, HAL, HAVELLS, IREDA, KFINTECH, MAXHEALTH, PGEL, PREMIERENE, RECLTD, SAMMAANCAP, SOLARINDS, TATAPOWER, TATASTEEL, TATATECH, TMPV, UNITDSPR, UPL</t>
+          <t>ACC, BERGEPAINT, AARTIIND, AIIL, ASIANPAINT, CANFINHOME, CCL, CROMPTON, DIXON, DLF, ENDURANCE, EXIDEIND, GLAXO, GODREJCP, GODREJIND, HAL, HAVELLS, HONASA, INOXINDIA, IREDA, JKTYRE, KFINTECH, MAXHEALTH, MGL, NAVA, PCBL, PGEL, PREMIERENE, PVRINOX, RAILTEL, RECLTD, SAMMAANCAP, SHYAMMETL, SJVN, SOLARINDS, TATAINVEST, TATAPOWER, TATASTEEL, TATATECH, TECHNOE, TMPV, UCOBANK, UNITDSPR, UPL</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>21</v>
+        <v>47</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>SBIN, HDFCLIFE, BAJFINANCE, BHARTIARTL, BPCL, COFORGE, GLENMARK, JSWENERGY, LT, NMDC, PAYTM, PERSISTENT, PFC, POLYCAB, SAIL, TCS, TVSMOTOR, ULTRACEMCO, WIPRO, YESBANK, ZYDUSLIFE</t>
+          <t>CGCL, COHANCE, HYUNDAI, NEWGEN, SBIN, HDFCLIFE, ITI, LINDEINDIA, AIAENG, BAJAJHFL, BAJFINANCE, BHARTIARTL, BPCL, CARBORUNIV, COFORGE, CRAFTSMAN, FINPIPE, GLENMARK, GRAVITA, HBLENGINE, HINDCOPPER, HONAUT, IFCI, IGL, IIFL, INDIAMART, IRCTC, JSWENERGY, LLOYDSME, LT, M&amp;MFIN, NMDC, PAYTM, PERSISTENT, PFC, POLYCAB, RKFORGE, SAIL, TCS, TRIDENT, TVSMOTOR, UBL, ULTRACEMCO, VTL, WIPRO, YESBANK, ZYDUSLIFE</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>ASHOKLEY, COLPAL, KPITTECH, NATIONALUM, TITAN, APOLLOHOSP, CIPLA, DABUR, HINDPETRO, INDIGO, KEI, LICI, LTM, LUPIN, SUNPHARMA, SUZLON, SYNGENE, WIPRO</t>
+          <t>ASHOKLEY, EIHOTEL, SCHNEIDER, WHIRLPOOL, COLPAL, KPITTECH, NATIONALUM, SYRMA, TITAN, AKZOINDIA, APOLLOHOSP, ATHERENERG, BAJAJHFL, BATAINDIA, BSOFT, CHOLAHLDNG, CIPLA, CYIENT, DABUR, GRSE, HINDPETRO, IKS, INDIGO, INOXINDIA, KEI, LICI, LTM, LUPIN, M&amp;MFIN, NIVABUPA, RADICO, SUNPHARMA, SUZLON, SYNGENE, TATACOMM, WIPRO, ZENTEC</t>
         </is>
       </c>
     </row>
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -2526,7 +2526,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>PATANJALI, SONACOMS, EICHERMOT, PIIND, POWERGRID, ABB, CAMS, CDSL, EXIDEIND, HINDZINC, IDEA, INDIGO, INDUSINDBK, INOXWIND, ITC, KFINTECH, LICHSGFIN, LUPIN, MFSL, SUZLON, TATACONSUM</t>
+          <t>NUVOCO, PATANJALI, SCHAEFFLER, SONACOMS, UTIAMC, VGUARD, EICHERMOT, GILLETTE, GLAXO, LINDEINDIA, PIIND, POWERGRID, THELEELA, ABB, ACC, CAMS, CAPLIPOINT, CDSL, CENTRALBK, CHOICEIN, CHOLAHLDNG, DATAPATTNS, EIDPARRY, EXIDEIND, GODFRYPHLP, GPIL, HAPPSTMNDS, HINDZINC, HONASA, IDBI, IDEA, IFCI, INDIGO, INDUSINDBK, INOXWIND, IPCALAB, ITC, JPPOWER, JSL, JSWINFRA, KFINTECH, LICHSGFIN, LUPIN, MFSL, MOTILALOFS, NEULANDLAB, SAPPHIRE, SARDAEN, SOBHA, SUZLON, TATACONSUM, VMM</t>
         </is>
       </c>
     </row>
@@ -2542,7 +2542,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>28</v>
+        <v>80</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>CGPOWER, HEROMOTOCO, LODHA, RELIANCE, SUPREMEIND, SWIGGY, MANKIND, ADANIENSOL, ADANIENT, ANGELONE, AUROPHARMA, BANKBARODA, BDL, BOSCHLTD, FORTIS, GMRAIRPORT, HAVELLS, INFY, IRFC, KALYANKJIL, LTF, MARICO, MFSL, NYKAA, ONGC, RVNL, SHRIRAMFIN, VEDL</t>
+          <t>CGPOWER, DEEPAKNTR, FIRSTCRY, GSPL, GUJGASLTD, HEROMOTOCO, LODHA, PGHH, RELIANCE, SUPREMEIND, SWIGGY, TIMKEN, MANKIND, NLCINDIA, PRAJIND, AADHARHFC, ABBOTINDIA, ABLBL, ACC, ACMESOLAR, ADANIENSOL, ADANIENT, ALKYLAMINE, ANGELONE, APOLLOTYRE, AUROPHARMA, BANKBARODA, BDL, BEML, BHARTIHEXA, BLUEDART, BOSCHLTD, CHAMBLFERT, CRISIL, DEVYANI, FIVESTAR, FORTIS, GESHIP, GLAND, GMRAIRPORT, GRANULES, HAVELLS, HONAUT, IGL, INDIAMART, INFY, IRFC, ITCHOTELS, ITI, JSWCEMENT, JWL, KALYANKJIL, KEC, KSB, LTF, MARICO, MFSL, NCC, NH, NTPCGREEN, NYKAA, OLECTRA, ONESOURCE, ONGC, POONAWALLA, RAILTEL, RHIM, RITES, RVNL, SBFC, SHRIRAMFIN, SOBHA, SUNDRMFAST, TARIL, TBOTEK, TITAGARH, TRIDENT, TTML, VEDL, WOCKPHARMA</t>
         </is>
       </c>
     </row>
@@ -2567,16 +2567,16 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>TATAELXSI, ASTRAL, BAJFINANCE, CROMPTON, DABUR, FORTIS, GMRAIRPORT, GODREJPROP, ICICIPRULI, JSWENERGY, LTF, M&amp;M, MANAPPURAM, MARUTI, ONGC, PAYTM, PNBHOUSING, SHRIRAMFIN, TIINDIA, VOLTAS</t>
+          <t>FORCEMOT, AEGISLOG, AFFLE, ENDURANCE, TATAELXSI, AADHARHFC, ACMESOLAR, ALKYLAMINE, ASTRAL, BAJFINANCE, BAYERCROP, BEML, BLUEDART, BRIGADE, CRISIL, CROMPTON, CUB, DABUR, DBREALTY, DEVYANI, EMAMILTD, EMCURE, FORTIS, GLAND, GMDCLTD, GMRAIRPORT, GODREJPROP, HINDCOPPER, ICICIPRULI, JKCEMENT, JMFINANCIL, JSWCEMENT, JSWENERGY, JWL, JYOTHYLAB, KEC, LTF, M&amp;M, MANAPPURAM, MARUTI, MEDANTA, NAVINFLUOR, NCC, NIVABUPA, OLECTRA, ONESOURCE, ONGC, PAYTM, PNBHOUSING, RPOWER, SAREGAMA, SHRIRAMFIN, SJVN, TARIL, TIINDIA, TITAGARH, TRIDENT, USHAMART, VOLTAS, WOCKPHARMA</t>
         </is>
       </c>
     </row>
@@ -2592,7 +2592,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -2601,7 +2601,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>NBCC, HAL, HDFCAMC, HINDALCO, MAXHEALTH, NESTLEIND, NUVAMA, PAGEIND, POLICYBZR, SBICARD, SOLARINDS, TATATECH, UPL</t>
+          <t>BASF, MOTILALOFS, NATCOPHARM, NBCC, NIACL, AJANTPHARM, AKZOINDIA, ANANDRATHI, ASAHIINDIA, BLUEJET, CENTURYPLY, CHALET, HAL, HDFCAMC, HINDALCO, JMFINANCIL, KIRLOSBROS, KPIL, MAXHEALTH, NAVA, NESTLEIND, NEWGEN, NUVAMA, PAGEIND, POLICYBZR, RAINBOW, RAMCOCEM, REDINGTON, SBICARD, SIGNATURE, SOLARINDS, TARIL, TATATECH, UPL, ZFCVINDIA</t>
         </is>
       </c>
     </row>
@@ -2617,16 +2617,16 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>ALKEM, GAIL, LAURUSLABS, SHREECEM, BAJAJHLDNG, BANDHANBNK, CGPOWER, HAVELLS, HCLTECH, ICICIGI, ICICIPRULI, INDUSTOWER, IREDA, LODHA, MPHASIS, MUTHOOTFIN, NMDC, ONGC, PAGEIND, PATANJALI, PETRONET, POLYCAB, SBILIFE, SOLARINDS, WIPRO, YESBANK</t>
+          <t>SWANCORP, ALKEM, CCL, ESCORTS, GAIL, INDGN, LAURUSLABS, SHREECEM, AADHARHFC, ADANIPOWER, AFCONS, AKUMS, ARE&amp;M, BAJAJHLDNG, BALKRISIND, BANDHANBNK, BATAINDIA, CGPOWER, COCHINSHIP, CRAFTSMAN, DOMS, ERIS, FINPIPE, GRAPHITE, HAPPSTMNDS, HAVELLS, HCLTECH, ICICIGI, ICICIPRULI, INDUSTOWER, IREDA, JKTYRE, JUBLPHARMA, JYOTHYLAB, LATENTVIEW, LEMONTREE, LODHA, LTTS, MINDACORP, MPHASIS, MSUMI, MUTHOOTFIN, NMDC, OLECTRA, ONGC, PAGEIND, PATANJALI, PETRONET, POLYCAB, RKFORGE, SBILIFE, SOLARINDS, TIMKEN, UTIAMC, VTL, WIPRO, YESBANK</t>
         </is>
       </c>
     </row>
@@ -2642,7 +2642,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -2651,7 +2651,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>SRF, AMBUJACEM, APLAPOLLO, CROMPTON, FORTIS, GAIL, HEROMOTOCO, ICICIGI, INDHOTEL, JINDALSTEL, KPITTECH, LICHSGFIN, MOTHERSON, NATIONALUM, SHRIRAMFIN, SIEMENS, SYNGENE, TIINDIA</t>
+          <t>FIRSTCRY, MRPL, SRF, AAVAS, AEGISVOPAK, AMBUJACEM, APLAPOLLO, BLUEDART, CARBORUNIV, CASTROLIND, CGCL, CHOLAHLDNG, COHANCE, CROMPTON, DEEPAKNTR, ENRIN, FORTIS, GAIL, GLAND, GODREJIND, GRAVITA, HEROMOTOCO, ICICIGI, IGIL, INDHOTEL, JINDALSTEL, JWL, KPITTECH, LICHSGFIN, MAHABANK, MOTHERSON, NATIONALUM, NTPCGREEN, PTCIL, RAILTEL, SAGILITY, SHRIRAMFIN, SIEMENS, SONATSOFTW, SYNGENE, SYRMA, TIINDIA, TIMKEN, VGUARD, WOCKPHARMA</t>
         </is>
       </c>
     </row>
@@ -2667,16 +2667,16 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>CGPOWER, POWERINDIA, AUBANK, AXISBANK, BEL, CAMS, CANBK, CDSL, COLPAL, DALBHARAT, FEDERALBNK, HINDALCO, HINDUNILVR, IDFCFIRSTB, ITC, JSWSTEEL, MAZDOCK, OFSS, RVNL, SWIGGY, UNIONBANK, WAAREEENER</t>
+          <t>GODREJAGRO, APTUS, CGPOWER, NETWEB, POWERINDIA, SAPPHIRE, SBFC, ABFRL, AFCONS, AUBANK, AXISBANK, BEL, BRIGADE, CAMS, CANBK, CDSL, CENTRALBK, CHALET, CHOICEIN, CLEAN, COLPAL, DALBHARAT, DATAPATTNS, DCMSHRIRAM, DEVYANI, ECLERX, FEDERALBNK, FLUOROCHEM, GLAND, GLAXO, GVT&amp;D, HEG, HINDALCO, HINDUNILVR, HOMEFIRST, HSCL, IDBI, IDFCFIRSTB, IPCALAB, ITC, JBMA, JPPOWER, JSL, JSWSTEEL, KAJARIACER, MAZDOCK, MRF, NSLNISP, OFSS, RADICO, RCF, RPOWER, RRKABEL, RVNL, SUMICHEM, SWIGGY, UNIONBANK, UTIAMC, WAAREEENER, WELCORP</t>
         </is>
       </c>
     </row>
@@ -2692,7 +2692,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -2701,7 +2701,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>ABB, BHARATFORG, BSE, DELHIVERY, DMART, HUDCO, INDUSINDBK, IOC, KALYANKJIL, OIL, TECHM, TRENT, VOLTAS</t>
+          <t>ABB, ELECON, METROPOLIS, ABSLAMC, ALOKINDS, BHARATFORG, BLUEJET, BSE, BSOFT, DELHIVERY, DEVYANI, DMART, GODIGIT, GRANULES, HFCL, HUDCO, IGL, INDGN, INDUSINDBK, IOC, JKTYRE, KALYANKJIL, OIL, OLECTRA, SONATSOFTW, TATACHEM, TECHM, TEJASNET, TRENT, VOLTAS</t>
         </is>
       </c>
     </row>
@@ -2717,7 +2717,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -2726,7 +2726,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>JIOFIN, TVSMOTOR, ADANIENSOL, BDL, CHOLAFIN, MARUTI, MOTHERSON, PAYTM, PGEL, POWERGRID, SBICARD, SBIN, TATACONSUM, TITAN</t>
+          <t>CONCORDBIO, J&amp;KBANK, JIOFIN, TVSMOTOR, ADANIENSOL, AGARWALEYE, APARINDS, APOLLOTYRE, BALRAMCHIN, BDL, BERGEPAINT, CAPLIPOINT, CHOLAFIN, FSL, GICRE, GRSE, HOMEFIRST, KPRMILL, LALPATHLAB, MARUTI, MOTHERSON, PAYTM, PGEL, POWERGRID, RADICO, SBICARD, SBIN, STARHEALTH, TATACONSUM, TITAN, ZEEL, ZENTEC</t>
         </is>
       </c>
     </row>
@@ -2742,7 +2742,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>AUROPHARMA, BHEL, ZYDUSLIFE, ADANIGREEN, BANKBARODA, BHARTIARTL, BRITANNIA, BSE, COFORGE, DLF, GLENMARK, HAL, HCLTECH, INDHOTEL, IRFC, KFINTECH, MAXHEALTH, MAZDOCK, MCX, NBCC, NUVAMA, PERSISTENT, PNB, TATATECH, TCS, TMPV</t>
+          <t>AUROPHARMA, BHEL, NAM-INDIA, ZENTEC, ZYDUSLIFE, AARTIIND, ADANIGREEN, AEGISVOPAK, AKZOINDIA, BANKBARODA, BHARTIARTL, BRITANNIA, BSE, COFORGE, COROMANDEL, DLF, EIDPARRY, ELGIEQUIP, FINCABLES, GLENMARK, GODREJIND, GRSE, HAL, HCLTECH, INDHOTEL, IRFC, KFINTECH, LTFOODS, MAXHEALTH, MAZDOCK, MCX, NBCC, NTPCGREEN, NUVAMA, PERSISTENT, PNB, SCI, SHYAMMETL, STARHEALTH, SWANCORP, TATATECH, TCS, TECHNOE, TMPV</t>
         </is>
       </c>
     </row>
@@ -2767,7 +2767,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>50</v>
+        <v>88</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -2776,7 +2776,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>BAJFINANCE, BANKINDIA, EXIDEIND, ICICIPRULI, KPITTECH, PNB, SAMMAANCAP, ADANIENSOL, APLAPOLLO, APOLLOHOSP, BAJAJHLDNG, BANDHANBNK, BHARATFORG, BLUESTARCO, BPCL, BRITANNIA, CANBK, CONCOR, CROMPTON, HDFCBANK, HINDALCO, IDEA, IDFCFIRSTB, INDHOTEL, INDUSTOWER, JINDALSTEL, JSWSTEEL, LAURUSLABS, LICHSGFIN, LICI, LODHA, LT, MAXHEALTH, NATIONALUM, NESTLEIND, NHPC, NTPC, OIL, PFC, PIIND, POWERGRID, PPLPHARMA, RECLTD, SAIL, SHRIRAMFIN, SOLARINDS, TATASTEEL, TATATECH, UNIONBANK, UNOMINDA</t>
+          <t>BAJFINANCE, BANKINDIA, EXIDEIND, ICICIPRULI, JSL, KPITTECH, PNB, SAMMAANCAP, SONATSOFTW, SUNDARMFIN, ABBOTINDIA, ADANIENSOL, APLAPOLLO, APOLLOHOSP, BAJAJHLDNG, BANDHANBNK, BHARATFORG, BLUEJET, BLUESTARCO, BPCL, BRITANNIA, CANBK, CENTRALBK, CHALET, CHAMBLFERT, CONCOR, CRAFTSMAN, CROMPTON, DOMS, ECLERX, EIHOTEL, GMDCLTD, GRAPHITE, HDFCBANK, HEG, HINDALCO, IDBI, IDEA, IDFCFIRSTB, IIFL, INDHOTEL, INDIACEM, INDUSTOWER, IRB, JINDALSTEL, JSWSTEEL, JUBLPHARMA, KIRLOSBROS, LAURUSLABS, LICHSGFIN, LICI, LODHA, LT, MAHABANK, MANYAVAR, MAPMYINDIA, MAXHEALTH, NATIONALUM, NESTLEIND, NHPC, NSLNISP, NTPC, OIL, OLECTRA, ONESOURCE, PFC, PIIND, POLYMED, POONAWALLA, POWERGRID, PPLPHARMA, PRAJIND, RECLTD, SAIL, SAPPHIRE, SBFC, SCHNEIDER, SHRIRAMFIN, SOLARINDS, SYRMA, TATASTEEL, TATATECH, UNIONBANK, UNOMINDA, VENTIVE, VIJAYA, WELCORP, WHIRLPOOL</t>
         </is>
       </c>
     </row>
@@ -2792,7 +2792,7 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>ADANIENT, CHOLAFIN, APOLLOHOSP, AUBANK, BAJAJFINSV, BAJAJHLDNG, FEDERALBNK, HDFCBANK, IEX, INFY, JSWSTEEL, KPITTECH, LICI, LODHA, OBEROIRLTY, PFC, POWERGRID, PPLPHARMA, SOLARINDS, TATATECH, UNITDSPR, UNOMINDA, VOLTAS</t>
+          <t>ADANIENT, CHOLAFIN, JSWCEMENT, ABLBL, APOLLOHOSP, APOLLOTYRE, AUBANK, BAJAJFINSV, BAJAJHLDNG, BATAINDIA, BLUEDART, BLUEJET, BRIGADE, CAMPUS, CENTRALBK, FEDERALBNK, GSPL, HDFCBANK, IEX, INFY, IRB, JKCEMENT, JSWSTEEL, KPITTECH, KSB, LEMONTREE, LICI, LODHA, OBEROIRLTY, PFC, POONAWALLA, POWERGRID, PPLPHARMA, RAINBOW, SAGILITY, SBFC, SCHAEFFLER, SOLARINDS, SYRMA, TATACOMM, TATATECH, TBOTEK, TEJASNET, UBL, UNITDSPR, UNOMINDA, VOLTAS</t>
         </is>
       </c>
     </row>
@@ -2817,7 +2817,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -2826,7 +2826,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>MOTHERSON, AMBUJACEM, GLENMARK, FORTIS, GAIL, HAL, HCLTECH, IREDA, JIOFIN, KALYANKJIL, KAYNES, MAXHEALTH, PGEL, POLICYBZR, POLYCAB, SYNGENE, TATAPOWER, TORNTPOWER</t>
+          <t>JINDALSAW, LATENTVIEW, MOTHERSON, AARTIIND, ALOKINDS, AMBUJACEM, CENTURYPLY, GLENMARK, JKTYRE, UCOBANK, USHAMART, ADANIPOWER, AEGISVOPAK, AGARWALEYE, ANANTRAJ, BAJAJHFL, BSOFT, DBREALTY, ELECON, FORTIS, GAIL, HAL, HCLTECH, HEXT, IGL, IREDA, JIOFIN, JMFINANCIL, JWL, KALYANKJIL, KAYNES, LTFOODS, LTTS, MAHSEAMLES, MAXHEALTH, MINDACORP, MOTILALOFS, NATCOPHARM, NCC, NETWEB, PGEL, POLICYBZR, POLYCAB, SAILIFE, SAREGAMA, SJVN, SYNGENE, TATAPOWER, TEJASNET, TORNTPOWER, VTL, WELSPUNLIV, ZFCVINDIA</t>
         </is>
       </c>
     </row>
@@ -2842,7 +2842,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -2851,7 +2851,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>KEI, TATAELXSI, ADANIENT, BDL, BRITANNIA, CGPOWER, KFINTECH, LT, PAGEIND, SUZLON, TIINDIA, TVSMOTOR</t>
+          <t>CASTROLIND, KEC, KEI, NAM-INDIA, SIGNATURE, TATAELXSI, AAVAS, ADANIENT, AKUMS, BALRAMCHIN, BDL, BRITANNIA, CGPOWER, CHOLAHLDNG, EIHOTEL, FINCABLES, GRANULES, GVT&amp;D, KFINTECH, KIRLOSENG, LLOYDSME, LT, NCC, PAGEIND, PRAJIND, RRKABEL, SAGILITY, SJVN, SUZLON, TIINDIA, TVSMOTOR, ZFCVINDIA</t>
         </is>
       </c>
     </row>
@@ -2867,16 +2867,16 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>CHOLAFIN, FEDERALBNK, PHOENIXLTD, UNITDSPR, VOLTAS, BHARTIARTL, CAMS, GODREJCP, GODREJPROP, HAVELLS, HUDCO, INDIGO, INOXWIND, M&amp;M, MAZDOCK, OBEROIRLTY, PREMIERENE, PRESTIGE, RELIANCE, SOLARINDS, SONACOMS, ULTRACEMCO</t>
+          <t>M&amp;MFIN, CHOLAFIN, FEDERALBNK, PHOENIXLTD, UNITDSPR, VOLTAS, 3MINDIA, ACE, ACMESOLAR, AGARWALEYE, ASTERDM, BHARTIARTL, CAMS, CENTRALBK, ECLERX, GODREJCP, GODREJPROP, HAVELLS, HEXT, HUDCO, INDIGO, INOXWIND, JSWINFRA, KIRLOSENG, KSB, LEMONTREE, LTTS, M&amp;M, MAZDOCK, MEDANTA, NATCOPHARM, NLCINDIA, OBEROIRLTY, OLECTRA, PREMIERENE, PRESTIGE, PTCIL, RELIANCE, RPOWER, SOLARINDS, SONACOMS, ULTRACEMCO</t>
         </is>
       </c>
     </row>
@@ -2892,16 +2892,16 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>24</v>
+        <v>66</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>AMBUJACEM, AUROPHARMA, DIVISLAB, GLENMARK, HDFCAMC, LUPIN, MOTHERSON, SYNGENE, TRENT, ADANIENSOL, BIOCON, GAIL, GMRAIRPORT, ICICIGI, IREDA, JINDALSTEL, PAYTM, PERSISTENT, PHOENIXLTD, PIIND, PNB, POLYCAB, RELIANCE, SIEMENS</t>
+          <t>IRCTC, RAMCOCEM, AKUMS, AMBUJACEM, AUROPHARMA, BRIGADE, CENTURYPLY, COCHINSHIP, DIVISLAB, GLENMARK, GRANULES, HDFCAMC, IFCI, JINDALSAW, KARURVYSYA, LATENTVIEW, LUPIN, MGL, MOTHERSON, NEWGEN, NUVOCO, SAILIFE, SARDAEN, SYNGENE, TRENT, VMM, VTL, ZENTEC, AARTIIND, ABFRL, ABREL, ADANIENSOL, ALOKINDS, BBTC, BIOCON, EIDPARRY, GAIL, GMRAIRPORT, ICICIGI, IIFL, IKS, IREDA, ITCHOTELS, JINDALSTEL, JKTYRE, JUBLINGREA, JWL, JYOTICNC, KPIL, MAHSEAMLES, NAVA, NIACL, PAYTM, PERSISTENT, PHOENIXLTD, PIIND, PNB, POLYCAB, RELIANCE, SCI, SIEMENS, SOBHA, TARIL, TITAGARH, TTML, USHAMART</t>
         </is>
       </c>
     </row>
@@ -2917,16 +2917,16 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>ABCAPITAL, ASHOKLEY, GLENMARK, HAVELLS, HINDUNILVR, KFINTECH, KPITTECH, MUTHOOTFIN, POLYCAB, SWIGGY, WAAREEENER</t>
+          <t>ACMESOLAR, GODFRYPHLP, TTML, ABCAPITAL, ALOKINDS, ASHOKLEY, BATAINDIA, BAYERCROP, GLENMARK, HAVELLS, HINDUNILVR, JSWINFRA, KFINTECH, KPITTECH, LLOYDSME, LTFOODS, MAHSCOOTER, MOTILALOFS, MUTHOOTFIN, NATCOPHARM, NAVA, POLYCAB, SWIGGY, THELEELA, USHAMART, WAAREEENER, WELCORP</t>
         </is>
       </c>
     </row>
@@ -2942,7 +2942,7 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -2951,7 +2951,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>SONACOMS, TRENT, ULTRACEMCO, APLAPOLLO, BDL, CAMS, EICHERMOT, INDIGO, INOXWIND, M&amp;M, MANAPPURAM, MAZDOCK, MUTHOOTFIN, PAYTM, PNBHOUSING, SOLARINDS</t>
+          <t>GODFRYPHLP, IRCON, MRF, RAILTEL, RAINBOW, SONACOMS, TRENT, ULTRACEMCO, ABBOTINDIA, ABFRL, APLAPOLLO, ASTERDM, BDL, BEML, CAMS, CAPLIPOINT, CASTROLIND, EICHERMOT, EIDPARRY, GLAXO, GRANULES, GRAPHITE, IGL, INDIGO, INOXINDIA, INOXWIND, IRB, JUBLINGREA, KIRLOSBROS, M&amp;M, MANAPPURAM, MAZDOCK, MEDANTA, MUTHOOTFIN, NETWEB, NUVOCO, OLECTRA, PAYTM, PNBHOUSING, RITES, RPOWER, SAREGAMA, SOBHA, SOLARINDS, TIMKEN, TRITURBINE</t>
         </is>
       </c>
     </row>
@@ -2967,16 +2967,16 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>CUMMINSIND, MCX, SRF, DABUR, SIEMENS, ZYDUSLIFE, BAJAJFINSV, HINDUNILVR, HINDZINC, KFINTECH, MANAPPURAM, MFSL, PNBHOUSING, POWERINDIA, RVNL, TATACONSUM, VBL</t>
+          <t>APTUS, CUMMINSIND, MCX, SRF, AWL, BHARTIHEXA, DABUR, ENDURANCE, ENGINERSIN, PFIZER, SIEMENS, STARHEALTH, ZYDUSLIFE, BAJAJFINSV, BEML, CEATLTD, CLEAN, CYIENT, EIDPARRY, ELGIEQUIP, ENRIN, FINPIPE, GRAVITA, HBLENGINE, HINDCOPPER, HINDUNILVR, HINDZINC, HONASA, INDIAMART, IRCON, KFINTECH, MANAPPURAM, MFSL, NEULANDLAB, NLCINDIA, NTPCGREEN, PNBHOUSING, POWERINDIA, PVRINOX, RAILTEL, REDINGTON, RITES, RVNL, TATACONSUM, THELEELA, VBL</t>
         </is>
       </c>
     </row>
@@ -2992,7 +2992,7 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>19</v>
+        <v>71</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
@@ -3001,7 +3001,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>IRFC, VEDL, ADANIPORTS, ANGELONE, BAJAJHLDNG, DALBHARAT, EICHERMOT, ICICIPRULI, IEX, KAYNES, MARICO, MCX, MFSL, NBCC, PRESTIGE, RVNL, SWIGGY, TORNTPHARM, YESBANK</t>
+          <t>AEGISLOG, CRISIL, EMAMILTD, EMCURE, IPCALAB, IRFC, J&amp;KBANK, JPPOWER, TRIDENT, VEDL, VGUARD, ABREL, ABSLAMC, ACC, ADANIPORTS, AFFLE, ANGELONE, APARINDS, ASAHIINDIA, ASTRAZEN, ATUL, BAJAJHLDNG, BAYERCROP, BERGEPAINT, BHARTIHEXA, BRIGADE, CUB, DALBHARAT, DCMSHRIRAM, DEEPAKNTR, EICHERMOT, ERIS, FORCEMOT, GICRE, GLAXO, GRAVITA, HBLENGINE, ICICIPRULI, IEX, JBMA, JYOTHYLAB, KAYNES, MAHSCOOTER, MARICO, MCX, MFSL, MGL, MMTC, NBCC, NEWGEN, PGHH, PRESTIGE, RADICO, RHIM, RVNL, SIGNATURE, SUMICHEM, SUNTV, SWIGGY, TARIL, TATACOMM, TBOTEK, TITAGARH, TORNTPHARM, TRITURBINE, TRIVENI, UTIAMC, WELCORP, YESBANK, ZEEL, ZENTEC</t>
         </is>
       </c>
     </row>
@@ -3017,7 +3017,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>34</v>
+        <v>75</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
@@ -3026,7 +3026,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>HINDALCO, PETRONET, 360ONE, ALKEM, AMBER, APLAPOLLO, ASHOKLEY, ASTRAL, AUBANK, BAJAJ-AUTO, BHARTIARTL, BOSCHLTD, BPCL, BSE, CDSL, CIPLA, COLPAL, DALBHARAT, DIXON, DMART, ETERNAL, EXIDEIND, HDFCLIFE, HINDZINC, JINDALSTEL, LAURUSLABS, LTF, MARUTI, MFSL, NESTLEIND, NMDC, POLICYBZR, RBLBANK, SHREECEM</t>
+          <t>HINDALCO, INTELLECT, PETRONET, SUNDARMFIN, VENTIVE, 360ONE, 3MINDIA, AAVAS, AIAENG, ALKEM, AMBER, APLAPOLLO, APLLTD, ARE&amp;M, ASHOKLEY, ASTRAL, AUBANK, BAJAJ-AUTO, BHARTIARTL, BOSCHLTD, BPCL, BSE, CDSL, CERA, CGCL, CIPLA, CLEAN, COLPAL, COROMANDEL, CRAFTSMAN, CREDITACC, DALBHARAT, DIXON, DMART, EMCURE, ENDURANCE, ETERNAL, EXIDEIND, FIVESTAR, GESHIP, GODREJAGRO, GODREJIND, HAPPSTMNDS, HDFCLIFE, HINDZINC, HOMEFIRST, IIFL, IPCALAB, JINDALSTEL, KIMS, KPRMILL, LAURUSLABS, LTF, M&amp;MFIN, MAHABANK, MARUTI, METROPOLIS, MFSL, MINDACORP, MRPL, NESTLEIND, NH, NMDC, PCBL, PFIZER, POLICYBZR, RADICO, RBLBANK, SHREECEM, SUMICHEM, SWANCORP, TATAINVEST, TECHNOE, TIMKEN, ZENSARTECH</t>
         </is>
       </c>
     </row>
@@ -3042,16 +3042,16 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>ADANIGREEN, IDEA, BAJAJ-AUTO, CONCOR, CROMPTON, GLENMARK, GRASIM, INDUSTOWER, IOC, NATIONALUM, NBCC, NHPC, POLYCAB, SHRIRAMFIN, TATACONSUM, TCS, TMPV, UNITDSPR, VEDL, VOLTAS</t>
+          <t>EIHOTEL, ADANIGREEN, CAPLIPOINT, DEVYANI, FORCEMOT, GICRE, GUJGASLTD, IDEA, UTIAMC, ANANDRATHI, ATUL, BAJAJ-AUTO, BATAINDIA, CHOICEIN, CHOLAHLDNG, CONCOR, CROMPTON, DCMSHRIRAM, ERIS, FACT, GLENMARK, GRAPHITE, GRASIM, IFCI, INDGN, INDUSTOWER, IOC, J&amp;KBANK, JPPOWER, KPIL, LEMONTREE, LLOYDSME, MANYAVAR, MMTC, MSUMI, NATIONALUM, NBCC, NHPC, NSLNISP, ONESOURCE, POLYCAB, POLYMED, PVRINOX, SAPPHIRE, SHRIRAMFIN, SUNTV, TARIL, TATACONSUM, TCS, TMPV, TRIVENI, UNITDSPR, VEDL, VOLTAS, WHIRLPOOL</t>
         </is>
       </c>
     </row>
@@ -3067,7 +3067,7 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>AXISBANK, BANKBARODA, PETRONET, SAIL, 360ONE, ADANIPORTS, BLUESTARCO, COFORGE, DIXON, ETERNAL, HCLTECH, HEROMOTOCO, HINDALCO, ICICIBANK, INDUSINDBK, PIIND, SBILIFE, SYNGENE, TITAN</t>
+          <t>AXISBANK, BANKBARODA, JSWCEMENT, KAJARIACER, NIVABUPA, PETRONET, SAIL, 360ONE, AADHARHFC, ADANIPORTS, AIIL, APARINDS, BALRAMCHIN, BEML, BLUESTARCO, CHENNPETRO, COFORGE, DIXON, ETERNAL, FLUOROCHEM, GODREJIND, HCLTECH, HEROMOTOCO, HINDALCO, ICICIBANK, INDUSINDBK, ITCHOTELS, JYOTHYLAB, LINDEINDIA, NAM-INDIA, NAVA, PIIND, SAILIFE, SBILIFE, SWANCORP, SYNGENE, TATACHEM, TATAINVEST, TITAN, VENTIVE, VTL, ZEEL</t>
         </is>
       </c>
     </row>
@@ -3092,7 +3092,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -3101,7 +3101,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>INDIANB, ABB, ASTRAL, BLUESTARCO, CONCOR, CROMPTON, HDFCBANK, HDFCLIFE, KFINTECH, LT, LTF, NHPC, RBLBANK, TCS, TECHM, TMPV, UPL</t>
+          <t>BLS, FIVESTAR, INDIANB, ABB, ANANDRATHI, ASTRAL, BLUESTARCO, CASTROLIND, CHAMBLFERT, CHOICEIN, COCHINSHIP, COHANCE, CONCOR, CROMPTON, GESHIP, GMDCLTD, GPIL, HDFCBANK, HDFCLIFE, KFINTECH, LT, LTF, MSUMI, NAVA, NAVINFLUOR, NETWEB, NHPC, NSLNISP, PRAJIND, RADICO, RBLBANK, SAPPHIRE, SCHNEIDER, SHYAMMETL, TCS, TECHM, TMPV, UPL</t>
         </is>
       </c>
     </row>
@@ -3117,7 +3117,7 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
@@ -3126,7 +3126,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>SAMMAANCAP, EXIDEIND, KPITTECH, UNITDSPR, VOLTAS, COALINDIA, COFORGE, HCLTECH, JSWSTEEL, JUBLFOOD, ONGC, SBICARD</t>
+          <t>SAMMAANCAP, AKZOINDIA, EXIDEIND, KPITTECH, SONATSOFTW, UNITDSPR, VOLTAS, AIIL, ALKYLAMINE, BASF, CAMPUS, CESC, CHENNPETRO, COALINDIA, COFORGE, FINPIPE, FLUOROCHEM, HCLTECH, JSWSTEEL, JUBLFOOD, LEMONTREE, ONGC, PTCIL, SBICARD, VIJAYA</t>
         </is>
       </c>
     </row>
@@ -3142,7 +3142,7 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>19</v>
+        <v>46</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
@@ -3151,7 +3151,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>AUROPHARMA, DIVISLAB, HDFCAMC, LUPIN, SYNGENE, ADANIGREEN, BIOCON, COALINDIA, CUMMINSIND, DELHIVERY, EICHERMOT, GODREJPROP, IRFC, KEI, MAZDOCK, PPLPHARMA, TATAELXSI, TORNTPOWER, UPL</t>
+          <t>AUROPHARMA, DIVISLAB, HDFCAMC, ITI, LUPIN, SAILIFE, SYNGENE, VMM, VTL, ABLBL, ADANIGREEN, BAYERCROP, BBTC, BEML, BIOCON, BSOFT, CAPLIPOINT, CARBORUNIV, CHALET, CHAMBLFERT, COALINDIA, CUMMINSIND, DEEPAKNTR, DELHIVERY, EICHERMOT, FIRSTCRY, FSL, GILLETTE, GODREJPROP, GPIL, IFCI, IRFC, JBMA, JYOTICNC, KEI, MAZDOCK, MRPL, NAM-INDIA, POONAWALLA, PPLPHARMA, SAREGAMA, TARIL, TATAELXSI, TORNTPOWER, UPL, VIJAYA</t>
         </is>
       </c>
     </row>
@@ -3167,7 +3167,7 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
@@ -3176,7 +3176,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>ITC, BANDHANBNK, ABB, AXISBANK, BANKINDIA, INDHOTEL, IOC, LICHSGFIN, LT, MAXHEALTH, PIDILITIND, PNB, TVSMOTOR, UNIONBANK</t>
+          <t>ITC, BANDHANBNK, MAPMYINDIA, ABB, AJANTPHARM, APOLLOTYRE, ATGL, AXISBANK, BANKINDIA, COROMANDEL, FINCABLES, GVT&amp;D, HAPPSTMNDS, HBLENGINE, HOMEFIRST, INDHOTEL, IOC, ITI, JINDALSAW, JUBLPHARMA, KEC, KIMS, LALPATHLAB, LICHSGFIN, LT, M&amp;MFIN, MAXHEALTH, PFIZER, PIDILITIND, PNB, RRKABEL, SAGILITY, SCI, SUMICHEM, TIMKEN, TVSMOTOR, UBL, UNIONBANK</t>
         </is>
       </c>
     </row>
@@ -3192,7 +3192,7 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
@@ -3201,7 +3201,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>AUBANK, MFSL, OFSS</t>
+          <t>AUBANK, CAMPUS, CCL, CLEAN, ENDURANCE, ENGINERSIN, GICRE, GSPL, INDIACEM, INDIAMART, KAJARIACER, MFSL, NATCOPHARM, OFSS, PVRINOX, SCHAEFFLER, UTIAMC</t>
         </is>
       </c>
     </row>
@@ -3217,7 +3217,7 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>37</v>
+        <v>81</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
@@ -3226,7 +3226,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>CHOLAFIN, FEDERALBNK, JIOFIN, PGEL, UNOMINDA, APOLLOHOSP, ASTRAL, BAJAJHLDNG, BLUESTARCO, CONCOR, CUMMINSIND, GAIL, HAL, HDFCBANK, HDFCLIFE, INDIGO, IREDA, JSWSTEEL, KALYANKJIL, KAYNES, LICI, LODHA, NHPC, PATANJALI, PFC, PIDILITIND, PIIND, POWERGRID, PPLPHARMA, RECLTD, RVNL, SAIL, SOLARINDS, SONACOMS, TATATECH, ULTRACEMCO, VBL</t>
+          <t>CHOLAFIN, FEDERALBNK, JIOFIN, LTFOODS, PGEL, UNOMINDA, ADANIPOWER, AEGISLOG, AEGISVOPAK, AGARWALEYE, ANANTRAJ, APOLLOHOSP, ASTRAL, BAJAJHFL, BAJAJHLDNG, BATAINDIA, BLS, BLUEDART, BLUEJET, BLUESTARCO, CENTRALBK, CONCOR, CRISIL, CUB, CUMMINSIND, DATAPATTNS, DBREALTY, ELECON, FIVESTAR, GAIL, GILLETTE, GRAVITA, HAL, HDFCBANK, HDFCLIFE, IGL, IKS, INDGN, INDIGO, IRB, IREDA, ITCHOTELS, J&amp;KBANK, JKCEMENT, JMFINANCIL, JPPOWER, JSWSTEEL, KALYANKJIL, KAYNES, KSB, LICI, LLOYDSME, LODHA, MAHSEAMLES, MOTILALOFS, NHPC, NSLNISP, PATANJALI, PFC, PIDILITIND, PIIND, POONAWALLA, POWERGRID, PPLPHARMA, RECLTD, RPOWER, RVNL, SAIL, SAPPHIRE, SAREGAMA, SBFC, SOLARINDS, SONACOMS, SYRMA, TATATECH, TRIVENI, UCOBANK, ULTRACEMCO, VBL, VENTIVE, WELSPUNLIV</t>
         </is>
       </c>
     </row>
@@ -3242,16 +3242,16 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>AMBUJACEM, GLENMARK, MOTHERSON, ADANIPORTS, DIXON, ETERNAL, HINDALCO, ICICIBANK, MARUTI, MCX, POLYCAB, SIEMENS</t>
+          <t>BALKRISIND, HSCL, AMBUJACEM, CENTURYPLY, GLENMARK, JINDALSAW, JWL, MOTHERSON, AARTIIND, ADANIPORTS, ALOKINDS, APARINDS, DIXON, EIHOTEL, ETERNAL, HEXT, HFCL, HINDALCO, HONAUT, ICICIBANK, IFCI, IGIL, INTELLECT, IOB, JKTYRE, JYOTHYLAB, KPIL, MARUTI, MCX, NATCOPHARM, NETWEB, NH, PFIZER, POLYCAB, SIEMENS, SWANCORP, TATACHEM, TATAINVEST, TEJASNET, USHAMART, ZEEL</t>
         </is>
       </c>
     </row>
@@ -3267,7 +3267,7 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -3276,7 +3276,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>HAVELLS, APLAPOLLO, BPCL, COALINDIA, HINDUNILVR, INOXWIND, KPITTECH, MFSL, PREMIERENE, RVNL, SUPREMEIND, SWIGGY, TATACONSUM, VBL</t>
+          <t>AKUMS, CANFINHOME, HAVELLS, AARTIIND, APLAPOLLO, ATUL, BPCL, BSOFT, COALINDIA, ERIS, FACT, GRAVITA, HBLENGINE, HFCL, HINDUNILVR, HONAUT, IGIL, INOXWIND, IOB, KPITTECH, MFSL, NTPCGREEN, PREMIERENE, RCF, RVNL, SUPREMEIND, SWIGGY, TATACONSUM, TECHNOE, TITAGARH, TRIVENI, VBL</t>
         </is>
       </c>
     </row>
@@ -3292,16 +3292,16 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>BIOCON, COFORGE, CROMPTON, GMRAIRPORT, ICICIGI, KFINTECH, NESTLEIND, OIL, PAGEIND, PAYTM, PHOENIXLTD, POWERINDIA, PRESTIGE, TATACONSUM, TATAPOWER, TORNTPOWER</t>
+          <t>ACMESOLAR, NCC, ZFCVINDIA, ACE, AIAENG, AKZOINDIA, ANANDRATHI, APLLTD, BBTC, BIOCON, COFORGE, CROMPTON, CYIENT, EMCURE, ERIS, FACT, GMRAIRPORT, ICICIGI, JSWINFRA, KFINTECH, LLOYDSME, MRPL, NESTLEIND, OIL, PAGEIND, PAYTM, PHOENIXLTD, POWERINDIA, PRESTIGE, RCF, RHIM, SIGNATURE, SJVN, SOBHA, TATACONSUM, TATAPOWER, TITAGARH, TORNTPOWER, WHIRLPOOL</t>
         </is>
       </c>
     </row>
@@ -3317,7 +3317,7 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>29</v>
+        <v>63</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
@@ -3326,7 +3326,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>GODREJPROP, SBILIFE, SONACOMS, TRENT, ULTRACEMCO, ADANIENSOL, APLAPOLLO, ASIANPAINT, BHARATFORG, BHARTIARTL, CAMS, CANBK, DELHIVERY, DMART, GAIL, GRASIM, IDFCFIRSTB, INDIGO, INFY, JINDALSTEL, LAURUSLABS, MANKIND, MARICO, NATIONALUM, NTPC, PRESTIGE, SHRIRAMFIN, SUNPHARMA, TATASTEEL</t>
+          <t>GODREJPROP, HONAUT, SBILIFE, SONACOMS, TRENT, ULTRACEMCO, ADANIENSOL, AIAENG, APLAPOLLO, ARE&amp;M, ASIANPAINT, BALKRISIND, BHARATFORG, BHARTIARTL, BIKAJI, CAMS, CANBK, CHAMBLFERT, CHENNPETRO, COHANCE, CRAFTSMAN, DEEPAKNTR, DELHIVERY, DMART, EMAMILTD, FIRSTCRY, FLUOROCHEM, FORCEMOT, GAIL, GLAND, GMDCLTD, GRAPHITE, GRASIM, HEG, IDBI, IDFCFIRSTB, IIFL, INDGN, INDIGO, INFY, IRCTC, JINDALSTEL, JKCEMENT, JYOTICNC, KIRLOSENG, LAURUSLABS, M&amp;MFIN, MAHABANK, MANKIND, MARICO, NATIONALUM, NTPC, NUVOCO, PRESTIGE, RAMCOCEM, RPOWER, SHRIRAMFIN, SUNPHARMA, TATACHEM, TATACOMM, TATASTEEL, TRIDENT, VENTIVE</t>
         </is>
       </c>
     </row>
@@ -3342,7 +3342,7 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>37</v>
+        <v>78</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
@@ -3351,7 +3351,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>BANKBARODA, BANKINDIA, INDHOTEL, LICHSGFIN, PNB, UNIONBANK, ADANIENSOL, ALKEM, ASHOKLEY, ASIANPAINT, BAJAJFINSV, BANDHANBNK, BDL, BHARATFORG, BOSCHLTD, CANBK, DABUR, HINDUNILVR, IDFCFIRSTB, IEX, IREDA, JINDALSTEL, KOTAKBANK, LAURUSLABS, LT, LTM, MARICO, MAXHEALTH, MAZDOCK, MPHASIS, NATIONALUM, NTPC, ONGC, RELIANCE, SHRIRAMFIN, SIEMENS, TATASTEEL</t>
+          <t>ABFRL, AWL, BANKBARODA, BANKINDIA, INDHOTEL, LICHSGFIN, MRF, NIVABUPA, PNB, STARHEALTH, TIMKEN, UNIONBANK, 3MINDIA, ADANIENSOL, AJANTPHARM, ALKEM, APARINDS, ASAHIINDIA, ASHOKLEY, ASIANPAINT, ASTERDM, ASTRAZEN, BAJAJFINSV, BANDHANBNK, BDL, BHARATFORG, BOSCHLTD, CANBK, CHAMBLFERT, CLEAN, CRAFTSMAN, CREDITACC, DABUR, ENDURANCE, FSL, GRANULES, GRAPHITE, HEG, HINDCOPPER, HINDUNILVR, IDBI, IDFCFIRSTB, IEX, IFCI, IIFL, INOXINDIA, IREDA, JBCHEPHARM, JINDALSTEL, JUBLINGREA, JUBLPHARMA, JYOTHYLAB, JYOTICNC, KIMS, KOTAKBANK, LAURUSLABS, LT, LTM, MAHABANK, MAPMYINDIA, MARICO, MAXHEALTH, MAZDOCK, MEDANTA, MPHASIS, NATIONALUM, NTPC, OLAELEC, ONGC, RADICO, RELIANCE, SHRIRAMFIN, SIEMENS, SUNDRMFAST, TATASTEEL, THERMAX, WOCKPHARMA, ZENSARTECH</t>
         </is>
       </c>
     </row>
@@ -3367,7 +3367,7 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>35</v>
+        <v>95</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
@@ -3376,7 +3376,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>POWERINDIA, AMBER, ANGELONE, AUBANK, CIPLA, ZYDUSLIFE, ADANIENT, ALKEM, ASTRAL, BAJAJ-AUTO, BAJAJFINSV, BAJFINANCE, BSE, CDSL, COLPAL, CONCOR, ETERNAL, HCLTECH, HDFCLIFE, HEROMOTOCO, HUDCO, ICICIBANK, INDIANB, INDUSINDBK, LTM, M&amp;M, MARUTI, MAZDOCK, MPHASIS, NHPC, PAYTM, PIIND, SOLARINDS, SWIGGY, TORNTPHARM</t>
+          <t>POWERINDIA, TECHNOE, AEGISLOG, AMBER, ANGELONE, AUBANK, CGCL, CIPLA, DOMS, INDIAMART, INTELLECT, J&amp;KBANK, KPRMILL, NH, TATACOMM, ZYDUSLIFE, 3MINDIA, ADANIENT, AFCONS, ALKEM, APLLTD, ARE&amp;M, ASTERDM, ASTRAL, BAJAJ-AUTO, BAJAJFINSV, BAJFINANCE, BERGEPAINT, BIKAJI, BSE, BSOFT, CDSL, CEATLTD, CERA, COLPAL, CONCOR, CONCORDBIO, CREDITACC, CRISIL, CYIENT, DEEPAKNTR, DEVYANI, ELGIEQUIP, ENRIN, ETERNAL, FIVESTAR, GLAND, GODREJAGRO, GPIL, GSPL, GUJGASLTD, HCLTECH, HDFCLIFE, HEROMOTOCO, HFCL, HUDCO, ICICIBANK, INDIANB, INDUSINDBK, ITCHOTELS, JBMA, JPPOWER, JSL, LTM, M&amp;M, MARUTI, MAZDOCK, MEDANTA, METROPOLIS, MOTILALOFS, MPHASIS, MRPL, NEULANDLAB, NHPC, NSLNISP, OLECTRA, PAYTM, PCBL, PIIND, PVRINOX, RAINBOW, REDINGTON, SAPPHIRE, SCHNEIDER, SOBHA, SOLARINDS, SWIGGY, SYRMA, TATAINVEST, TORNTPHARM, TRIDENT, VGUARD, WOCKPHARMA, ZEEL, ZENSARTECH</t>
         </is>
       </c>
     </row>
@@ -3392,7 +3392,7 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>21</v>
+        <v>53</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>BOSCHLTD, CUMMINSIND, EXIDEIND, HINDALCO, SAMMAANCAP, ASIANPAINT, BLUESTARCO, GLENMARK, HUDCO, ICICIPRULI, IEX, KPITTECH, MANAPPURAM, MARICO, ONGC, PNBHOUSING, POLYCAB, SBICARD, SBIN, UNITDSPR, VOLTAS</t>
+          <t>AKZOINDIA, APTUS, ASTRAZEN, BOSCHLTD, CEATLTD, CUMMINSIND, EXIDEIND, HINDALCO, INOXINDIA, MRF, RAILTEL, SAMMAANCAP, SCI, SUNDARMFIN, TIMKEN, ASIANPAINT, AWL, BEML, BIKAJI, BLUESTARCO, CLEAN, DATAPATTNS, DOMS, EIDPARRY, ELGIEQUIP, GLAND, GLENMARK, HAPPSTMNDS, HUDCO, ICICIPRULI, IEX, IRCON, KIMS, KPITTECH, LEMONTREE, MANAPPURAM, MARICO, NLCINDIA, ONGC, PNBHOUSING, POLYCAB, RAMCOCEM, REDINGTON, RITES, SBICARD, SBIN, SONATSOFTW, STARHEALTH, TBOTEK, THELEELA, UNITDSPR, VIJAYA, VOLTAS</t>
         </is>
       </c>
     </row>
@@ -3417,7 +3417,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>32</v>
+        <v>81</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -3426,7 +3426,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>BAJFINANCE, BAJAJFINSV, IDEA, JIOFIN, MCX, POLICYBZR, ZYDUSLIFE, ADANIPORTS, ALKEM, CROMPTON, DABUR, EICHERMOT, GAIL, GODREJCP, HAL, INDUSTOWER, IREDA, IRFC, KALYANKJIL, KAYNES, LT, LTM, MAXHEALTH, MPHASIS, MUTHOOTFIN, OBEROIRLTY, PGEL, POWERINDIA, PRESTIGE, SRF, SUNPHARMA, SYNGENE</t>
+          <t>BAJFINANCE, ABLBL, BAJAJFINSV, BAJAJHFL, CYIENT, DBREALTY, IDEA, INDIAMART, JIOFIN, JMFINANCIL, JSL, MCX, NEULANDLAB, POLICYBZR, ZYDUSLIFE, 3MINDIA, AAVAS, ADANIPORTS, ADANIPOWER, AEGISVOPAK, AGARWALEYE, ALKEM, ANANTRAJ, APARINDS, BHARTIHEXA, CEATLTD, CHALET, CRISIL, CROMPTON, DABUR, DEEPAKNTR, EICHERMOT, ELECON, ELGIEQUIP, ENDURANCE, ENGINERSIN, ENRIN, FSL, GAIL, GLAXO, GODREJCP, HAL, IGL, INDUSTOWER, IREDA, IRFC, KALYANKJIL, KAYNES, KSB, LT, LTFOODS, LTM, MAHSEAMLES, MANYAVAR, MAXHEALTH, MINDACORP, MOTILALOFS, MPHASIS, MUTHOOTFIN, NAVA, OBEROIRLTY, ONESOURCE, PGEL, POLYMED, POWERINDIA, PRESTIGE, PVRINOX, RADICO, REDINGTON, SAREGAMA, SONATSOFTW, SRF, SUNPHARMA, SYNGENE, TATACHEM, TITAGARH, TRIDENT, UCOBANK, VTL, WELSPUNLIV, WHIRLPOOL</t>
         </is>
       </c>
     </row>
@@ -3442,7 +3442,7 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>PETRONET, ANGELONE, ICICIPRULI, IEX, ADANIENSOL, APLAPOLLO, AXISBANK, DMART, GODREJCP, HCLTECH, JINDALSTEL, KEI, MARICO, MFSL, MOTHERSON, OFSS, TATAELXSI, TORNTPHARM</t>
+          <t>LATENTVIEW, PETRONET, ANGELONE, EMCURE, ICICIPRULI, IEX, IPCALAB, JPPOWER, TATACOMM, WELCORP, ABREL, ACE, ADANIENSOL, AEGISLOG, APLAPOLLO, APOLLOTYRE, ASTRAZEN, AXISBANK, BAYERCROP, CAMPUS, CHOLAHLDNG, COCHINSHIP, COROMANDEL, DMART, EIHOTEL, GODREJCP, GSPL, HCLTECH, IIFL, J&amp;KBANK, JINDALSTEL, JSWCEMENT, KEI, KIMS, MAHSCOOTER, MARICO, MFSL, MOTHERSON, OFSS, OLAELEC, PFIZER, SCHAEFFLER, SUMICHEM, TATAELXSI, THERMAX, TORNTPHARM, UBL, VGUARD, ZEEL</t>
         </is>
       </c>
     </row>
@@ -3467,16 +3467,16 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>33</v>
+        <v>67</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>HINDZINC, LODHA, LTM, POWERGRID, ABCAPITAL, ADANIENT, AMBER, APOLLOHOSP, ASHOKLEY, BAJAJHLDNG, BOSCHLTD, BSE, CDSL, CIPLA, DALBHARAT, DIXON, HDFCBANK, HINDALCO, INDIGO, JSWSTEEL, KFINTECH, LICI, MARUTI, NMDC, PFC, PPLPHARMA, PREMIERENE, SOLARINDS, SONACOMS, TATATECH, TVSMOTOR, ULTRACEMCO, UNOMINDA</t>
+          <t>BATAINDIA, HINDZINC, LODHA, LTM, POWERGRID, SBFC, SUNDARMFIN, ABCAPITAL, ADANIENT, AMBER, APLLTD, APOLLOHOSP, ARE&amp;M, ASHOKLEY, ATHERENERG, BAJAJHLDNG, BALRAMCHIN, BLUEDART, BLUEJET, BOSCHLTD, BSE, CDSL, CENTRALBK, CERA, CGCL, CIPLA, CREDITACC, DALBHARAT, DIXON, FINCABLES, GVT&amp;D, HBLENGINE, HDFCBANK, HINDALCO, INDIGO, INTELLECT, IRB, JSWSTEEL, KEC, KFINTECH, KPRMILL, LICI, M&amp;MFIN, MARUTI, METROPOLIS, MMTC, MRPL, NAM-INDIA, NH, NMDC, PCBL, PFC, POONAWALLA, PPLPHARMA, PREMIERENE, RPOWER, RRKABEL, SAGILITY, SOLARINDS, SONACOMS, SYRMA, TATAINVEST, TATATECH, TECHNOE, TVSMOTOR, ULTRACEMCO, UNOMINDA</t>
         </is>
       </c>
     </row>
@@ -3492,7 +3492,7 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>CHOLAFIN, FEDERALBNK, NBCC, UNITDSPR, VOLTAS, CAMS, GODREJPROP, HAVELLS, INOXWIND, IOC, OBEROIRLTY, PHOENIXLTD, SIEMENS, VEDL</t>
+          <t>CHOLAFIN, FEDERALBNK, LEMONTREE, NBCC, UNITDSPR, VOLTAS, 3MINDIA, ATUL, CAMS, FORCEMOT, GICRE, GODREJPROP, GRAPHITE, HAVELLS, HEXT, INOXWIND, IOC, LTTS, MMTC, NATCOPHARM, OBEROIRLTY, PGHH, PHOENIXLTD, PTCIL, SIEMENS, TEJASNET, TRIVENI, UTIAMC, VEDL</t>
         </is>
       </c>
     </row>
@@ -3517,7 +3517,7 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>AMBUJACEM, AUROPHARMA, DIVISLAB, HDFCAMC, ICICIGI, LUPIN, MOTHERSON, SYNGENE, 360ONE, ADANIENSOL, ADANIENT, BRITANNIA, CROMPTON, DELHIVERY, GAIL, GLENMARK, GMRAIRPORT, IDEA, INDUSTOWER, PAGEIND, PAYTM, PRESTIGE, SAIL, TATAPOWER, TITAN, UNIONBANK</t>
+          <t>AMBUJACEM, AUROPHARMA, CASTROLIND, DIVISLAB, HDFCAMC, ICICIGI, JINDALSAW, LATENTVIEW, LUPIN, MOTHERSON, SAILIFE, SYNGENE, USHAMART, VTL, 360ONE, 3MINDIA, AARTIIND, ADANIENSOL, ADANIENT, ALOKINDS, ATHERENERG, BRITANNIA, CENTURYPLY, CROMPTON, DELHIVERY, GAIL, GLENMARK, GMRAIRPORT, GODREJIND, IDEA, IKS, INDUSTOWER, JKTYRE, JWL, JYOTICNC, KIRLOSENG, MANYAVAR, NCC, NETWEB, NLCINDIA, ONESOURCE, PAGEIND, PAYTM, POLYMED, PRESTIGE, RAINBOW, SAIL, SJVN, SOBHA, TARIL, TATAPOWER, TITAN, TTML, UNIONBANK, VENTIVE, VMM, WHIRLPOOL, ZFCVINDIA</t>
         </is>
       </c>
     </row>
@@ -3542,7 +3542,7 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
@@ -3551,7 +3551,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>INDUSTOWER, 360ONE, BHARATFORG, COFORGE, KFINTECH, LTM, MPHASIS, POWERGRID, RECLTD, ASTRAL, BAJAJ-AUTO, BSE, DELHIVERY, DRREDDY, GLENMARK, IDFCFIRSTB, KEI, LTF, NHPC, TCS</t>
+          <t>INDUSTOWER, 360ONE, APTUS, BHARATFORG, BIKAJI, CEATLTD, COFORGE, ECLERX, GUJGASLTD, KFINTECH, LTM, MAPMYINDIA, MPHASIS, NAVINFLUOR, POWERGRID, RAILTEL, RECLTD, SOBHA, ABSLAMC, AKUMS, ASTRAL, ATUL, BAJAJ-AUTO, BASF, BSE, CASTROLIND, CENTURYPLY, COROMANDEL, DEEPAKNTR, DELHIVERY, DRREDDY, GLENMARK, IDFCFIRSTB, KEI, KIRLOSBROS, LTF, LTFOODS, NHPC, NUVOCO, TCS, TRIDENT, TRITURBINE</t>
         </is>
       </c>
     </row>
@@ -3567,16 +3567,16 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>28</v>
+        <v>79</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>BIOCON, DABUR, DALBHARAT, GRASIM, PETRONET, PIIND, WAAREEENER, ASTRAL, BOSCHLTD, BPCL, DIVISLAB, DMART, GLENMARK, KFINTECH, LUPIN, MOTHERSON, NMDC, POWERINDIA, RVNL, SUPREMEIND, TATATECH, TCS, TMPV, TRENT, UNITDSPR, UNOMINDA, UPL, VOLTAS</t>
+          <t>J&amp;KBANK, AARTIIND, ALOKINDS, APARINDS, BIOCON, CARBORUNIV, DABUR, DALBHARAT, DCMSHRIRAM, GLAXO, GODIGIT, GRASIM, IDBI, JKTYRE, MINDACORP, NIACL, PETRONET, PIIND, SCHNEIDER, TRIVENI, WAAREEENER, AEGISVOPAK, AKUMS, ASTRAL, BALRAMCHIN, BLUEDART, BOSCHLTD, BPCL, CASTROLIND, CENTURYPLY, CHAMBLFERT, CHENNPETRO, CLEAN, COCHINSHIP, CREDITACC, DEEPAKNTR, DIVISLAB, DMART, ELGIEQUIP, FSL, GLENMARK, GRANULES, HSCL, INDIAMART, IRB, KARURVYSYA, KFINTECH, KIRLOSBROS, KIRLOSENG, KPIL, LALPATHLAB, LUPIN, M&amp;MFIN, MAHABANK, MOTHERSON, NMDC, NSLNISP, NTPCGREEN, OLECTRA, POWERINDIA, RAILTEL, RVNL, SUPREMEIND, SWANCORP, TATACHEM, TATATECH, TCS, TIMKEN, TITAGARH, TMPV, TRENT, TRIDENT, UCOBANK, UNITDSPR, UNOMINDA, UPL, VOLTAS, WELSPUNLIV, WOCKPHARMA</t>
         </is>
       </c>
     </row>
@@ -3592,7 +3592,7 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>28</v>
+        <v>67</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
@@ -3601,7 +3601,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>AXISBANK, BHARATFORG, COFORGE, POWERGRID, RECLTD, TRENT, ADANIPORTS, ANGELONE, ASHOKLEY, BAJAJFINSV, BIOCON, BOSCHLTD, DLF, ETERNAL, GMRAIRPORT, INFY, KFINTECH, LTM, MARUTI, MCX, MOTHERSON, NAUKRI, PNB, RVNL, UNOMINDA, UPL, VOLTAS, ZYDUSLIFE</t>
+          <t>APTUS, AXISBANK, BAJAJHFL, BHARATFORG, CENTURYPLY, CHAMBLFERT, COCHINSHIP, COFORGE, ELGIEQUIP, HSCL, INDIACEM, JUBLPHARMA, KIRLOSENG, MINDACORP, POWERGRID, RECLTD, SWANCORP, TITAGARH, TRENT, WELSPUNLIV, AADHARHFC, AARTIIND, ADANIPORTS, ADANIPOWER, ANGELONE, ASHOKLEY, BAJAJFINSV, BIOCON, BOSCHLTD, CASTROLIND, CRAFTSMAN, DCMSHRIRAM, DLF, ECLERX, ELECON, ENRIN, ETERNAL, GMRAIRPORT, GUJGASLTD, IDBI, IKS, INFY, IPCALAB, KFINTECH, KIRLOSBROS, LTM, MARUTI, MCX, METROPOLIS, MOTHERSON, NAUKRI, NAVINFLUOR, NIACL, PNB, RVNL, SCHAEFFLER, SCHNEIDER, SCI, SIGNATURE, SOBHA, SUNDARMFIN, TRITURBINE, UNOMINDA, UPL, VOLTAS, ZENSARTECH, ZYDUSLIFE</t>
         </is>
       </c>
     </row>
@@ -3617,16 +3617,16 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>APOLLOHOSP, CAMS, TORNTPOWER, ADANIENT, AMBER, ANGELONE, BAJAJ-AUTO, BRITANNIA, BSE, DIVISLAB, DLF, IRFC, KEI, LUPIN, MANKIND, MPHASIS, PETRONET, PREMIERENE, SIEMENS, WAAREEENER</t>
+          <t>LATENTVIEW, APOLLOHOSP, CAMS, SAILIFE, TORNTPOWER, ACMESOLAR, ADANIENT, ALOKINDS, AMBER, ANGELONE, APARINDS, BAJAJ-AUTO, BALRAMCHIN, BRITANNIA, BSE, CREDITACC, DIVISLAB, DLF, ELECON, IRB, IRFC, J&amp;KBANK, JINDALSAW, JWL, KEI, KPIL, LALPATHLAB, LUPIN, MANKIND, MPHASIS, PETRONET, PREMIERENE, SIEMENS, SUNTV, TATACHEM, TECHNOE, TRIVENI, WAAREEENER</t>
         </is>
       </c>
     </row>
@@ -3642,7 +3642,7 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
@@ -3651,7 +3651,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>SRF, ADANIENSOL, ADANIGREEN, APOLLOHOSP, ASTRAL, AUROPHARMA, CAMS, COFORGE, GODREJCP, GRASIM, HEROMOTOCO, PATANJALI, PERSISTENT, PNB, TCS, TORNTPOWER</t>
+          <t>NSLNISP, SRF, WOCKPHARMA, ADANIENSOL, ADANIGREEN, APOLLOHOSP, ASTRAL, AUROPHARMA, CAMS, CARBORUNIV, COFORGE, CRAFTSMAN, ENRIN, GLAXO, GODREJCP, GRANULES, GRAPHITE, GRASIM, HEROMOTOCO, HFCL, HONASA, INDIACEM, JSWINFRA, JUBLPHARMA, MSUMI, NLCINDIA, PATANJALI, PERSISTENT, PFIZER, PNB, REDINGTON, TCS, TORNTPOWER</t>
         </is>
       </c>
     </row>
@@ -3667,7 +3667,7 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
@@ -3676,7 +3676,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>ADANIPORTS, LT, CDSL, INDUSTOWER, POLYCAB, POWERINDIA, 360ONE, ADANIENT, AUBANK, BAJAJHLDNG, BHEL, CGPOWER, DABUR, GODREJPROP, HINDZINC, ICICIBANK, IEX, JIOFIN, LUPIN, MAZDOCK, MPHASIS, SHREECEM, TATAELXSI</t>
+          <t>ADANIPORTS, LT, AIAENG, BSOFT, CAMPUS, CCL, CDSL, INDUSTOWER, POLYCAB, POWERINDIA, 360ONE, AADHARHFC, ADANIENT, ATGL, AUBANK, BAJAJHLDNG, BHEL, CENTRALBK, CGPOWER, CRAFTSMAN, CYIENT, DABUR, GODREJIND, GODREJPROP, HINDZINC, HOMEFIRST, ICICIBANK, IEX, IFCI, INOXINDIA, INTELLECT, JIOFIN, JKCEMENT, JSWINFRA, LUPIN, MAZDOCK, MPHASIS, REDINGTON, SCHAEFFLER, SHREECEM, TATAELXSI, THELEELA, TRITURBINE</t>
         </is>
       </c>
     </row>
@@ -3692,7 +3692,7 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>39</v>
+        <v>102</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
@@ -3701,7 +3701,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>MAZDOCK, AUROPHARMA, CIPLA, FORTIS, GODREJCP, HDFCLIFE, HEROMOTOCO, INDHOTEL, INDUSINDBK, IRFC, LODHA, MANKIND, SRF, ULTRACEMCO, WIPRO, ADANIENSOL, ALKEM, AUBANK, BAJAJFINSV, BEL, CONCOR, EICHERMOT, GAIL, GMRAIRPORT, HAVELLS, HINDZINC, ICICIGI, IEX, JUBLFOOD, KALYANKJIL, KOTAKBANK, LICHSGFIN, LICI, OFSS, PGEL, PRESTIGE, RVNL, TATAPOWER, YESBANK</t>
+          <t>LINDEINDIA, MAZDOCK, AFFLE, ANANDRATHI, AUROPHARMA, BBTC, CAMPUS, CHALET, CIPLA, EIDPARRY, ENDURANCE, FORTIS, GODREJCP, GSPL, HDFCLIFE, HEROMOTOCO, HFCL, INDGN, INDHOTEL, INDUSINDBK, IRFC, JSL, KSB, LODHA, MANKIND, NAVA, NLCINDIA, PCBL, PVRINOX, SRF, TATAINVEST, UBL, ULTRACEMCO, USHAMART, VENTIVE, WIPRO, 3MINDIA, AAVAS, ADANIENSOL, AEGISLOG, AIIL, ALKEM, APLLTD, AUBANK, AWL, BAJAJFINSV, BEL, BEML, CAPLIPOINT, CASTROLIND, CCL, CHOLAHLDNG, COHANCE, CONCOR, COROMANDEL, DATAPATTNS, DBREALTY, DEVYANI, EICHERMOT, FACT, FLUOROCHEM, GAIL, GMRAIRPORT, GPIL, HAVELLS, HEG, HEXT, HINDZINC, HOMEFIRST, ICICIGI, IEX, IGIL, IGL, IIFL, IKS, IOB, JBMA, JUBLFOOD, KALYANKJIL, KIMS, KOTAKBANK, LICHSGFIN, LICI, NH, OFSS, OLAELEC, PGEL, PRAJIND, PRESTIGE, RHIM, RITES, RVNL, SAREGAMA, SONATSOFTW, SUMICHEM, TATACOMM, TATAPOWER, TITAGARH, UCOBANK, VMM, YESBANK, ZFCVINDIA</t>
         </is>
       </c>
     </row>
@@ -3717,16 +3717,16 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>30</v>
+        <v>75</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>BEL, BRITANNIA, CGPOWER, NUVAMA, PNBHOUSING, AMBER, BAJAJHLDNG, BHEL, BLUESTARCO, CDSL, CUMMINSIND, ETERNAL, GODREJPROP, HDFCAMC, HINDPETRO, HINDZINC, IDEA, IEX, INOXWIND, IREDA, JSWENERGY, JSWSTEEL, KAYNES, NBCC, NHPC, NYKAA, OBEROIRLTY, PATANJALI, POLYCAB, SUZLON</t>
+          <t>MOTILALOFS, ACMESOLAR, BEL, BRITANNIA, CGPOWER, ENGINERSIN, GMDCLTD, NUVAMA, PNBHOUSING, TECHNOE, TTML, ACE, AIAENG, AMBER, ATGL, BAJAJHLDNG, BATAINDIA, BAYERCROP, BHEL, BLUESTARCO, BSOFT, CANFINHOME, CDSL, CENTRALBK, CESC, CGCL, CHOICEIN, CRISIL, CUMMINSIND, CYIENT, DATAPATTNS, DOMS, EIHOTEL, ERIS, ETERNAL, FINPIPE, GODREJAGRO, GODREJIND, GODREJPROP, HDFCAMC, HEXT, HINDPETRO, HINDZINC, HOMEFIRST, IDEA, IEX, INOXINDIA, INOXWIND, IRCON, IRCTC, IREDA, ITI, JSWCEMENT, JSWENERGY, JSWSTEEL, JYOTICNC, KAYNES, KEC, LTFOODS, NBCC, NHPC, NYKAA, OBEROIRLTY, OLECTRA, PATANJALI, POLYCAB, RCF, RPOWER, SCI, SJVN, SUZLON, TEJASNET, THELEELA, UTIAMC, WELCORP</t>
         </is>
       </c>
     </row>
@@ -3742,7 +3742,7 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>36</v>
+        <v>73</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>CANBK, COALINDIA, DALBHARAT, EXIDEIND, FEDERALBNK, HINDALCO, KALYANKJIL, NESTLEIND, NTPC, ONGC, SAIL, SOLARINDS, UNIONBANK, VBL, APLAPOLLO, BSE, CAMS, GODREJPROP, HAL, HAVELLS, HINDUNILVR, ICICIPRULI, JSWSTEEL, LAURUSLABS, MPHASIS, NATIONALUM, OIL, PAGEIND, RBLBANK, SIEMENS, SUNPHARMA, TATASTEEL, TMPV, TORNTPOWER, VEDL, WIPRO</t>
+          <t>CANBK, CLEAN, COALINDIA, DALBHARAT, ELECON, EXIDEIND, FEDERALBNK, FSL, HINDALCO, JKTYRE, JMFINANCIL, KALYANKJIL, MAPMYINDIA, NESTLEIND, NTPC, ONGC, POLYMED, SAIL, SHYAMMETL, SOLARINDS, UNIONBANK, VBL, VIJAYA, AARTIIND, AFCONS, ALOKINDS, APLAPOLLO, APOLLOTYRE, BBTC, BIKAJI, BLS, BSE, CAMS, DOMS, FIRSTCRY, FIVESTAR, GODREJPROP, HAL, HAVELLS, HINDCOPPER, HINDUNILVR, ICICIPRULI, IRB, JBMA, JINDALSAW, JSL, JSWSTEEL, LAURUSLABS, LEMONTREE, LINDEINDIA, M&amp;MFIN, MAHABANK, MANYAVAR, METROPOLIS, MPHASIS, MRPL, NATIONALUM, OIL, PAGEIND, RADICO, RBLBANK, RHIM, SAILIFE, SIEMENS, SIGNATURE, SUNPHARMA, TATACHEM, TATAINVEST, TATASTEEL, TMPV, TORNTPOWER, VEDL, WIPRO</t>
         </is>
       </c>
     </row>
@@ -3767,7 +3767,7 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>42</v>
+        <v>89</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
@@ -3776,7 +3776,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>BANKINDIA, JINDALSTEL, PHOENIXLTD, TECHM, APLAPOLLO, AXISBANK, BHARTIARTL, CANBK, MAXHEALTH, PPLPHARMA, SHRIRAMFIN, ALKEM, AMBUJACEM, CIPLA, COALINDIA, COLPAL, CONCOR, DELHIVERY, DIVISLAB, DIXON, ETERNAL, FORTIS, GRASIM, HCLTECH, HDFCLIFE, HINDALCO, ICICIBANK, IDEA, INDIGO, JSWSTEEL, KOTAKBANK, MARICO, NESTLEIND, PERSISTENT, PIDILITIND, PRESTIGE, SBICARD, SOLARINDS, TATACONSUM, TVSMOTOR, UNIONBANK, UPL</t>
+          <t>BANKINDIA, JINDALSTEL, PHOENIXLTD, TECHM, APLAPOLLO, CUB, AXISBANK, BHARTIARTL, CANBK, FINCABLES, FORCEMOT, MAXHEALTH, MRPL, PPLPHARMA, SBFC, SHRIRAMFIN, STARHEALTH, ZENTEC, ABSLAMC, AFCONS, AFFLE, ALKEM, AMBUJACEM, ASTRAZEN, ATUL, BAJAJHFL, BALKRISIND, BERGEPAINT, BLS, CIPLA, COALINDIA, COLPAL, CONCOR, DCMSHRIRAM, DELHIVERY, DIVISLAB, DIXON, EMAMILTD, ETERNAL, FORTIS, GESHIP, GILLETTE, GRASIM, GSPL, HCLTECH, HDFCLIFE, HINDALCO, HINDCOPPER, HONASA, HONAUT, HYUNDAI, ICICIBANK, IDEA, IIFL, INDIGO, JSWSTEEL, KOTAKBANK, KSB, LLOYDSME, MANYAVAR, MARICO, NAVA, NESTLEIND, NEULANDLAB, NSLNISP, NTPCGREEN, PERSISTENT, PFIZER, PIDILITIND, PRESTIGE, RADICO, RAILTEL, RKFORGE, SAGILITY, SAPPHIRE, SBICARD, SOLARINDS, SUMICHEM, SUNDARMFIN, SUNDRMFAST, TARIL, TATACONSUM, TIMKEN, TVSMOTOR, UNIONBANK, UPL, VENTIVE, WOCKPHARMA, ZENSARTECH</t>
         </is>
       </c>
     </row>
@@ -3792,7 +3792,7 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>28</v>
+        <v>74</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
@@ -3801,7 +3801,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>ASIANPAINT, INDIANB, ITC, SWIGGY, CROMPTON, ICICIPRULI, JIOFIN, POLICYBZR, ANGELONE, BHARTIARTL, BPCL, CHOLAFIN, CUMMINSIND, DIXON, HINDUNILVR, INDIGO, IREDA, KPITTECH, LTF, MARUTI, NHPC, NUVAMA, NYKAA, POWERINDIA, RVNL, SBIN, TITAN, TORNTPHARM</t>
+          <t>ASIANPAINT, INDIANB, DEEPAKFERT, ITC, LTTS, PGHH, SWIGGY, ANANDRATHI, CROMPTON, ICICIPRULI, JIOFIN, POLICYBZR, TBOTEK, VGUARD, ABBOTINDIA, AEGISVOPAK, AGARWALEYE, ANANTRAJ, ANGELONE, APARINDS, ATHERENERG, BASF, BATAINDIA, BAYERCROP, BHARTIARTL, BPCL, BRIGADE, CASTROLIND, CHOLAFIN, CONCORDBIO, CUMMINSIND, DIXON, ENGINERSIN, GMDCLTD, GODREJAGRO, HINDCOPPER, HINDUNILVR, INDIGO, IRCTC, IREDA, ITI, KAJARIACER, KARURVYSYA, KPITTECH, LATENTVIEW, LTF, LTFOODS, MARUTI, MRF, MSUMI, NEWGEN, NHPC, NIVABUPA, NUVAMA, NYKAA, ONESOURCE, POWERINDIA, RAINBOW, RAMCOCEM, RCF, RPOWER, RRKABEL, RVNL, SBIN, SHYAMMETL, SYRMA, THERMAX, TITAGARH, TITAN, TORNTPHARM, TRITURBINE, TTML, WELCORP, ZENTEC</t>
         </is>
       </c>
     </row>
@@ -3817,16 +3817,16 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>SYNGENE, HUDCO, OIL, ONGC, SAIL, VBL, VEDL</t>
+          <t>GILLETTE, GESHIP, SYNGENE, AADHARHFC, ACC, AKZOINDIA, BALKRISIND, CHALET, CRISIL, CUB, DEVYANI, ESCORTS, GRSE, HAPPSTMNDS, HUDCO, JBCHEPHARM, JKCEMENT, NAM-INDIA, NATCOPHARM, OIL, ONGC, POLYMED, PTCIL, RAILTEL, RAINBOW, RAMCOCEM, RKFORGE, SAIL, SUNDRMFAST, VBL, VEDL</t>
         </is>
       </c>
     </row>
@@ -3842,16 +3842,16 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>BDL, BPCL, CAMS, COLPAL, INDUSTOWER, LAURUSLABS, SHRIRAMFIN, TATACONSUM, TORNTPHARM, TORNTPOWER, TVSMOTOR, ULTRACEMCO, YESBANK</t>
+          <t>MAHSCOOTER, ABBOTINDIA, AEGISVOPAK, ALKYLAMINE, ATHERENERG, BASF, BDL, BPCL, CAMS, CHENNPETRO, COLPAL, CREDITACC, HONAUT, HYUNDAI, INDIACEM, INDUSTOWER, JKCEMENT, KPRMILL, LAURUSLABS, MMTC, NETWEB, SAGILITY, SAILIFE, SHRIRAMFIN, STARHEALTH, SUNDRMFAST, TATACONSUM, TORNTPHARM, TORNTPOWER, TRIVENI, TVSMOTOR, ULTRACEMCO, YESBANK</t>
         </is>
       </c>
     </row>
@@ -3867,16 +3867,16 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>ADANIENSOL, BSE, CHOLAFIN, CROMPTON, HDFCAMC, INFY, MUTHOOTFIN, PREMIERENE</t>
+          <t>AAVAS, MOTILALOFS, THELEELA, ADANIENSOL, AGARWALEYE, BSE, CENTRALBK, CHOLAFIN, CROMPTON, GICRE, HDFCAMC, INFY, LATENTVIEW, MUTHOOTFIN, NIVABUPA, PREMIERENE, SUNDARMFIN</t>
         </is>
       </c>
     </row>
@@ -3892,16 +3892,16 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>ADANIENSOL, ADANIGREEN, ASTRAL, BEL, ETERNAL, HAL, ICICIBANK, INDUSINDBK, PFC, PIIND, POWERINDIA, PREMIERENE, SONACOMS, ZYDUSLIFE</t>
+          <t>MAHSCOOTER, ADANIENSOL, ADANIGREEN, AKUMS, AKZOINDIA, ALKYLAMINE, ALOKINDS, ASTRAL, BALKRISIND, BEL, COROMANDEL, ETERNAL, FSL, GRSE, HAL, HOMEFIRST, ICICIBANK, INDUSINDBK, IRB, JBCHEPHARM, M&amp;MFIN, MAHABANK, MMTC, NAM-INDIA, NATCOPHARM, PFC, PIIND, POWERINDIA, PREMIERENE, PTCIL, RAMCOCEM, SONACOMS, STARHEALTH, TATACHEM, TRIDENT, ZYDUSLIFE</t>
         </is>
       </c>
     </row>
@@ -3917,16 +3917,16 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>ABB, ADANIGREEN, ANGELONE, BAJAJHLDNG, BANDHANBNK, CDSL, DIVISLAB, GLENMARK, GODREJPROP, JSWSTEEL, PETRONET, PNB, SUPREMEIND, TCS, VOLTAS</t>
+          <t>CCL, ABB, ADANIGREEN, AIAENG, AJANTPHARM, ANANDRATHI, ANGELONE, ASAHIINDIA, ATGL, ATUL, BAJAJHLDNG, BANDHANBNK, CDSL, DIVISLAB, ESCORTS, GLAND, GLAXO, GLENMARK, GODREJPROP, GRANULES, GVT&amp;D, IFCI, INDIAMART, JSWSTEEL, KARURVYSYA, NSLNISP, PETRONET, PNB, REDINGTON, SAGILITY, SBFC, SCHAEFFLER, SUPREMEIND, SYRMA, TCS, TIMKEN, VOLTAS, VTL, WOCKPHARMA</t>
         </is>
       </c>
     </row>
@@ -3942,7 +3942,7 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
@@ -3951,7 +3951,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>GRASIM, AUROPHARMA, BHEL, COALINDIA, COLPAL, GODREJCP, HINDALCO, LODHA, MANKIND, SOLARINDS, SRF, TORNTPHARM, UNIONBANK</t>
+          <t>CARBORUNIV, EMCURE, GODIGIT, GRASIM, AUROPHARMA, BAYERCROP, BHEL, CENTRALBK, COALINDIA, COLPAL, GODREJCP, HFCL, HINDALCO, INTELLECT, J&amp;KBANK, LODHA, MANKIND, MANYAVAR, NH, NLCINDIA, NUVOCO, RHIM, SAPPHIRE, SAREGAMA, SOLARINDS, SONATSOFTW, SRF, TATAINVEST, THELEELA, TORNTPHARM, UNIONBANK</t>
         </is>
       </c>
     </row>
@@ -3967,7 +3967,7 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
@@ -3976,7 +3976,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>POWERGRID, BHARATFORG, IDFCFIRSTB, INDUSTOWER, RECLTD, ASHOKLEY, ASTRAL, BAJAJFINSV, BAJAJHLDNG, BHARTIARTL, CDSL, HDFCLIFE, IRFC, PAGEIND, PETRONET</t>
+          <t>POWERGRID, APTUS, BHARATFORG, CEATLTD, IDFCFIRSTB, INDUSTOWER, LTFOODS, RECLTD, AADHARHFC, ASHOKLEY, ASTRAL, BAJAJFINSV, BAJAJHLDNG, BHARTIARTL, CAMPUS, CDSL, CHOLAHLDNG, CYIENT, ECLERX, ERIS, FIRSTCRY, GUJGASLTD, HDFCLIFE, HEG, HOMEFIRST, IRFC, JBMA, KIMS, LALPATHLAB, OLAELEC, PAGEIND, PETRONET, PVRINOX, REDINGTON, SOBHA, TRITURBINE, USHAMART, VENTIVE, ZFCVINDIA</t>
         </is>
       </c>
     </row>
@@ -3992,7 +3992,7 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>42</v>
+        <v>106</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>TRENT, DALBHARAT, ALKEM, AMBER, AUROPHARMA, BAJAJFINSV, BAJFINANCE, BDL, BHEL, BIOCON, BOSCHLTD, BSE, DMART, EICHERMOT, GMRAIRPORT, GODREJCP, HDFCBANK, HDFCLIFE, HINDPETRO, ICICIBANK, IRFC, ITC, JSWENERGY, JSWSTEEL, KAYNES, KEI, KFINTECH, LICI, LODHA, LTF, MANKIND, MCX, OBEROIRLTY, PATANJALI, PGEL, PNBHOUSING, RVNL, SAMMAANCAP, SRF, SWIGGY, TECHM, UNOMINDA</t>
+          <t>TRENT, WELSPUNLIV, CEATLTD, CENTURYPLY, CHAMBLFERT, CLEAN, COCHINSHIP, DALBHARAT, ELGIEQUIP, HSCL, JKTYRE, KIRLOSENG, MINDACORP, SWANCORP, TITAGARH, AARTIIND, ACE, ACMESOLAR, AEGISLOG, AFFLE, ALKEM, AMBER, AUROPHARMA, BAJAJFINSV, BAJFINANCE, BDL, BHEL, BIOCON, BOSCHLTD, BSE, CASTROLIND, CCL, CESC, CGCL, CHENNPETRO, CHOLAHLDNG, DMART, EICHERMOT, EIHOTEL, ENGINERSIN, FIRSTCRY, GMRAIRPORT, GODREJAGRO, GODREJCP, GPIL, HDFCBANK, HDFCLIFE, HFCL, HINDCOPPER, HINDPETRO, ICICIBANK, IDBI, INDIAMART, INTELLECT, IOB, IPCALAB, IRCTC, IRFC, ITC, J&amp;KBANK, JKCEMENT, JSWENERGY, JSWSTEEL, KARURVYSYA, KAYNES, KEI, KFINTECH, KIMS, KIRLOSBROS, KPIL, LICI, LODHA, LTF, MANKIND, MCX, NH, NIACL, OBEROIRLTY, ONESOURCE, PATANJALI, PGEL, PGHH, PNBHOUSING, PVRINOX, RAINBOW, RHIM, RITES, RVNL, SAMMAANCAP, SARDAEN, SAREGAMA, SCHAEFFLER, SCI, SJVN, SRF, SWIGGY, TATAINVEST, TECHM, TECHNOE, UCOBANK, UNOMINDA, USHAMART, UTIAMC, VENTIVE, WELCORP, ZFCVINDIA</t>
         </is>
       </c>
     </row>
@@ -4017,7 +4017,7 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
@@ -4026,7 +4026,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>AMBER, ASHOKLEY, AXISBANK, BAJFINANCE, COFORGE, DLF, ETERNAL, GMRAIRPORT, HDFCBANK, HINDPETRO, KAYNES, LICHSGFIN, LICI, LTM, NESTLEIND, OBEROIRLTY, PATANJALI, PGEL, PNBHOUSING, RELIANCE, SAIL, SAMMAANCAP</t>
+          <t>ACE, ACMESOLAR, AEGISLOG, AMBER, ASHOKLEY, AXISBANK, BAJFINANCE, BATAINDIA, CESC, CGCL, COFORGE, CRAFTSMAN, CRISIL, DEEPAKNTR, DLF, EIHOTEL, ENGINERSIN, ENRIN, ERIS, ETERNAL, FINPIPE, GMRAIRPORT, GODREJAGRO, GPIL, HDFCBANK, HINDPETRO, IKS, INDIACEM, INDIAMART, IOB, IRCTC, JINDALSAW, KAYNES, KPRMILL, LICHSGFIN, LICI, LLOYDSME, LTM, NAVINFLUOR, NESTLEIND, NEWGEN, OBEROIRLTY, PATANJALI, PGEL, PNBHOUSING, POLYMED, PTCIL, RAILTEL, RELIANCE, RITES, SAIL, SAMMAANCAP, SCI, SJVN, SYRMA, TECHNOE, UCOBANK, UTIAMC, WELCORP</t>
         </is>
       </c>
     </row>
@@ -4042,7 +4042,7 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>21</v>
+        <v>69</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>HCLTECH, YESBANK, 360ONE, APOLLOHOSP, BDL, BLUESTARCO, BOSCHLTD, CAMS, GAIL, JUBLFOOD, MOTHERSON, MPHASIS, MUTHOOTFIN, OIL, PPLPHARMA, SAIL, TIINDIA, TITAN, TORNTPOWER, TVSMOTOR, UPL</t>
+          <t>HCLTECH, CREDITACC, YESBANK, 360ONE, AAVAS, ABFRL, ABLBL, ANANDRATHI, APLLTD, APOLLOHOSP, AWL, BDL, BHARTIHEXA, BLUESTARCO, BOSCHLTD, CAMS, CAPLIPOINT, CERA, CHALET, DCMSHRIRAM, DEVYANI, EIDPARRY, FACT, GAIL, GODFRYPHLP, GRAPHITE, GRAVITA, HINDCOPPER, HONASA, HONAUT, HYUNDAI, IDBI, IGIL, IGL, INDIACEM, IRCON, J&amp;KBANK, JBMA, JPPOWER, JUBLFOOD, JUBLPHARMA, KEC, MAHABANK, MAHSEAMLES, MAPMYINDIA, MGL, MOTHERSON, MPHASIS, MUTHOOTFIN, NCC, NETWEB, NUVOCO, OIL, OLECTRA, PCBL, PPLPHARMA, PRAJIND, SAIL, SCHNEIDER, SIGNATURE, TIINDIA, TITAN, TORNTPOWER, TTML, TVSMOTOR, UBL, UPL, ZEEL, ZENSARTECH</t>
         </is>
       </c>
     </row>
@@ -4067,7 +4067,7 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>CHOLAFIN, COFORGE, INDHOTEL, TATAPOWER, UNITDSPR, ABCAPITAL, ADANIENT, BPCL, GAIL, IOC, LTM, PIDILITIND, PPLPHARMA, SIEMENS, SUNPHARMA, TITAN, WAAREEENER</t>
+          <t>3MINDIA, AGARWALEYE, BALRAMCHIN, CHOLAFIN, COFORGE, ELECON, INDHOTEL, LALPATHLAB, TATAPOWER, UNITDSPR, ABCAPITAL, ABFRL, ADANIENT, ALOKINDS, ANANTRAJ, APARINDS, BATAINDIA, BLUEDART, BPCL, CHALET, DEVYANI, ENDURANCE, FACT, GAIL, GMDCLTD, GRAVITA, HONASA, HYUNDAI, IOC, IRB, IRCON, KAJARIACER, KEC, KPIL, KSB, LATENTVIEW, LINDEINDIA, LTM, MGL, NAVINFLUOR, OLECTRA, PIDILITIND, POLYMED, PPLPHARMA, PRAJIND, RRKABEL, SIEMENS, SIGNATURE, SUNPHARMA, TATACHEM, TITAN, TRIVENI, WAAREEENER, ZENSARTECH</t>
         </is>
       </c>
     </row>
@@ -4092,7 +4092,7 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>23</v>
+        <v>68</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
@@ -4101,7 +4101,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>EXIDEIND, JIOFIN, LAURUSLABS, MFSL, SBILIFE, SYNGENE, TMPV, PFC, SONACOMS, ULTRACEMCO, ANGELONE, BEL, CROMPTON, GAIL, HAL, JUBLFOOD, KPITTECH, MANAPPURAM, NAUKRI, NHPC, PNB, SBIN, TIINDIA</t>
+          <t>ABLBL, AKZOINDIA, APLLTD, ARE&amp;M, BRIGADE, CONCORDBIO, EXIDEIND, ITCHOTELS, JBCHEPHARM, JIOFIN, JYOTHYLAB, LAURUSLABS, METROPOLIS, MFSL, NCC, PFIZER, SBILIFE, SYNGENE, TMPV, CAPLIPOINT, CERA, COHANCE, EIDPARRY, IGIL, NATCOPHARM, PFC, SONACOMS, ULTRACEMCO, AADHARHFC, AIIL, ANANTRAJ, ANGELONE, ASTERDM, AWL, BEL, CHENNPETRO, CRAFTSMAN, CREDITACC, CROMPTON, EMAMILTD, FLUOROCHEM, GAIL, GODFRYPHLP, HAL, HEXT, IGL, INDIAMART, J&amp;KBANK, JPPOWER, JUBLFOOD, KAJARIACER, KPITTECH, MAHSEAMLES, MANAPPURAM, MAPMYINDIA, NAUKRI, NHPC, NIVABUPA, PCBL, PNB, RRKABEL, SBIN, SUNDARMFIN, TATACOMM, TIINDIA, UBL, VMM, ZEEL</t>
         </is>
       </c>
     </row>
@@ -4117,7 +4117,7 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
@@ -4126,7 +4126,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>MARICO, SBICARD, COALINDIA, SOLARINDS, ADANIPORTS, ALKEM, AMBUJACEM, BAJAJFINSV, COLPAL, CONCOR, DIVISLAB, FEDERALBNK, HINDALCO, HINDZINC, IDFCFIRSTB, IEX, INDUSTOWER, LT, M&amp;M, MANKIND, MARUTI, MAZDOCK, NATIONALUM, NTPC, PAYTM, SUZLON, TATACONSUM, TORNTPHARM, UNIONBANK</t>
+          <t>BAJAJHFL, BLUEJET, CAMPUS, MARICO, MSUMI, SBICARD, SUNDRMFAST, COALINDIA, EIDPARRY, JMFINANCIL, RADICO, SOLARINDS, TIMKEN, VIJAYA, ABREL, ACC, ADANIPORTS, AFCONS, AJANTPHARM, ALKEM, AMBUJACEM, BAJAJFINSV, BASF, BLS, CANFINHOME, CAPLIPOINT, CERA, COLPAL, CONCOR, DIVISLAB, DOMS, ESCORTS, FEDERALBNK, FIVESTAR, FSL, GRAVITA, HAPPSTMNDS, HBLENGINE, HINDALCO, HINDZINC, HOMEFIRST, IDFCFIRSTB, IEX, INDGN, INDUSTOWER, JUBLINGREA, LEMONTREE, LLOYDSME, LT, M&amp;M, M&amp;MFIN, MAHSEAMLES, MANKIND, MANYAVAR, MARUTI, MAZDOCK, NATIONALUM, NSLNISP, NTPC, NTPCGREEN, PAYTM, POONAWALLA, REDINGTON, SAGILITY, SUZLON, TATACONSUM, TORNTPHARM, UCOBANK, UNIONBANK, WHIRLPOOL, WOCKPHARMA</t>
         </is>
       </c>
     </row>
@@ -4142,7 +4142,7 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>34</v>
+        <v>101</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>MAXHEALTH, TIINDIA, BHARTIARTL, CDSL, CUMMINSIND, DIXON, INDHOTEL, POLYCAB, SRF, ABB, AMBUJACEM, AUROPHARMA, BAJAJHLDNG, BANDHANBNK, BEL, BRITANNIA, CGPOWER, DMART, ETERNAL, GMRAIRPORT, GODREJCP, GODREJPROP, GRASIM, HDFCAMC, HEROMOTOCO, INDIGO, IRFC, M&amp;M, MARUTI, MUTHOOTFIN, NHPC, PAYTM, POLICYBZR, TATAPOWER</t>
+          <t>LTTS, MAXHEALTH, PCBL, TIINDIA, ABSLAMC, AIAENG, ASAHIINDIA, BERGEPAINT, BHARTIARTL, BSOFT, CDSL, CUMMINSIND, DIXON, EMCURE, FINCABLES, FSL, HEXT, INDHOTEL, MOTILALOFS, NEULANDLAB, NEWGEN, POLYCAB, RAINBOW, SRF, TATACOMM, THELEELA, UBL, VMM, 3MINDIA, ABB, ABBOTINDIA, ABREL, ACC, AIIL, AMBUJACEM, ASTRAZEN, ATUL, AUROPHARMA, AWL, BAJAJHLDNG, BANDHANBNK, BBTC, BEL, BEML, BRITANNIA, CENTRALBK, CGPOWER, CHALET, COHANCE, CYIENT, DEEPAKFERT, DMART, EIDPARRY, ETERNAL, FLUOROCHEM, FORCEMOT, GICRE, GLAND, GMRAIRPORT, GODREJCP, GODREJIND, GODREJPROP, GRASIM, HAPPSTMNDS, HDFCAMC, HEROMOTOCO, HFCL, IGIL, IKS, INDIGO, INOXINDIA, IRFC, JSL, JUBLINGREA, KARURVYSYA, LLOYDSME, M&amp;M, M&amp;MFIN, MARUTI, MRF, MUTHOOTFIN, NAM-INDIA, NCC, NHPC, NLCINDIA, NTPCGREEN, ONESOURCE, PAYTM, PGHH, POLICYBZR, POONAWALLA, SCI, SHYAMMETL, SYRMA, TARIL, TATAPOWER, TBOTEK, VGUARD, VTL, WHIRLPOOL, ZEEL</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
@@ -4176,7 +4176,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>MPHASIS, 360ONE, ADANIENSOL, AMBER, ASTRAL, BHEL, BLUESTARCO, HUDCO, ITC, LTM, NAUKRI, PATANJALI, PIIND, TMPV</t>
+          <t>MPHASIS, 360ONE, DOMS, JINDALSAW, LTFOODS, ABLBL, ACMESOLAR, ADANIENSOL, AKUMS, ALOKINDS, AMBER, APOLLOTYRE, ASTRAL, BHEL, BLUESTARCO, CHOICEIN, DBREALTY, HUDCO, IRB, IRCON, ITC, JPPOWER, KEC, LTM, MEDANTA, NAUKRI, NTPCGREEN, PATANJALI, PIIND, PRAJIND, SUNTV, TATACHEM, TECHNOE, TMPV, TRIDENT, TRITURBINE</t>
         </is>
       </c>
     </row>
@@ -4192,7 +4192,7 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>39</v>
+        <v>79</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
@@ -4201,7 +4201,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>APLAPOLLO, BANKINDIA, CANBK, COALINDIA, GRASIM, HINDALCO, JINDALSTEL, NESTLEIND, PHOENIXLTD, RVNL, SOLARINDS, TECHM, UNIONBANK, ANGELONE, AXISBANK, BDL, DIVISLAB, GLENMARK, HAVELLS, IOC, KALYANKJIL, LODHA, LUPIN, M&amp;M, MCX, NATIONALUM, NTPC, PERSISTENT, PETRONET, POWERINDIA, SBIN, SHRIRAMFIN, SUPREMEIND, SWIGGY, TATASTEEL, TCS, UNOMINDA, VOLTAS, WIPRO</t>
+          <t>APLAPOLLO, BAJAJHFL, BANKINDIA, BLS, CANBK, CASTROLIND, COALINDIA, GRASIM, HINDALCO, JINDALSTEL, JMFINANCIL, LEMONTREE, MAPMYINDIA, NESTLEIND, PHOENIXLTD, RVNL, SOLARINDS, TECHM, UNIONBANK, VIJAYA, ABREL, ACC, AFCONS, ANGELONE, AWL, AXISBANK, BALKRISIND, BBTC, BDL, CARBORUNIV, DEEPAKNTR, DIVISLAB, ELECON, FIVESTAR, GLAXO, GLENMARK, GODIGIT, GRANULES, HAVELLS, HONASA, IOC, IPCALAB, JBMA, JSL, KALYANKJIL, KIRLOSBROS, LODHA, LUPIN, M&amp;M, MANYAVAR, MCX, METROPOLIS, NATIONALUM, NSLNISP, NTPC, NTPCGREEN, OLECTRA, PERSISTENT, PETRONET, POWERINDIA, RADICO, RAMCOCEM, RHIM, SAGILITY, SBIN, SCHAEFFLER, SHRIRAMFIN, SHYAMMETL, SUPREMEIND, SWIGGY, TATAINVEST, TATASTEEL, TCS, TITAGARH, UNOMINDA, VOLTAS, WIPRO, WOCKPHARMA, ZENTEC</t>
         </is>
       </c>
     </row>
@@ -4217,7 +4217,7 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>33</v>
+        <v>76</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
@@ -4226,7 +4226,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>ADANIGREEN, ASIANPAINT, IDEA, INDIANB, MARUTI, POWERGRID, BHARATFORG, BHARTIARTL, BOSCHLTD, CANBK, CIPLA, COLPAL, CONCOR, DIXON, FORTIS, HDFCBANK, HDFCLIFE, ICICIBANK, ICICIPRULI, INDIGO, KFINTECH, KOTAKBANK, MAXHEALTH, MOTHERSON, NAUKRI, NESTLEIND, PAYTM, PRESTIGE, RECLTD, TMPV, TORNTPHARM, UPL, ZYDUSLIFE</t>
+          <t>ADANIGREEN, ASIANPAINT, ECLERX, FORCEMOT, IDEA, INDIANB, MAPMYINDIA, MARUTI, OLECTRA, POWERGRID, AAVAS, ABFRL, AFFLE, APTUS, ATGL, BAJAJHFL, BERGEPAINT, BHARATFORG, BHARTIARTL, BOSCHLTD, CANBK, CIPLA, COLPAL, CONCOR, CUB, DCMSHRIRAM, DIXON, FINCABLES, FORTIS, GRAPHITE, GSPL, GUJGASLTD, HBLENGINE, HDFCBANK, HDFCLIFE, ICICIBANK, ICICIPRULI, IIFL, IKS, INDIGO, KARURVYSYA, KFINTECH, KOTAKBANK, LLOYDSME, MAXHEALTH, MOTHERSON, NAUKRI, NAVA, NESTLEIND, NEULANDLAB, NIACL, NTPCGREEN, OLAELEC, PAYTM, PFIZER, PRESTIGE, PVRINOX, RECLTD, RITES, SBFC, SCHNEIDER, SHYAMMETL, SIGNATURE, SOBHA, SUMICHEM, SUNDRMFAST, TARIL, TMPV, TORNTPHARM, TRITURBINE, UPL, USHAMART, VENTIVE, ZEEL, ZENSARTECH, ZYDUSLIFE</t>
         </is>
       </c>
     </row>
@@ -4242,7 +4242,7 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>COALINDIA, KFINTECH, LODHA, ICICIBANK, INDIGO, IREDA, M&amp;M, OIL, TITAN, BSE, CAMS, CROMPTON, DMART, HAVELLS, ICICIGI, INDUSINDBK, PATANJALI, PREMIERENE, RBLBANK, UNITDSPR, WAAREEENER</t>
+          <t>COALINDIA, GODIGIT, IGL, KFINTECH, LODHA, BLUEDART, ICICIBANK, IIFL, INDIGO, IREDA, M&amp;M, OIL, SIGNATURE, TATACHEM, TITAN, AGARWALEYE, BBTC, BSE, CAMS, CROMPTON, DMART, GLAND, GPIL, GRSE, GUJGASLTD, HAVELLS, HINDCOPPER, ICICIGI, INDUSINDBK, JKTYRE, JSL, KIRLOSENG, PATANJALI, POONAWALLA, PREMIERENE, RBLBANK, RITES, SAREGAMA, UBL, UNITDSPR, UTIAMC, VIJAYA, VMM, WAAREEENER</t>
         </is>
       </c>
     </row>
@@ -4267,7 +4267,7 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
@@ -4276,7 +4276,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>ITC, MARUTI, PPLPHARMA, ABB, ADANIENT, AMBUJACEM, APLAPOLLO, BAJAJFINSV, BDL, BEL, CONCOR, FEDERALBNK, GODREJPROP, HINDUNILVR, HUDCO, INDHOTEL, INDUSTOWER, MAXHEALTH, PFC, PHOENIXLTD, RECLTD, RVNL, SBICARD, SHREECEM, SIEMENS, SONACOMS, TMPV, UNOMINDA</t>
+          <t>ITC, NEWGEN, GSPL, INOXINDIA, MARUTI, NLCINDIA, PPLPHARMA, TATACOMM, ABB, ADANIENT, AMBUJACEM, ANANTRAJ, APLAPOLLO, ATHERENERG, BAJAJFINSV, BAYERCROP, BDL, BEL, BEML, CHAMBLFERT, COCHINSHIP, CONCOR, DBREALTY, ENGINERSIN, FEDERALBNK, GODFRYPHLP, GODREJIND, GODREJPROP, GRSE, HFCL, HINDUNILVR, HUDCO, INDHOTEL, INDUSTOWER, INTELLECT, IPCALAB, JKCEMENT, JMFINANCIL, LALPATHLAB, MAXHEALTH, OLECTRA, PFC, PHOENIXLTD, RAMCOCEM, RECLTD, RVNL, SBICARD, SCI, SHREECEM, SIEMENS, SJVN, SONACOMS, TMPV, TRIVENI, UNOMINDA, WHIRLPOOL, ZENTEC</t>
         </is>
       </c>
     </row>
@@ -4292,7 +4292,7 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>23</v>
+        <v>69</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
@@ -4301,7 +4301,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>CIPLA, ABCAPITAL, AXISBANK, BLUESTARCO, DELHIVERY, TRENT, ASHOKLEY, ASIANPAINT, BANKBARODA, BEL, CDSL, CROMPTON, GODREJPROP, HAVELLS, HDFCAMC, IEX, INOXWIND, JIOFIN, MANAPPURAM, MCX, NESTLEIND, PATANJALI, RVNL</t>
+          <t>CIPLA, ABCAPITAL, ABFRL, ADANIPOWER, ATUL, AXISBANK, BLUESTARCO, CARBORUNIV, CRAFTSMAN, CREDITACC, CRISIL, DELHIVERY, FORCEMOT, GPIL, HONASA, KPRMILL, MSUMI, NAM-INDIA, TRENT, ABLBL, AGARWALEYE, AIIL, ASHOKLEY, ASIANPAINT, BAJAJHFL, BALKRISIND, BANKBARODA, BEL, CDSL, COHANCE, COROMANDEL, CROMPTON, CUB, DEEPAKFERT, GLAND, GLAXO, GODREJAGRO, GODREJPROP, GRSE, HAVELLS, HDFCAMC, HEG, HFCL, HONAUT, IEX, INOXWIND, ITCHOTELS, JINDALSAW, JIOFIN, JYOTHYLAB, JYOTICNC, KAJARIACER, LINDEINDIA, M&amp;MFIN, MANAPPURAM, MCX, MEDANTA, NAVINFLUOR, NESTLEIND, NLCINDIA, PATANJALI, RVNL, SAPPHIRE, TRIDENT, TRITURBINE, VIJAYA, VMM, WELCORP, ZEEL</t>
         </is>
       </c>
     </row>
@@ -4317,16 +4317,16 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>14</v>
+        <v>44</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>ABCAPITAL, CIPLA, PIIND, PNBHOUSING, ADANIGREEN, AXISBANK, BEL, CGPOWER, EXIDEIND, ICICIGI, NMDC, OIL, SONACOMS, UNITDSPR</t>
+          <t>KPRMILL, ABCAPITAL, ABLBL, ATUL, CIPLA, CRAFTSMAN, CREDITACC, IFCI, MSUMI, NAM-INDIA, PIIND, PNBHOUSING, TRIDENT, ADANIGREEN, ANANTRAJ, AXISBANK, BEL, BEML, CAPLIPOINT, CGPOWER, COHANCE, CUB, DOMS, ELGIEQUIP, EXIDEIND, GODFRYPHLP, HINDCOPPER, HYUNDAI, ICICIGI, INTELLECT, JUBLPHARMA, KIMS, NEULANDLAB, NEWGEN, NMDC, OIL, PVRINOX, SAREGAMA, SONACOMS, SUNDRMFAST, TATAINVEST, UNITDSPR, WHIRLPOOL, WOCKPHARMA</t>
         </is>
       </c>
     </row>
@@ -4342,7 +4342,7 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
@@ -4351,7 +4351,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>ASIANPAINT, 360ONE, ADANIGREEN, BLUESTARCO, BOSCHLTD, CONCOR, DALBHARAT, HEROMOTOCO, HINDPETRO, ICICIGI, INFY, NATIONALUM, NESTLEIND, OFSS, PATANJALI, RELIANCE, SBICARD, UNITDSPR</t>
+          <t>ACMESOLAR, ASIANPAINT, BLUEJET, 360ONE, ADANIGREEN, AKUMS, ANANTRAJ, BLUESTARCO, BOSCHLTD, CONCOR, COROMANDEL, DALBHARAT, EMAMILTD, FORCEMOT, GODREJIND, HEROMOTOCO, HINDPETRO, ICICIGI, INFY, JPPOWER, KIRLOSENG, MAHSCOOTER, MEDANTA, MOTILALOFS, NATIONALUM, NESTLEIND, OFSS, PATANJALI, PTCIL, RELIANCE, RHIM, RKFORGE, SBICARD, UNITDSPR</t>
         </is>
       </c>
     </row>
@@ -4367,16 +4367,16 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>ADANIENT, AUBANK, BAJAJ-AUTO, EXIDEIND, INDUSTOWER, KOTAKBANK, MCX, MPHASIS, PFC, PIIND, POLICYBZR, PRESTIGE, RECLTD, SBICARD</t>
+          <t>CAPLIPOINT, DOMS, LLOYDSME, WELSPUNLIV, ZFCVINDIA, ACE, ADANIENT, ADANIPOWER, AKUMS, APOLLOTYRE, APTUS, AUBANK, BAJAJ-AUTO, BHARTIHEXA, DEVYANI, EMCURE, EXIDEIND, GMDCLTD, GODREJIND, IGIL, INDUSTOWER, ITCHOTELS, JUBLPHARMA, KOTAKBANK, MCX, MPHASIS, OLECTRA, PFC, PIIND, POLICYBZR, PRESTIGE, RAMCOCEM, RECLTD, RHIM, RKFORGE, SAGILITY, SBICARD, SOBHA, VMM, WOCKPHARMA</t>
         </is>
       </c>
     </row>
@@ -4392,7 +4392,7 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="D159" t="inlineStr">
         <is>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>HDFCLIFE, NATIONALUM, OBEROIRLTY, 360ONE, AMBUJACEM, ASIANPAINT, BOSCHLTD, CDSL, COALINDIA, CONCOR, HAVELLS, HDFCAMC, HINDPETRO, HINDUNILVR, INDUSTOWER, JIOFIN, KFINTECH, MFSL, PERSISTENT, RELIANCE, ULTRACEMCO, VBL</t>
+          <t>AARTIIND, BALRAMCHIN, GODIGIT, HDFCLIFE, IRB, MMTC, NATIONALUM, OBEROIRLTY, 360ONE, ABREL, ABSLAMC, AEGISLOG, AMBUJACEM, ANANTRAJ, APOLLOTYRE, ASIANPAINT, BOSCHLTD, CDSL, COALINDIA, CONCOR, DEEPAKFERT, EIDPARRY, ELGIEQUIP, ESCORTS, FLUOROCHEM, HAVELLS, HDFCAMC, HINDPETRO, HINDUNILVR, INDUSTOWER, ITCHOTELS, JIOFIN, JKCEMENT, JPPOWER, JSWINFRA, KAJARIACER, KFINTECH, M&amp;MFIN, MFSL, NAVINFLUOR, NEULANDLAB, NIACL, PERSISTENT, PFIZER, PRAJIND, PTCIL, RELIANCE, RPOWER, SIGNATURE, TARIL, TATAINVEST, ULTRACEMCO, USHAMART, VBL, WELCORP</t>
         </is>
       </c>
     </row>
@@ -4417,16 +4417,16 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>BHEL, NUVAMA, BAJAJFINSV, CAMS, DALBHARAT, DIXON, DLF, DMART, GMRAIRPORT, HINDALCO, IDFCFIRSTB, INFY, KALYANKJIL, KPITTECH, LODHA, M&amp;M, OFSS, SAMMAANCAP, SWIGGY, TITAN, WAAREEENER</t>
+          <t>SUMICHEM, BHEL, CAMPUS, GRAVITA, NUVAMA, 3MINDIA, AADHARHFC, AGARWALEYE, AIIL, ALOKINDS, APOLLOTYRE, BAJAJFINSV, BBTC, BLUEDART, CAMS, CONCORDBIO, DALBHARAT, DIXON, DLF, DMART, EIDPARRY, ELECON, FIRSTCRY, GICRE, GMRAIRPORT, HINDALCO, IDFCFIRSTB, IIFL, INFY, IOB, JKTYRE, KALYANKJIL, KPITTECH, LLOYDSME, LODHA, M&amp;M, MAHSCOOTER, NCC, OFSS, POONAWALLA, SAMMAANCAP, SWIGGY, SYRMA, TARIL, TATAINVEST, TITAN, UBL, UTIAMC, WAAREEENER, WELSPUNLIV</t>
         </is>
       </c>
     </row>
@@ -4442,16 +4442,16 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>24</v>
+        <v>65</v>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>ALKEM, HINDZINC, IEX, JUBLFOOD, MAXHEALTH, ASHOKLEY, AUROPHARMA, BANKBARODA, DIVISLAB, GRASIM, HUDCO, ICICIPRULI, INDUSINDBK, ITC, KOTAKBANK, LICHSGFIN, MANKIND, MARUTI, NYKAA, PERSISTENT, PHOENIXLTD, PIDILITIND, SOLARINDS, ZYDUSLIFE</t>
+          <t>CONCORDBIO, ALKEM, HINDZINC, IEX, JUBLFOOD, JYOTHYLAB, LEMONTREE, MAXHEALTH, REDINGTON, AKZOINDIA, ALKYLAMINE, ARE&amp;M, ASHOKLEY, ASTRAZEN, AUROPHARMA, BANKBARODA, BIKAJI, BRIGADE, BSOFT, CENTRALBK, CESC, CHAMBLFERT, CHOLAHLDNG, CLEAN, DBREALTY, DEVYANI, DIVISLAB, ENDURANCE, FINPIPE, GESHIP, GLAXO, GODFRYPHLP, GRASIM, HEG, HUDCO, ICICIPRULI, INDUSINDBK, ITC, JINDALSAW, JYOTICNC, KOTAKBANK, LALPATHLAB, LICHSGFIN, LINDEINDIA, LTTS, MANKIND, MARUTI, MRF, NH, NYKAA, PERSISTENT, PHOENIXLTD, PIDILITIND, RKFORGE, SAREGAMA, SBFC, SCI, SHYAMMETL, SJVN, SOLARINDS, STARHEALTH, SUNTV, TATACOMM, TEJASNET, ZYDUSLIFE</t>
         </is>
       </c>
     </row>
@@ -4467,16 +4467,16 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>BHARTIARTL, AMBUJACEM, APLAPOLLO, DELHIVERY, FEDERALBNK, IDEA, INDHOTEL, INDUSTOWER, LICI, LUPIN, PRESTIGE, RECLTD, SBILIFE, SHREECEM, SIEMENS, TMPV, UNOMINDA</t>
+          <t>ACC, BHARTIARTL, CGCL, AEGISVOPAK, ATGL, BLUEDART, HOMEFIRST, INDGN, IRB, REDINGTON, SUNDARMFIN, AFFLE, AMBUJACEM, APLAPOLLO, BLS, BSOFT, CEATLTD, CERA, CLEAN, CRISIL, DELHIVERY, EMCURE, ERIS, FEDERALBNK, GICRE, GVT&amp;D, HONAUT, IDEA, INDHOTEL, INDUSTOWER, JKCEMENT, JSWCEMENT, KIMS, KPIL, KSB, LICI, LTTS, LUPIN, METROPOLIS, MGL, NEULANDLAB, PCBL, PRESTIGE, RCF, RECLTD, RHIM, RITES, SBILIFE, SCHAEFFLER, SCHNEIDER, SHREECEM, SIEMENS, TIMKEN, TMPV, TRITURBINE, UNOMINDA, VIJAYA</t>
         </is>
       </c>
     </row>
@@ -4492,7 +4492,7 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>29</v>
+        <v>69</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
@@ -4501,7 +4501,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>INDIGO, JIOFIN, KEI, M&amp;M, TITAN, BSE, CAMS, DMART, EICHERMOT, ETERNAL, GRASIM, HAVELLS, HDFCAMC, INOXWIND, LODHA, MARICO, MUTHOOTFIN, NBCC, NHPC, PNB, PREMIERENE, TATAELXSI, TATAPOWER, TCS, TECHM, TORNTPOWER, TRENT, VBL, WAAREEENER</t>
+          <t>IIFL, INDIGO, JIOFIN, KEI, M&amp;M, NAVINFLUOR, NETWEB, SUMICHEM, TITAN, ABFRL, AFCONS, ASTRAZEN, AWL, BATAINDIA, BBTC, BIKAJI, BSE, CAMS, CHAMBLFERT, CHOLAHLDNG, DMART, EICHERMOT, EIHOTEL, ETERNAL, FINCABLES, FORCEMOT, GODREJAGRO, GRASIM, HAVELLS, HBLENGINE, HDFCAMC, HINDCOPPER, HONASA, INOXWIND, ITI, JKTYRE, KAJARIACER, LATENTVIEW, LODHA, M&amp;MFIN, MANYAVAR, MAPMYINDIA, MARICO, MUTHOOTFIN, NBCC, NHPC, NSLNISP, PCBL, PNB, POONAWALLA, PREMIERENE, RAILTEL, SCHNEIDER, SONATSOFTW, SUNTV, TATAELXSI, TATAPOWER, TCS, TECHM, THERMAX, TORNTPOWER, TRENT, UBL, UTIAMC, VBL, VENTIVE, WAAREEENER, ZEEL, ZENSARTECH</t>
         </is>
       </c>
     </row>
@@ -4517,7 +4517,7 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>17</v>
+        <v>56</v>
       </c>
       <c r="D164" t="inlineStr">
         <is>
@@ -4526,7 +4526,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>HINDZINC, MARUTI, ASHOKLEY, BAJAJ-AUTO, DABUR, ETERNAL, HDFCLIFE, HUDCO, KFINTECH, NHPC, SAMMAANCAP, SOLARINDS, TATAELXSI, TECHM, VOLTAS, WIPRO, YESBANK</t>
+          <t>BLUEJET, CEATLTD, GSPL, HINDZINC, MARUTI, MOTILALOFS, PTCIL, TATACOMM, TEJASNET, AFFLE, ARE&amp;M, ASAHIINDIA, ASHOKLEY, BAJAJ-AUTO, BAYERCROP, DABUR, DBREALTY, ETERNAL, GLAXO, GODFRYPHLP, GODIGIT, GRANULES, HAPPSTMNDS, HDFCLIFE, HEXT, HFCL, HOMEFIRST, HUDCO, IKS, JINDALSAW, JYOTICNC, KFINTECH, KIRLOSBROS, MAHABANK, MRF, NATCOPHARM, NHPC, NSLNISP, NUVOCO, RKFORGE, RPOWER, RRKABEL, SAMMAANCAP, SARDAEN, SCI, SJVN, SOLARINDS, TATAELXSI, TBOTEK, TECHM, THERMAX, VENTIVE, VOLTAS, WIPRO, YESBANK, ZENSARTECH</t>
         </is>
       </c>
     </row>
@@ -4542,7 +4542,7 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="D165" t="inlineStr">
         <is>
@@ -4551,7 +4551,7 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>DELHIVERY, ICICIBANK, IREDA, MUTHOOTFIN, ADANIENSOL, ANGELONE, APLAPOLLO, AUBANK, COALINDIA, INDHOTEL, INOXWIND, MARICO, TATACONSUM, UNOMINDA</t>
+          <t>CRISIL, DELHIVERY, ICICIBANK, IGL, INDGN, IREDA, METROPOLIS, MUTHOOTFIN, ADANIENSOL, AFCONS, ANGELONE, APLAPOLLO, AUBANK, BASF, BATAINDIA, BERGEPAINT, BLS, CENTRALBK, CERA, COALINDIA, ECLERX, EIDPARRY, ENDURANCE, ERIS, HONAUT, INDHOTEL, INOXWIND, MARICO, SIGNATURE, SWANCORP, TATACONSUM, TRITURBINE, TTML, UNOMINDA, WOCKPHARMA</t>
         </is>
       </c>
     </row>
@@ -4567,7 +4567,7 @@
         </is>
       </c>
       <c r="C166" t="n">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="D166" t="inlineStr">
         <is>
@@ -4576,7 +4576,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>TRENT, ANGELONE, BIOCON, GODREJPROP, HAL, HEROMOTOCO, HINDUNILVR, ICICIPRULI, SUZLON, UNIONBANK, VBL, VEDL, YESBANK</t>
+          <t>ABFRL, HONASA, TBOTEK, TRENT, AFCONS, ANGELONE, APARINDS, APLLTD, BASF, BATAINDIA, BHARTIHEXA, BIOCON, CARBORUNIV, CEATLTD, CERA, GLAND, GODREJAGRO, GODREJPROP, GUJGASLTD, HAL, HAPPSTMNDS, HEROMOTOCO, HINDUNILVR, ICICIPRULI, IKS, MAHSEAMLES, MOTILALOFS, NAVA, NUVOCO, SUZLON, SWANCORP, TATACHEM, TTML, UNIONBANK, VBL, VEDL, VMM, YESBANK, ZEEL</t>
         </is>
       </c>
     </row>
@@ -4592,7 +4592,7 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="D167" t="inlineStr">
         <is>
@@ -4601,7 +4601,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>AUROPHARMA, EICHERMOT, LTM, MUTHOOTFIN, PGEL</t>
+          <t>AUROPHARMA, BSOFT, CANFINHOME, EICHERMOT, EIHOTEL, GRANULES, IRCTC, LTM, LTTS, MUTHOOTFIN, NETWEB, NIVABUPA, PGEL, RHIM</t>
         </is>
       </c>
     </row>
@@ -4617,7 +4617,7 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="D168" t="inlineStr">
         <is>
@@ -4626,7 +4626,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>PPLPHARMA, ADANIENSOL, RELIANCE, SUZLON, TATACONSUM</t>
+          <t>INOXINDIA, PPLPHARMA, ZFCVINDIA, ADANIENSOL, APLLTD, ENGINERSIN, GLAND, KIRLOSBROS, PGHH, RELIANCE, SUZLON, TATACONSUM, TRIVENI</t>
         </is>
       </c>
     </row>
@@ -4642,7 +4642,7 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="D169" t="inlineStr">
         <is>
@@ -4651,7 +4651,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>BAJFINANCE, BDL, ETERNAL, UNIONBANK</t>
+          <t>ACC, BAJFINANCE, BDL, COCHINSHIP, COHANCE, CUB, ELGIEQUIP, ETERNAL, FIRSTCRY, IGIL, INTELLECT, JPPOWER, NAVA, NCC, PCBL, RAMCOCEM, SBFC, THERMAX, UNIONBANK, VIJAYA, ZENTEC</t>
         </is>
       </c>
     </row>
@@ -4667,7 +4667,7 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="D170" t="inlineStr">
         <is>
@@ -4676,7 +4676,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>PNB, ALKEM, BAJFINANCE, CROMPTON, HAL, HCLTECH, HDFCLIFE, INFY, KFINTECH, KPITTECH, LODHA, LTM, MANKIND, MFSL, NAUKRI, NMDC, OFSS, OIL, SBILIFE, TATATECH, TCS, VEDL</t>
+          <t>GODIGIT, PNB, ALKEM, BAJFINANCE, CANFINHOME, CCL, CROMPTON, ELGIEQUIP, HAL, HCLTECH, HDFCLIFE, HINDCOPPER, IGIL, INFY, KFINTECH, KPITTECH, LODHA, LTM, MANKIND, MFSL, NAUKRI, NEULANDLAB, NEWGEN, NIVABUPA, NMDC, NSLNISP, OFSS, OIL, OLECTRA, PCBL, SBILIFE, SCHNEIDER, TATATECH, TCS, VEDL, VENTIVE, VIJAYA</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="D171" t="inlineStr">
         <is>
@@ -4701,7 +4701,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>AUROPHARMA, COALINDIA, DALBHARAT, HCLTECH, INFY, ITC, KPITTECH, MARICO, MFSL, NAUKRI, OFSS, SBILIFE, TATATECH, TCS</t>
+          <t>AEGISLOG, AUROPHARMA, BAJAJHFL, BERGEPAINT, CCL, CHOICEIN, COALINDIA, DALBHARAT, GPIL, HCLTECH, HINDCOPPER, INFY, ITC, JPPOWER, KPITTECH, MAHSCOOTER, MARICO, MFSL, NAUKRI, NSLNISP, OFSS, OLECTRA, SBILIFE, SIGNATURE, TATATECH, TCS, VENTIVE, VGUARD</t>
         </is>
       </c>
     </row>
@@ -4717,7 +4717,7 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="D172" t="inlineStr">
         <is>
@@ -4726,7 +4726,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>LT, ETERNAL, GODREJPROP, HEROMOTOCO, INOXWIND, MARICO, MUTHOOTFIN, PNBHOUSING, SBIN</t>
+          <t>KEC, LT, AADHARHFC, AAVAS, ACC, ALOKINDS, CHOLAHLDNG, ETERNAL, GODREJPROP, HEROMOTOCO, HFCL, IFCI, INOXWIND, JMFINANCIL, MARICO, MUTHOOTFIN, NEWGEN, PNBHOUSING, SBIN, STARHEALTH, VMM, WHIRLPOOL, WOCKPHARMA</t>
         </is>
       </c>
     </row>
@@ -4742,7 +4742,7 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="D173" t="inlineStr">
         <is>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>BAJAJFINSV, BRITANNIA, LICHSGFIN, LTF, POWERGRID, SAMMAANCAP, TATASTEEL, RVNL, ABB, BLUESTARCO, HEROMOTOCO, PATANJALI, UPL</t>
+          <t>BAJAJFINSV, BRITANNIA, IOB, LICHSGFIN, LTF, POWERGRID, SAMMAANCAP, TATASTEEL, CAPLIPOINT, COROMANDEL, DOMS, PVRINOX, RVNL, AADHARHFC, AAVAS, ABB, ACMESOLAR, ALOKINDS, ARE&amp;M, AWL, BLUESTARCO, FORCEMOT, GRANULES, HEROMOTOCO, HEXT, MEDANTA, MOTILALOFS, NEULANDLAB, PATANJALI, UCOBANK, UPL, VGUARD</t>
         </is>
       </c>
     </row>
@@ -4767,7 +4767,7 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="D174" t="inlineStr">
         <is>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>ADANIENSOL, ADANIPORTS, BEL, GMRAIRPORT, JSWSTEEL, TATACONSUM, WIPRO, ADANIENT, ADANIGREEN, CAMS, DMART, ICICIGI, KOTAKBANK, LICI, NTPC, PAGEIND, PIIND, PRESTIGE, TITAN, UNITDSPR, WAAREEENER</t>
+          <t>ADANIENSOL, ADANIPORTS, AGARWALEYE, AKZOINDIA, ALKYLAMINE, BEL, ENDURANCE, GMRAIRPORT, GRSE, JSWSTEEL, KARURVYSYA, LATENTVIEW, MRPL, TATACONSUM, WIPRO, GESHIP, IRCTC, JUBLINGREA, ACE, ADANIENT, ADANIGREEN, AEGISVOPAK, AWL, BBTC, BHARTIHEXA, BSOFT, CAMS, DMART, FIRSTCRY, HAPPSTMNDS, ICICIGI, JKTYRE, KOTAKBANK, LEMONTREE, LICI, LTTS, NH, NTPC, PAGEIND, PIIND, POONAWALLA, PRESTIGE, RAMCOCEM, REDINGTON, SAILIFE, SHYAMMETL, SOBHA, TITAN, UBL, UNITDSPR, UTIAMC, WAAREEENER</t>
         </is>
       </c>
     </row>
@@ -4792,7 +4792,7 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>37</v>
+        <v>77</v>
       </c>
       <c r="D175" t="inlineStr">
         <is>
@@ -4801,7 +4801,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>BANDHANBNK, BANKBARODA, BIOCON, DRREDDY, IEX, JINDALSTEL, MAXHEALTH, NBCC, SHRIRAMFIN, TATAPOWER, TORNTPHARM, NMDC, ULTRACEMCO, AMBUJACEM, ASTRAL, BAJAJ-AUTO, BOSCHLTD, CANBK, CDSL, CGPOWER, GODREJCP, HDFCLIFE, HINDUNILVR, HUDCO, ICICIPRULI, INDUSINDBK, JIOFIN, JSWENERGY, LAURUSLABS, MARUTI, OBEROIRLTY, PAGEIND, PIDILITIND, SBICARD, SUNPHARMA, SUPREMEIND, ZYDUSLIFE</t>
+          <t>ASTERDM, BANDHANBNK, BANKBARODA, BIOCON, CENTRALBK, CESC, DRREDDY, ENRIN, IEX, IPCALAB, JINDALSTEL, KIMS, MAXHEALTH, NBCC, SHRIRAMFIN, TATAPOWER, TORNTPHARM, ABREL, AKUMS, EMAMILTD, JSWINFRA, NMDC, RPOWER, ULTRACEMCO, AARTIIND, AJANTPHARM, AMBUJACEM, ASTRAL, BAJAJ-AUTO, BALRAMCHIN, BOSCHLTD, CANBK, CDSL, CGPOWER, DBREALTY, EMCURE, ESCORTS, FINPIPE, FLUOROCHEM, GODREJCP, GODREJIND, GVT&amp;D, HDFCLIFE, HINDUNILVR, HUDCO, ICICIPRULI, INDUSINDBK, JBCHEPHARM, JIOFIN, JKCEMENT, JSWENERGY, LAURUSLABS, M&amp;MFIN, MARUTI, MMTC, NAVA, NAVINFLUOR, NIACL, OBEROIRLTY, PAGEIND, PFIZER, PIDILITIND, PRAJIND, PTCIL, REDINGTON, RHIM, RKFORGE, SBICARD, SCI, SJVN, SUNPHARMA, SUPREMEIND, TATACOMM, USHAMART, VTL, WELCORP, ZYDUSLIFE</t>
         </is>
       </c>
     </row>
@@ -4817,7 +4817,7 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>54</v>
+        <v>124</v>
       </c>
       <c r="D176" t="inlineStr">
         <is>
@@ -4826,7 +4826,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>COFORGE, HDFCBANK, SYNGENE, VEDL, HINDALCO, AMBER, APLAPOLLO, APOLLOHOSP, BAJAJ-AUTO, BANKINDIA, BHARATFORG, BHEL, CANBK, CGPOWER, CUMMINSIND, DABUR, DALBHARAT, DELHIVERY, DIXON, DLF, EICHERMOT, FEDERALBNK, FORTIS, GAIL, GLENMARK, HAL, ICICIPRULI, INDHOTEL, INDIANB, INDUSINDBK, IOC, IRFC, JSWENERGY, KALYANKJIL, KEI, KFINTECH, LTM, LUPIN, MAZDOCK, NUVAMA, ONGC, PETRONET, POLYCAB, POWERINDIA, SIEMENS, SUNPHARMA, SUPREMEIND, SWIGGY, TIINDIA, TMPV, TORNTPOWER, UNIONBANK, UNOMINDA, VOLTAS</t>
+          <t>ABBOTINDIA, ASAHIINDIA, CANFINHOME, CENTURYPLY, CHALET, COFORGE, CYIENT, DCMSHRIRAM, ECLERX, GILLETTE, HDFCBANK, INDIAMART, MANYAVAR, NIVABUPA, OLAELEC, RADICO, SONATSOFTW, SUNDRMFAST, SYNGENE, VEDL, ELECON, HINDALCO, IRB, TECHNOE, 3MINDIA, AIIL, AJANTPHARM, AMBER, APARINDS, APLAPOLLO, APOLLOHOSP, BAJAJ-AUTO, BAJAJHFL, BANKINDIA, BHARATFORG, BHEL, BLUEDART, CAMPUS, CANBK, CGPOWER, CHENNPETRO, CRISIL, CUMMINSIND, DABUR, DALBHARAT, DATAPATTNS, DELHIVERY, DIXON, DLF, EICHERMOT, EIDPARRY, FACT, FEDERALBNK, FINCABLES, FIVESTAR, FORTIS, FSL, GAIL, GLENMARK, GODIGIT, GRAPHITE, GRAVITA, GVT&amp;D, HAL, HBLENGINE, ICICIPRULI, IDBI, INDHOTEL, INDIACEM, INDIANB, INDUSINDBK, IOC, IRCON, IRFC, ITCHOTELS, J&amp;KBANK, JBCHEPHARM, JSWCEMENT, JSWENERGY, JWL, KALYANKJIL, KEI, KFINTECH, KSB, LTM, LUPIN, MAHABANK, MAHSCOOTER, MAHSEAMLES, MAPMYINDIA, MAZDOCK, MGL, NATCOPHARM, NAVA, NUVAMA, OLECTRA, ONGC, PETRONET, PGHH, POLYCAB, POLYMED, POWERINDIA, RCF, RITES, RRKABEL, SAGILITY, SARDAEN, SCHAEFFLER, SIEMENS, SUNDARMFIN, SUNPHARMA, SUPREMEIND, SWIGGY, THERMAX, TIINDIA, TIMKEN, TITAGARH, TMPV, TORNTPOWER, TRITURBINE, UNIONBANK, UNOMINDA, VOLTAS, VTL</t>
         </is>
       </c>
     </row>
@@ -4842,7 +4842,7 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>30</v>
+        <v>67</v>
       </c>
       <c r="D177" t="inlineStr">
         <is>
@@ -4851,7 +4851,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>MOTHERSON, PGEL, SAIL, APOLLOHOSP, ASHOKLEY, BAJAJFINSV, BANKINDIA, COALINDIA, CUMMINSIND, DABUR, DIVISLAB, EICHERMOT, FEDERALBNK, FORTIS, GAIL, GLENMARK, GRASIM, INDIANB, INDUSTOWER, JUBLFOOD, LUPIN, NYKAA, ONGC, PFC, PHOENIXLTD, TIINDIA, TRENT, TVSMOTOR, UNIONBANK, VOLTAS</t>
+          <t>ANANDRATHI, HEG, LALPATHLAB, MOTHERSON, PGEL, SAIL, SUMICHEM, ABFRL, ABSLAMC, AJANTPHARM, APOLLOHOSP, ARE&amp;M, ASHOKLEY, ASTRAZEN, BAJAJFINSV, BANKINDIA, CHAMBLFERT, CHOLAHLDNG, COALINDIA, CUMMINSIND, DABUR, DEVYANI, DIVISLAB, EICHERMOT, ELGIEQUIP, FEDERALBNK, FINCABLES, FORTIS, GAIL, GLAXO, GLENMARK, GODREJAGRO, GRANULES, GRAPHITE, GRASIM, HONASA, IDBI, INDIANB, INDUSTOWER, J&amp;KBANK, JINDALSAW, JPPOWER, JSWCEMENT, JUBLFOOD, JYOTICNC, KIRLOSENG, LUPIN, MAHSEAMLES, MGL, MRF, NATCOPHARM, NTPCGREEN, NYKAA, ONGC, PFC, PHOENIXLTD, RAILTEL, RRKABEL, SARDAEN, SIGNATURE, SYRMA, TIINDIA, TRENT, TVSMOTOR, UNIONBANK, VOLTAS, ZEEL</t>
         </is>
       </c>
     </row>
@@ -4867,7 +4867,7 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>37</v>
+        <v>78</v>
       </c>
       <c r="D178" t="inlineStr">
         <is>
@@ -4876,7 +4876,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>ICICIBANK, AMBER, BHARATFORG, BSE, CAMS, COLPAL, DMART, FORTIS, GODREJCP, HAL, ICICIPRULI, INDIGO, INDUSINDBK, INFY, INOXWIND, IOC, IREDA, IRFC, KAYNES, KEI, M&amp;M, MANAPPURAM, MAXHEALTH, MAZDOCK, OFSS, PETRONET, PIDILITIND, POLYCAB, POWERINDIA, PREMIERENE, RECLTD, SHREECEM, SIEMENS, TITAN, TMPV, TORNTPOWER, WAAREEENER</t>
+          <t>ICICIBANK, AMBER, PGHH, RITES, TATAINVEST, AGARWALEYE, APARINDS, APOLLOTYRE, APTUS, BBTC, BHARATFORG, BIKAJI, BSE, CAMS, CHENNPETRO, COLPAL, DATAPATTNS, DEEPAKNTR, DMART, FACT, FIVESTAR, FORTIS, FSL, GLAND, GODREJCP, GRSE, HAL, HBLENGINE, ICICIPRULI, IGL, IIFL, INDIACEM, INDIGO, INDUSINDBK, INFY, INOXWIND, IOC, IPCALAB, IRCON, IREDA, IRFC, JKTYRE, JWL, KAYNES, KEI, KSB, M&amp;M, MAHABANK, MANAPPURAM, MAPMYINDIA, MAXHEALTH, MAZDOCK, OFSS, PETRONET, PIDILITIND, POLYCAB, POONAWALLA, POWERINDIA, PREMIERENE, RCF, RECLTD, SCHAEFFLER, SHREECEM, SIEMENS, SUNDARMFIN, SUNTV, TARIL, TATACHEM, THELEELA, TIMKEN, TITAGARH, TITAN, TMPV, TORNTPOWER, UBL, UTIAMC, WAAREEENER, ZENSARTECH</t>
         </is>
       </c>
     </row>
@@ -4892,7 +4892,7 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="D179" t="inlineStr">
         <is>
@@ -4901,7 +4901,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>FEDERALBNK, HDFCAMC, IEX, BANKBARODA, BEL, BHARTIARTL, BRITANNIA, COLPAL, CONCOR, DABUR, GAIL, HAVELLS, HUDCO, INDUSINDBK, JSWENERGY, MARUTI, MPHASIS, PIDILITIND, PNBHOUSING, PPLPHARMA, RVNL, SHRIRAMFIN, TMPV, TVSMOTOR, ZYDUSLIFE</t>
+          <t>FEDERALBNK, GSPL, HDFCAMC, IEX, INDGN, REDINGTON, RITES, ACC, ANANDRATHI, BANKBARODA, BAYERCROP, BEL, BHARTIARTL, BLUEDART, BRITANNIA, CCL, COLPAL, CONCOR, CONCORDBIO, DABUR, DBREALTY, ENGINERSIN, FIVESTAR, GAIL, GILLETTE, GRAPHITE, HAVELLS, HUDCO, IFCI, INDUSINDBK, INOXINDIA, JBCHEPHARM, JMFINANCIL, JSWENERGY, KAJARIACER, MARUTI, MPHASIS, PIDILITIND, PNBHOUSING, PPLPHARMA, PVRINOX, RVNL, SCI, SHRIRAMFIN, SJVN, SWANCORP, TATACOMM, THELEELA, TMPV, TRIVENI, TVSMOTOR, VMM, WOCKPHARMA, ZYDUSLIFE</t>
         </is>
       </c>
     </row>
@@ -4917,7 +4917,7 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>30</v>
+        <v>78</v>
       </c>
       <c r="D180" t="inlineStr">
         <is>
@@ -4926,7 +4926,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>CIPLA, SIEMENS, ABB, ABCAPITAL, AXISBANK, DALBHARAT, MUTHOOTFIN, AMBUJACEM, APLAPOLLO, APOLLOHOSP, BANKINDIA, BDL, BLUESTARCO, DELHIVERY, HAL, HAVELLS, IOC, IRFC, ITC, JIOFIN, LODHA, LTF, MAXHEALTH, MAZDOCK, NAUKRI, ONGC, PERSISTENT, SBIN, TMPV, UNOMINDA</t>
+          <t>CIPLA, SIEMENS, ABB, ABCAPITAL, AXISBANK, CRAFTSMAN, CREDITACC, DALBHARAT, JSWCEMENT, KIMS, MSUMI, MUTHOOTFIN, REDINGTON, TEJASNET, ABLBL, ACMESOLAR, AKZOINDIA, AMBUJACEM, APLAPOLLO, APOLLOHOSP, ATUL, BAJAJHFL, BANKINDIA, BDL, BEML, BLUEJET, BLUESTARCO, BSOFT, CARBORUNIV, CENTURYPLY, CGCL, CHENNPETRO, COHANCE, CRISIL, CUB, DELHIVERY, EMAMILTD, GRSE, HAL, HAVELLS, HBLENGINE, IGIL, INDIACEM, INTELLECT, IOC, IRCON, IRFC, ITC, JIOFIN, JKCEMENT, KPIL, KPRMILL, KSB, LODHA, LTF, LTTS, MAHSCOOTER, MAHSEAMLES, MAXHEALTH, MAZDOCK, METROPOLIS, MOTILALOFS, NAM-INDIA, NAUKRI, NH, ONGC, PERSISTENT, SBIN, SCHAEFFLER, SUNDRMFAST, TIMKEN, TITAGARH, TMPV, TRIDENT, TRITURBINE, UNOMINDA, VTL, ZENTEC</t>
         </is>
       </c>
     </row>
@@ -4942,7 +4942,7 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="D181" t="inlineStr">
         <is>
@@ -4951,7 +4951,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>ABCAPITAL, CIPLA, TRENT, AXISBANK, BANKBARODA, BEL, CGPOWER, COLPAL, CROMPTON, ETERNAL, GODREJPROP, HDFCBANK, IEX, KEI, LAURUSLABS, MFSL, NYKAA, OIL, POLYCAB, RBLBANK, TORNTPOWER</t>
+          <t>ABCAPITAL, ABFRL, ATUL, CIPLA, CRAFTSMAN, CREDITACC, HFCL, HOMEFIRST, HONASA, KPRMILL, MSUMI, NAM-INDIA, RKFORGE, TRENT, TRIDENT, ABLBL, ABSLAMC, ADANIPOWER, AGARWALEYE, AXISBANK, BANKBARODA, BEL, CGPOWER, CLEAN, COLPAL, CROMPTON, DATAPATTNS, DEVYANI, ETERNAL, GLAND, GODFRYPHLP, GODREJAGRO, GODREJPROP, GPIL, GRSE, GVT&amp;D, HDFCBANK, IEX, JINDALSAW, JWL, KEC, KEI, LAURUSLABS, LINDEINDIA, MFSL, NATCOPHARM, NAVINFLUOR, NLCINDIA, NYKAA, OIL, POLYCAB, RBLBANK, SCHAEFFLER, TECHNOE, TORNTPOWER, VIJAYA, ZEEL</t>
         </is>
       </c>
     </row>
@@ -4967,16 +4967,16 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>HINDUNILVR, ADANIENT, AMBER, BEL, CGPOWER, HDFCLIFE, HEROMOTOCO, INDIANB, IOC, KEI, KOTAKBANK, NBCC, POWERINDIA, PRESTIGE, TATASTEEL, TATATECH, TORNTPOWER, VOLTAS</t>
+          <t>PTCIL, CEATLTD, HINDUNILVR, TBOTEK, ACE, ADANIENT, AKZOINDIA, ALOKINDS, AMBER, ATHERENERG, BEL, CGPOWER, DCMSHRIRAM, ENRIN, FINCABLES, HDFCLIFE, HEROMOTOCO, HINDCOPPER, HONAUT, IKS, INDIANB, IOC, JPPOWER, KEI, KOTAKBANK, KPRMILL, LINDEINDIA, MAPMYINDIA, MOTILALOFS, NBCC, NUVOCO, POWERINDIA, PRESTIGE, RAMCOCEM, RPOWER, SAGILITY, SOBHA, SUNTV, TATASTEEL, TATATECH, THELEELA, THERMAX, TORNTPOWER, VOLTAS, WHIRLPOOL</t>
         </is>
       </c>
     </row>
@@ -4992,7 +4992,7 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>14</v>
+        <v>49</v>
       </c>
       <c r="D183" t="inlineStr">
         <is>
@@ -5001,7 +5001,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>CDSL, AMBER, AMBUJACEM, ANGELONE, BAJAJ-AUTO, BANDHANBNK, BLUESTARCO, GODREJPROP, JIOFIN, MANKIND, OBEROIRLTY, OFSS, PATANJALI, ULTRACEMCO</t>
+          <t>AARTIIND, CDSL, ABREL, AFCONS, AMBER, AMBUJACEM, ANGELONE, BAJAJ-AUTO, BALRAMCHIN, BANDHANBNK, BASF, BATAINDIA, BLUESTARCO, CERA, COROMANDEL, DEEPAKFERT, DEEPAKNTR, ESCORTS, FLUOROCHEM, FORCEMOT, GODREJPROP, HOMEFIRST, JIOFIN, JKCEMENT, JSWINFRA, LTFOODS, M&amp;MFIN, MAHABANK, MANKIND, MANYAVAR, MEDANTA, MMTC, NATCOPHARM, NAVINFLUOR, NIACL, OBEROIRLTY, OFSS, PATANJALI, PCBL, PFIZER, PRAJIND, SARDAEN, SCHNEIDER, TEJASNET, TTML, ULTRACEMCO, USHAMART, WELCORP, ZFCVINDIA</t>
         </is>
       </c>
     </row>

</xml_diff>